<commit_message>
Correct Martin's incumbent to Martin's Pork Products (Falcon, NC)
The incumbent 'Martin's' supplier is Martin's Pork Products, Inc. in Falcon, NC
(active USDA Talmadge-Aiken slaughter + processing plant, Est. TA-6720, ~75 staff,
NC Meat Processors Association member) — not the unrelated Martin's Abattoir &
Wholesale Meats in Godwin (a cattle plant that closed in 2013), which the earlier
draft had matched by mistake.

Updates the reference roster row (now REFERENCE, federally FSIS-inspected via
Talmadge-Aiken; APHIS export listing noted as separate/to-verify), the Overview
key-findings benchmark note, the Sources tab, and the README. Verified via NCDA&CS
Talmadge-Aiken plant directory, NC Meat Processors Association, and business records.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvB48tbAk8juvoi9bxkFTf
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
+++ b/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
@@ -223,13 +223,13 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -881,10 +881,10 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1">
+    <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>•  TWO CORRECTIONS on your benchmarks: (1) Martin's Abattoir (Godwin) CLOSED in 2013 and was primarily a CATTLE plant — not a reliable hog supplier. (2) Nahunta is NC STATE-inspected, NOT USDA-FSIS inspected — which ties directly to your APHIS/EU-export point below.</t>
+          <t>•  BENCHMARK NOTES: (1) Your 'Martin's' incumbent is Martin's Pork Products, Falcon NC — an ACTIVE USDA Talmadge-Aiken slaughter+processing plant (Est. TA-6720, ~75 staff), NOT the unrelated Martin's Abattoir in Godwin (a cattle plant that closed 2013). It's federally FSIS-inspected; the APHIS export listing is separate and still to verify. (2) Nahunta is NC STATE-inspected, not USDA-FSIS — which ties directly to your APHIS/EU-export point below.</t>
         </is>
       </c>
     </row>
@@ -1410,68 +1410,70 @@
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Martin's Abattoir &amp; Wholesale Meats</t>
+          <t>Martin's Pork Products, Inc.</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Godwin, NC</t>
+          <t>Falcon, NC</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>CLOSED 2013 (was cattle/beef)</t>
+          <t>USDA (Talmadge-Aiken) slaughter + processing</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>unknown — 'has volume' (est. mid-size)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Mostly cattle</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>n/a
-(closed)</t>
+          <t>USDA ✓
+(T-A, TA-6720)</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>unknown
+(verify)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>n/a — plant closed</t>
+          <t>Incumbent — 'ok' experience; quality issues harder to resolve (weaker culture/responsiveness than Nahunta); ~75 staff</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Pork slaughter + processing + wholesale</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Possible</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (incumbent)</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>residual: (910) 567-6102</t>
-        </is>
-      </c>
-      <c r="M7" s="15" t="inlineStr">
-        <is>
-          <t>OUT / FLAG</t>
+          <t>(910) 980-1501
+beth@martinspork.com · martinspork.com</t>
+        </is>
+      </c>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -1481,7 +1483,7 @@
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>CORRECTION: Martin's Abattoir CLOSED Sept 2013 (~180 laid off); was primarily a CATTLE/BEEF plant, not a hog specialist. Do not rely on as a hog supplier. Nearby Smithfield 'KC Sausage' sow plant is a different, industrial business.</t>
+          <t>YOUR INCUMBENT (corrected): Martin's Pork Products, Falcon, NC — NOT the unrelated Martin's Abattoir in Godwin (a cattle plant that closed 2013). Active USDA Talmadge-Aiken plant (federal FSIS inspection via NC state inspectors; Est. TA-6720), slaughter + processing since ~2000, ~75 staff, NC Meat Processors Assn member. 'Has volume' per your note — confirm weekly hog count. Federal FSIS confirmed; APHIS export listing separate &amp; to verify (you believe APHIS-certified).</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1556,7 @@
 piedmontcustommeats.com</t>
         </is>
       </c>
-      <c r="M9" s="16" t="inlineStr">
+      <c r="M9" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -1633,7 +1635,7 @@
 acrestationmeatfarm.com</t>
         </is>
       </c>
-      <c r="M10" s="16" t="inlineStr">
+      <c r="M10" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -1710,7 +1712,7 @@
           <t>(252) 235-3558</t>
         </is>
       </c>
-      <c r="M11" s="17" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -1787,7 +1789,7 @@
           <t>(252) 237-2982</t>
         </is>
       </c>
-      <c r="M12" s="17" t="inlineStr">
+      <c r="M12" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -1865,7 +1867,7 @@
 maysmeats.net</t>
         </is>
       </c>
-      <c r="M13" s="17" t="inlineStr">
+      <c r="M13" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -1942,7 +1944,7 @@
           <t>(336) 591-7420</t>
         </is>
       </c>
-      <c r="M14" s="17" t="inlineStr">
+      <c r="M14" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2022,7 +2024,7 @@
 keypackingcompany.com</t>
         </is>
       </c>
-      <c r="M15" s="17" t="inlineStr">
+      <c r="M15" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2100,7 +2102,7 @@
           <t>(252) 332-2978</t>
         </is>
       </c>
-      <c r="M16" s="17" t="inlineStr">
+      <c r="M16" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2177,7 +2179,7 @@
           <t>(336) 667-1346</t>
         </is>
       </c>
-      <c r="M17" s="17" t="inlineStr">
+      <c r="M17" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2254,7 +2256,7 @@
           <t>(704) 786-8616</t>
         </is>
       </c>
-      <c r="M18" s="17" t="inlineStr">
+      <c r="M18" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2331,7 +2333,7 @@
           <t>(336) 949-9696</t>
         </is>
       </c>
-      <c r="M19" s="17" t="inlineStr">
+      <c r="M19" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2408,7 +2410,7 @@
           <t>(828) 245-5544</t>
         </is>
       </c>
-      <c r="M20" s="17" t="inlineStr">
+      <c r="M20" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2488,7 +2490,7 @@
 riversidemeatsnc.com</t>
         </is>
       </c>
-      <c r="M21" s="17" t="inlineStr">
+      <c r="M21" s="16" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -2572,7 +2574,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M23" s="15" t="inlineStr">
+      <c r="M23" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -2649,7 +2651,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M24" s="17" t="inlineStr">
+      <c r="M24" s="16" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -2734,7 +2736,7 @@
 caughmans.com</t>
         </is>
       </c>
-      <c r="M26" s="17" t="inlineStr">
+      <c r="M26" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2812,7 +2814,7 @@
 knockoutbutchery.com</t>
         </is>
       </c>
-      <c r="M27" s="17" t="inlineStr">
+      <c r="M27" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2889,7 +2891,7 @@
           <t>864-374-3571</t>
         </is>
       </c>
-      <c r="M28" s="17" t="inlineStr">
+      <c r="M28" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -2968,7 +2970,7 @@
           <t>803-707-1040</t>
         </is>
       </c>
-      <c r="M29" s="17" t="inlineStr">
+      <c r="M29" s="16" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -3047,7 +3049,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M30" s="15" t="inlineStr">
+      <c r="M30" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -3132,7 +3134,7 @@
 fayettepackingco.com</t>
         </is>
       </c>
-      <c r="M32" s="17" t="inlineStr">
+      <c r="M32" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -3209,7 +3211,7 @@
           <t>931-330-6328</t>
         </is>
       </c>
-      <c r="M33" s="17" t="inlineStr">
+      <c r="M33" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -3287,7 +3289,7 @@
 cherrymeat.com</t>
         </is>
       </c>
-      <c r="M34" s="17" t="inlineStr">
+      <c r="M34" s="16" t="inlineStr">
         <is>
           <t>CAUTION
 (below floor)</t>
@@ -3365,7 +3367,7 @@
           <t>see notes →</t>
         </is>
       </c>
-      <c r="M35" s="17" t="inlineStr">
+      <c r="M35" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -3450,7 +3452,7 @@
 ecofriendly.com</t>
         </is>
       </c>
-      <c r="M37" s="16" t="inlineStr">
+      <c r="M37" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -3528,7 +3530,7 @@
 temeats.com</t>
         </is>
       </c>
-      <c r="M38" s="16" t="inlineStr">
+      <c r="M38" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -3606,7 +3608,7 @@
 blueridgemeats.com</t>
         </is>
       </c>
-      <c r="M39" s="16" t="inlineStr">
+      <c r="M39" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -3685,7 +3687,7 @@
 finestbutcher.com</t>
         </is>
       </c>
-      <c r="M40" s="17" t="inlineStr">
+      <c r="M40" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -3762,7 +3764,7 @@
           <t>see notes →</t>
         </is>
       </c>
-      <c r="M41" s="17" t="inlineStr">
+      <c r="M41" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -3841,7 +3843,7 @@
           <t>see notes →</t>
         </is>
       </c>
-      <c r="M42" s="17" t="inlineStr">
+      <c r="M42" s="16" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -3928,7 +3930,7 @@
 (phone via site)</t>
         </is>
       </c>
-      <c r="M44" s="16" t="inlineStr">
+      <c r="M44" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -4009,7 +4011,7 @@
           <t>smithfieldbioscience.com</t>
         </is>
       </c>
-      <c r="M45" s="16" t="inlineStr">
+      <c r="M45" s="15" t="inlineStr">
         <is>
           <t>STRONG FIT
 (organ exc.)</t>
@@ -4095,7 +4097,7 @@
 lorentzmeats.com</t>
         </is>
       </c>
-      <c r="M47" s="17" t="inlineStr">
+      <c r="M47" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -4175,7 +4177,7 @@
 sigiowa.com</t>
         </is>
       </c>
-      <c r="M48" s="17" t="inlineStr">
+      <c r="M48" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -4253,7 +4255,7 @@
 eickmans.com</t>
         </is>
       </c>
-      <c r="M49" s="17" t="inlineStr">
+      <c r="M49" s="16" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -4331,7 +4333,7 @@
           <t>(712) 837-5334</t>
         </is>
       </c>
-      <c r="M50" s="17" t="inlineStr">
+      <c r="M50" s="16" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -4416,7 +4418,7 @@
           <t>(712) 722-2555</t>
         </is>
       </c>
-      <c r="M52" s="15" t="inlineStr">
+      <c r="M52" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -4493,7 +4495,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M53" s="15" t="inlineStr">
+      <c r="M53" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -4570,7 +4572,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M54" s="15" t="inlineStr">
+      <c r="M54" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -4647,7 +4649,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M55" s="15" t="inlineStr">
+      <c r="M55" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -4724,7 +4726,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="M56" s="15" t="inlineStr">
+      <c r="M56" s="17" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -4808,7 +4810,7 @@
           <t>sinclairbioresources.com</t>
         </is>
       </c>
-      <c r="M58" s="17" t="inlineStr">
+      <c r="M58" s="16" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6878,7 +6880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7146,12 +7148,12 @@
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Nahunta / Martin's corrections</t>
+          <t>Martin's Pork Products (incumbent)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>southernfoodways.org; nahuntapork.com; wcnc.com (Martin's closure); meatpoultry.com</t>
+          <t>NCDA&amp;CS Talmadge-Aiken plant directory (Est. TA-6720); ncmpa.com; D&amp;B/Manta; martinspork.com</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
@@ -7161,41 +7163,41 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Nahunta = NC STATE-inspected (not USDA), ~150 hogs/day. Martin's Abattoir CLOSED Sept 2013, was primarily cattle.</t>
+          <t>CORRECTED to Martin's Pork Products, Falcon NC — active USDA T-A slaughter+processing, ~75 staff, (910) 980-1501, beth@martinspork.com. Distinct from the closed Martin's Abattoir (Godwin, cattle, closed 2013).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>SC facilities</t>
+          <t>Nahunta</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>caughmans.com; knockoutbutchery.com; FSIS notice (Palmetto Fresh suspension); Clemson SCMPID lists (803-788-8747)</t>
-        </is>
-      </c>
-      <c r="C16" s="27" t="inlineStr">
-        <is>
-          <t>Med</t>
+          <t>southernfoodways.org; nahuntapork.com; bitandgrain.com</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Caughman's USDA + family verified; several SC 'deer &amp; hog' shops likely custom-exempt — flag. Palmetto Fresh slaughter suspended Feb 2022.</t>
+          <t>Nahunta = NC STATE-inspected (not USDA-FSIS), ~150 hogs/day, 3rd-gen Pierce family.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>TN facilities</t>
+          <t>SC facilities</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>UT Center for Profitable Agriculture USDA-processor list (cpa.tennessee.edu); company sites</t>
+          <t>caughmans.com; knockoutbutchery.com; FSIS notice (Palmetto Fresh suspension); Clemson SCMPID lists (803-788-8747)</t>
         </is>
       </c>
       <c r="C17" s="27" t="inlineStr">
@@ -7205,85 +7207,85 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>13 USDA hog-slaughter shops listed. Cherry Meat ~80 hogs/month verified. Most well under a few hundred/wk — confirm.</t>
+          <t>Caughman's USDA + family verified; several SC 'deer &amp; hog' shops likely custom-exempt — flag. Palmetto Fresh slaughter suspended Feb 2022.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>VA facilities</t>
+          <t>TN facilities</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>ecofriendly.com; temeats.com; blueridgemeats.com; FSIS listing (Fauquier's); VDACS (omps@vdacs.virginia.gov, 804-786-4569); vabeef.org</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>UT Center for Profitable Agriculture USDA-processor list (cpa.tennessee.edu); company sites</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>Med</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>EcoFriendly Certified Humane; T&amp;E + Blue Ridge AWA — all verified USDA + hog slaughter. Strongest welfare bench.</t>
+          <t>13 USDA hog-slaughter shops listed. Cherry Meat ~80 hogs/month verified. Most well under a few hundred/wk — confirm.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Iowa / Midwest</t>
+          <t>VA facilities</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>postbulletin.com (MRS); smithfieldbioscience.com; proteinintel.com (FSIS est. data); lorentzmeats.com; sigiowa.com; eickmans.com</t>
+          <t>ecofriendly.com; temeats.com; blueridgemeats.com; FSIS listing (Fauquier's); VDACS (omps@vdacs.virginia.gov, 804-786-4569); vabeef.org</t>
         </is>
       </c>
       <c r="C19" s="26" t="inlineStr">
         <is>
-          <t>Med-High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>MRS ~20k/yr verified; Smithfield BioScience organ program verified. Large-packer biologics programs (Seaboard/Prestage/Wholestone) NOT confirmed — do not assume.</t>
+          <t>EcoFriendly Certified Humane; T&amp;E + Blue Ridge AWA — all verified USDA + hog slaughter. Strongest welfare bench.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Authoritative confirmation source</t>
+          <t>Iowa / Midwest</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>USDA FSIS MPI Directory + Establishment Demographic Data — fsis.usda.gov/inspection/establishments</t>
+          <t>postbulletin.com (MRS); smithfieldbioscience.com; proteinintel.com (FSIS est. data); lorentzmeats.com; sigiowa.com; eickmans.com</t>
         </is>
       </c>
       <c r="C20" s="26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Med-High</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Lists species slaughtered + size class per establishment, updated weekly. FSIS blocked automated fetches (Akamai 403) — pull via browser or the 'USDA MPI Directory' mobile app.</t>
+          <t>MRS ~20k/yr verified; Smithfield BioScience organ program verified. Large-packer biologics programs (Seaboard/Prestage/Wholestone) NOT confirmed — do not assume.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>APHIS vs FSIS vs state inspection</t>
+          <t>Authoritative confirmation source</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>aphis.usda.gov/animal-product-export (IREGS); fsis.usda.gov/inspection/import-export</t>
+          <t>USDA FSIS MPI Directory + Establishment Demographic Data — fsis.usda.gov/inspection/establishments</t>
         </is>
       </c>
       <c r="C21" s="26" t="inlineStr">
@@ -7293,19 +7295,19 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Three distinct regimes. APHIS Veterinary Services (not FSIS) is the export pathway for non-food tissue; a state-inspected plant is NOT disqualified from it.</t>
+          <t>Lists species slaughtered + size class per establishment, updated weekly. FSIS blocked automated fetches (Akamai 403) — pull via browser or the 'USDA MPI Directory' mobile app.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>EU animal by-products law</t>
+          <t>APHIS vs FSIS vs state inspection</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>EUR-Lex Reg (EC) 1069/2009; Reg (EU) 142/2011 (legislation.gov.uk consolidated); Annex XIV via Reg (EU) 2022/384</t>
+          <t>aphis.usda.gov/animal-product-export (IREGS); fsis.usda.gov/inspection/import-export</t>
         </is>
       </c>
       <c r="C22" s="26" t="inlineStr">
@@ -7315,19 +7317,19 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Governs import of porcine tissue not for human consumption. Typically Category 3; US is a listed third country; origin establishment must be APHIS-listed on TRACES; APHIS-VS-endorsed model health certificate required.</t>
+          <t>Three distinct regimes. APHIS Veterinary Services (not FSIS) is the export pathway for non-food tissue; a state-inspected plant is NOT disqualified from it.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>EU medical-device angle</t>
+          <t>EU animal by-products law</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>MDR (EU) 2017/745 Annex I 13.1; Reg (EU) 722/2012 (legislation.gov.uk); ISO 22442 (practice)</t>
+          <t>EUR-Lex Reg (EC) 1069/2009; Reg (EU) 142/2011 (legislation.gov.uk consolidated); Annex XIV via Reg (EU) 2022/384</t>
         </is>
       </c>
       <c r="C23" s="26" t="inlineStr">
@@ -7337,27 +7339,49 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>722/2012 (TSE) does NOT cover porcine (bovine/ovine/caprine/deer/elk/mink/cats only). Porcine devices fall under MDR general animal-origin requirements. A training 'model' may not be a device at all — classification call for a specialist/notified body.</t>
+          <t>Governs import of porcine tissue not for human consumption. Typically Category 3; US is a listed third country; origin establishment must be APHIS-listed on TRACES; APHIS-VS-endorsed model health certificate required.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
+          <t>EU medical-device angle</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>MDR (EU) 2017/745 Annex I 13.1; Reg (EU) 722/2012 (legislation.gov.uk); ISO 22442 (practice)</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>722/2012 (TSE) does NOT cover porcine (bovine/ovine/caprine/deer/elk/mink/cats only). Porcine devices fall under MDR general animal-origin requirements. A training 'model' may not be a device at all — classification call for a specialist/notified body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
           <t>APHIS / EU — caveat</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>APHIS VS Field Operations / Veterinary Export Trade Services; EU importer; notified body</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>NOT legal advice. Exact ABP category, CN code, and 142/2011 model certificate must be confirmed per product line with APHIS VS and a customs/regulatory specialist.</t>
         </is>

</xml_diff>

<commit_message>
Split volume tiers into four: add Medium-High 2,500-5,000, High now >5,000
Volume tiers are now SMALL 0-300/wk, MEDIUM 350-2,500/wk, MEDIUM-HIGH 2,500-5,000/wk,
HIGH >5,000/wk. Medium-High is where regional packers and cull-sow plants cluster
(~500-1,000 head/day) — sow anatomy is also closer to adult human scale, a potential
advantage for pelvic and bariatric blocks.

Re-tiered existing entries against the new boundaries (Smithfield/KC Sausage sow plant
moves to Medium-High), added the fourth band to the roster colour coding and the legend,
and updated the Overview requirements, meeting agenda and README.

Re-investigation to expand the roster under the open-capacity criteria is in progress.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvB48tbAk8juvoi9bxkFTf
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
+++ b/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
@@ -35,7 +35,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -128,6 +128,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00833C0C"/>
       <sz val="10"/>
     </font>
@@ -153,7 +159,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -208,6 +214,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -296,7 +307,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -376,7 +387,10 @@
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -391,11 +405,14 @@
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -412,13 +429,13 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -451,16 +468,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -469,7 +486,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -489,7 +506,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -899,7 +916,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Weekly kill volume — OPEN</t>
@@ -907,7 +924,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>CAPACITY IS NOT A FILTER. No plant is excluded for being too small or too large; every supplier is listed and CLASSIFIED into a volume tier instead:  SMALL 0–300/wk  ·  MEDIUM 350–2,500/wk  ·  HIGH over 2,500/wk. Use the tier to decide the operating model and whether aggregation is needed — see 'Legend &amp; Scoring'. (301–349/wk is the Small/Medium boundary.)</t>
+          <t>CAPACITY IS NOT A FILTER. No plant is excluded for being too small or too large; every supplier is listed and CLASSIFIED into a volume tier instead:  SMALL 0–300/wk  ·  MEDIUM 350–2,500/wk  ·  MEDIUM-HIGH 2,500–5,000/wk  ·  HIGH over 5,000/wk. Use the tier to decide the operating model and whether aggregation is needed — see 'Legend &amp; Scoring'. (301–349/wk is the Small/Medium boundary; 2,500/wk is the Medium / Medium-High hinge.)</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1113,7 @@
           <t>•  BEST OVERALL FIT — Midwest Research Swine (Glencoe/Gibbon, MN): a porcine-ONLY abattoir already harvesting whole organs and tissue for biomedical/xeno research at ~385 hogs/week (in-band), closed herd, holds USDA APHIS licenses. It is essentially your exact operation at your exact scale — contact first.</t>
         </is>
       </c>
-      <c r="B26" s="62" t="n"/>
+      <c r="B26" s="64" t="n"/>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1104,7 +1121,7 @@
           <t>•  LARGE-BUT-ACCEPTABLE via the organ exception — Smithfield BioScience (Denison, IA + Monmouth IL / Milan MO): ~10,000 hogs/day, but runs a full in-house porcine harvest program spanning all three of your target regions (pelvic, abdominal, thoracic) to customer spec. Natural Model B partner; the one giant packer that qualifies.</t>
         </is>
       </c>
-      <c r="B27" s="62" t="n"/>
+      <c r="B27" s="64" t="n"/>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1112,7 +1129,7 @@
           <t>•  NORTH CAROLINA best new fits — Piedmont Custom Meats (Gibsonville/Asheboro): USDA + AWA humane + runs a SEPARATE dedicated harvesting facility (best structural match for Model A or B); and Acre Station Meat Farm (Pinetown): USDA-equivalent, ~80 hogs/day (~400/wk), AWA. Both squarely in-band.</t>
         </is>
       </c>
-      <c r="B28" s="62" t="n"/>
+      <c r="B28" s="64" t="n"/>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1120,7 +1137,7 @@
           <t>•  BENCHMARK NOTES: (1) Your 'Martin's' incumbent is Martin's Pork Products, Falcon NC — an ACTIVE USDA Talmadge-Aiken slaughter+processing plant (Est. TA-6720, ~75 staff), NOT the unrelated Martin's Abattoir in Godwin (a cattle plant that closed 2013). It's federally FSIS-inspected; the APHIS export listing is separate and still to verify. (2) Nahunta is NC STATE-inspected, not USDA-FSIS — which ties directly to your APHIS/EU-export point below.</t>
         </is>
       </c>
-      <c r="B29" s="62" t="n"/>
+      <c r="B29" s="64" t="n"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -1128,7 +1145,7 @@
           <t>•  VIRGINIA welfare bench (updated after the enforcement pass): T&amp;E Meats (Harrisonburg, AWA) and Blue Ridge Meats (Middletown, AWA) are the LIVE, humane, USDA-inspected picks — the closest match to the Nahunta standard and a natural Model B fit. Two caveats: EcoFriendly Foods (Certified Humane) reportedly CEASED operations ~2020 — verify before relying on it; and Fauquier's Finest has REPEAT humane-handling suspensions (2018/2021/2024), now downgraded to CAUTION.</t>
         </is>
       </c>
-      <c r="B30" s="62" t="n"/>
+      <c r="B30" s="64" t="n"/>
     </row>
     <row r="31" ht="84" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -1136,7 +1153,7 @@
           <t>•  USDA/FSIS ENFORCEMENT (new roster column): several plants carry documented FSIS humane-handling actions — flagged with ⚠ and re-scored to CAUTION: Fauquier's Finest (VA, repeat), Thomas Brothers (NC, repeat), Wayne Mays (NC), M.L. Mitchell (NC), Triad Meat (NC), plus a single 2023 action at Fayette Packing (TN). Among large packers, Smithfield-Denison, Sioux-Preme/Perdue, Prestage and Wholestone all have humane-handling records. Given your 'Nahunta test', weigh these heavily. IMPORTANT: 'none found' for the small plants means no PUBLIC record — not a clean bill (FSIS data was only reachable via search snippets).</t>
         </is>
       </c>
-      <c r="B31" s="62" t="n"/>
+      <c r="B31" s="64" t="n"/>
     </row>
     <row r="32" ht="72" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -1144,7 +1161,7 @@
           <t>•  BUY-DIRECT × EU EXPORT: buying finished tissue can HELP or HURT EU-export eligibility depending on the vendor. Your cheapest published-price vendor, Innovative Research, labels tissue 'research use only, not for human or animal use' — a LIKELY BLOCKER for EU device-bound product. EU-cleanest vendors (ISO 13485/22442, human-food-chain traceability): Tissue Source, Smithfield BioScience, Midwest Research Swine, SSR. See the 'EU-export fit' column on the National Direct Suppliers tab.</t>
         </is>
       </c>
-      <c r="B32" s="62" t="n"/>
+      <c r="B32" s="64" t="n"/>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -1152,7 +1169,7 @@
           <t>•  HOW TO CHECK APHIS/EXPORT YOURSELF: no facility could be confirmed EU/APHIS-listed for research tissue; six large plants are FSIS export-certified for EDIBLE meat only (not the same thing). The 'APHIS &amp; EU Export' tab now lists the exact websites — FSIS 'Eligible Establishments by Country', the APHIS Export-to-EU page (research tissue goes through APHIS VS), and EU TRACES-NT.</t>
         </is>
       </c>
-      <c r="B33" s="62" t="n"/>
+      <c r="B33" s="64" t="n"/>
     </row>
     <row r="34" ht="72" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -1160,7 +1177,7 @@
           <t>•  CAPACITY IS NOW OPEN — no plant is excluded on size. Every supplier is classified into a VOLUME TIER instead: SMALL 0-300/wk, MEDIUM 350-2,500/wk, HIGH over 2,500/wk. Current spread across the 44 roster entries: 13 SMALL, 4 MEDIUM, 8 HIGH, 18 still to confirm on the call. This brings back plants previously dropped on throughput (Piedmont, Acre Station, Cherry Meat, EcoFriendly, the small custom shops) and un-excludes the large packers — the constraint at HIGH tier is ACCESS, not volume.</t>
         </is>
       </c>
-      <c r="B34" s="62" t="n"/>
+      <c r="B34" s="64" t="n"/>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -1168,7 +1185,7 @@
           <t>•  SC/TN/VA reality: there are essentially NO mid-industrial hog plants in these states — the pool is small custom/USDA shops (mostly SMALL tier, e.g. Cherry Meat TN ~18/wk). With capacity open these are legitimate high-touch Model A/B partners and AGGREGATION candidates; they simply cannot carry volume individually.</t>
         </is>
       </c>
-      <c r="B35" s="62" t="n"/>
+      <c r="B35" s="64" t="n"/>
     </row>
     <row r="36" ht="84" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -1176,7 +1193,7 @@
           <t>•  APHIS / EU EXPORT (now investigated — see dedicated tab): the EU does NOT require suppliers to hand you a standalone 'APHIS certificate.' It requires the ORIGIN plant to be APHIS-approved and listed on the EU TRACES establishment list for the right animal-by-product category (typically Category 3 under Reg (EU) 142/2011), PLUS an APHIS Veterinary Services-endorsed health certificate that YOUR company carries as the exporter. A state-inspected plant (like Nahunta) CAN still qualify — APHIS listing, not an FSIS grant, is the key. No candidate plant's APHIS listing could be verified, so it is the top diligence item for every shortlist plant.</t>
         </is>
       </c>
-      <c r="B36" s="62" t="n"/>
+      <c r="B36" s="64" t="n"/>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -1184,7 +1201,7 @@
           <t>•  NATIONAL DIRECT VENDORS are almost all QUOTE-ONLY. The only published price anchors: Innovative Research ~$141 per single porcine organ and $582 for a full pelvic block (list, base config); Pel-Freez porcine thyroid $361. Tissue Source and ABI stand out on regulatory pedigree (ISO 13485 / USDA-inspected sourcing) if you need EU-grade traceability.</t>
         </is>
       </c>
-      <c r="B37" s="62" t="n"/>
+      <c r="B37" s="64" t="n"/>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -1192,7 +1209,7 @@
           <t>•  MAKE-VS-BUY: self-harvest is generally cheaper per tissue when you pull multiple blocks from one hog and already have labor + cold-chain + abattoir access; buying direct wins for low/irregular volume, or when you need certified traceability you can't yet document in-house (again, the EU-export angle).</t>
         </is>
       </c>
-      <c r="B38" s="62" t="n"/>
+      <c r="B38" s="64" t="n"/>
     </row>
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -1200,7 +1217,7 @@
           <t>•  ALWAYS VERIFY BY PHONE: nearly every weekly-volume and certification figure for small/custom plants is unpublished. Use the 'Call Question Sheet' tab; the authoritative confirmation source is the USDA FSIS MPI Directory + Establishment Demographic Data (species slaughtered + size class per plant).</t>
         </is>
       </c>
-      <c r="B39" s="62" t="n"/>
+      <c r="B39" s="64" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="24">
@@ -1262,7 +1279,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="56" t="inlineStr"/>
+      <c r="A4" s="58" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Plant / contact</t>
@@ -1271,7 +1288,7 @@
       <c r="C4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="56" t="inlineStr"/>
+      <c r="A5" s="58" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Phone / email</t>
@@ -1280,7 +1297,7 @@
       <c r="C5" s="8" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="56" t="inlineStr"/>
+      <c r="A6" s="58" t="inlineStr"/>
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Date of call / caller</t>
@@ -1289,31 +1306,31 @@
       <c r="C6" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="41" t="inlineStr">
+      <c r="A8" s="43" t="inlineStr">
         <is>
           <t>A. HARD GATE — volume &amp; species</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="52" t="inlineStr">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B9" s="52" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C9" s="52" t="inlineStr">
+      <c r="C9" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="59" t="n">
+      <c r="A10" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1324,7 +1341,7 @@
       <c r="C10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="59" t="n">
+      <c r="A11" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1335,7 +1352,7 @@
       <c r="C11" s="8" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="59" t="n">
+      <c r="A12" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1346,31 +1363,31 @@
       <c r="C12" s="8" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
+      <c r="A14" s="43" t="inlineStr">
         <is>
           <t>B. Inspection &amp; certification</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="52" t="inlineStr">
+      <c r="A15" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B15" s="52" t="inlineStr">
+      <c r="B15" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C15" s="52" t="inlineStr">
+      <c r="C15" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="59" t="n">
+      <c r="A16" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1381,7 +1398,7 @@
       <c r="C16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="59" t="n">
+      <c r="A17" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1392,7 +1409,7 @@
       <c r="C17" s="8" t="inlineStr"/>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="59" t="n">
+      <c r="A18" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1403,7 +1420,7 @@
       <c r="C18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="59" t="n">
+      <c r="A19" s="61" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1414,31 +1431,31 @@
       <c r="C19" s="8" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="41" t="inlineStr">
+      <c r="A21" s="43" t="inlineStr">
         <is>
           <t>C. Tissue &amp; organ harvesting</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="52" t="inlineStr">
+      <c r="A22" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B22" s="52" t="inlineStr">
+      <c r="B22" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C22" s="52" t="inlineStr">
+      <c r="C22" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="59" t="n">
+      <c r="A23" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1449,7 +1466,7 @@
       <c r="C23" s="8" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="59" t="n">
+      <c r="A24" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1460,7 +1477,7 @@
       <c r="C24" s="8" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="59" t="n">
+      <c r="A25" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1471,7 +1488,7 @@
       <c r="C25" s="8" t="inlineStr"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="59" t="n">
+      <c r="A26" s="61" t="n">
         <v>4</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1482,31 +1499,31 @@
       <c r="C26" s="8" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="41" t="inlineStr">
+      <c r="A28" s="43" t="inlineStr">
         <is>
           <t>D. Operating model fit</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="52" t="inlineStr">
+      <c r="A29" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B29" s="52" t="inlineStr">
+      <c r="B29" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C29" s="52" t="inlineStr">
+      <c r="C29" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="59" t="n">
+      <c r="A30" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1517,7 +1534,7 @@
       <c r="C30" s="8" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="59" t="n">
+      <c r="A31" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1528,7 +1545,7 @@
       <c r="C31" s="8" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="59" t="n">
+      <c r="A32" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1539,31 +1556,31 @@
       <c r="C32" s="8" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="41" t="inlineStr">
+      <c r="A34" s="43" t="inlineStr">
         <is>
           <t>E. Culture &amp; workforce (the Nahunta test)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="52" t="inlineStr">
+      <c r="A35" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B35" s="52" t="inlineStr">
+      <c r="B35" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C35" s="52" t="inlineStr">
+      <c r="C35" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="59" t="n">
+      <c r="A36" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1574,7 +1591,7 @@
       <c r="C36" s="8" t="inlineStr"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="59" t="n">
+      <c r="A37" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1585,7 +1602,7 @@
       <c r="C37" s="8" t="inlineStr"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="59" t="n">
+      <c r="A38" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -1596,31 +1613,31 @@
       <c r="C38" s="8" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="41" t="inlineStr">
+      <c r="A40" s="43" t="inlineStr">
         <is>
           <t>F. Commercial</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="52" t="inlineStr">
+      <c r="A41" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B41" s="52" t="inlineStr">
+      <c r="B41" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C41" s="52" t="inlineStr">
+      <c r="C41" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="59" t="n">
+      <c r="A42" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -1631,7 +1648,7 @@
       <c r="C42" s="8" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="59" t="n">
+      <c r="A43" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1642,7 +1659,7 @@
       <c r="C43" s="8" t="inlineStr"/>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="59" t="n">
+      <c r="A44" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -1653,31 +1670,31 @@
       <c r="C44" s="8" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="41" t="inlineStr">
+      <c r="A46" s="43" t="inlineStr">
         <is>
           <t>G. EU-EXPORT ELIGIBILITY — APHIS / animal by-products (ask if models go to Europe)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="52" t="inlineStr">
+      <c r="A47" s="54" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B47" s="52" t="inlineStr">
+      <c r="B47" s="54" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C47" s="52" t="inlineStr">
+      <c r="C47" s="54" t="inlineStr">
         <is>
           <t>Answer / Notes</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="59" t="n">
+      <c r="A48" s="61" t="n">
         <v>1</v>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -1688,7 +1705,7 @@
       <c r="C48" s="8" t="inlineStr"/>
     </row>
     <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="59" t="n">
+      <c r="A49" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -1699,7 +1716,7 @@
       <c r="C49" s="8" t="inlineStr"/>
     </row>
     <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="59" t="n">
+      <c r="A50" s="61" t="n">
         <v>3</v>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -1710,7 +1727,7 @@
       <c r="C50" s="8" t="inlineStr"/>
     </row>
     <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="59" t="n">
+      <c r="A51" s="61" t="n">
         <v>4</v>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -1721,7 +1738,7 @@
       <c r="C51" s="8" t="inlineStr"/>
     </row>
     <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="59" t="n">
+      <c r="A52" s="61" t="n">
         <v>5</v>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -1777,22 +1794,22 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="52" t="inlineStr">
+      <c r="A4" s="54" t="inlineStr">
         <is>
           <t>Topic / entity</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="54" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="C4" s="52" t="inlineStr">
+      <c r="C4" s="54" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -1809,7 +1826,7 @@
           <t>innov-research.com porcine product pages (heart/lung/kidney/bladder/liver/stomach/pelvic-block)</t>
         </is>
       </c>
-      <c r="C5" s="60" t="inlineStr">
+      <c r="C5" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1831,7 +1848,7 @@
           <t>pel-freez.com/pig-thyroid-59452</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1853,7 +1870,7 @@
           <t>animaltechnologies.com/porcine</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C7" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1875,7 +1892,7 @@
           <t>animalbiotech.com/porcine-tissues</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1897,7 +1914,7 @@
           <t>tissue-source.com</t>
         </is>
       </c>
-      <c r="C9" s="60" t="inlineStr">
+      <c r="C9" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1919,7 +1936,7 @@
           <t>smithfieldbioscience.com/products/porcine</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1941,7 +1958,7 @@
           <t>wgbiomedical.com</t>
         </is>
       </c>
-      <c r="C11" s="60" t="inlineStr">
+      <c r="C11" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1963,7 +1980,7 @@
           <t>respective vendor sites (see National tab)</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1985,7 +2002,7 @@
           <t>premierbiosource.com; sciencecare.com; zivic listing</t>
         </is>
       </c>
-      <c r="C13" s="60" t="inlineStr">
+      <c r="C13" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2007,7 +2024,7 @@
           <t>NCDA&amp;CS Meat &amp; Poultry Inspection 'plants that slaughter for farmers' (via cefs.ncsu.edu PDF, dated Oct 2018); div. 919-707-3180</t>
         </is>
       </c>
-      <c r="C14" s="61" t="inlineStr">
+      <c r="C14" s="63" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -2029,7 +2046,7 @@
           <t>NCDA&amp;CS Talmadge-Aiken plant directory (Est. TA-6720); ncmpa.com; D&amp;B/Manta; martinspork.com</t>
         </is>
       </c>
-      <c r="C15" s="60" t="inlineStr">
+      <c r="C15" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2051,7 +2068,7 @@
           <t>southernfoodways.org; nahuntapork.com; bitandgrain.com</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2073,7 +2090,7 @@
           <t>caughmans.com; knockoutbutchery.com; FSIS notice (Palmetto Fresh suspension); Clemson SCMPID lists (803-788-8747)</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C17" s="63" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -2095,7 +2112,7 @@
           <t>UT Center for Profitable Agriculture USDA-processor list (cpa.tennessee.edu); company sites</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr">
+      <c r="C18" s="63" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -2117,7 +2134,7 @@
           <t>ecofriendly.com; temeats.com; blueridgemeats.com; FSIS listing (Fauquier's); VDACS (omps@vdacs.virginia.gov, 804-786-4569); vabeef.org</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2139,7 +2156,7 @@
           <t>postbulletin.com (MRS); smithfieldbioscience.com; proteinintel.com (FSIS est. data); lorentzmeats.com; sigiowa.com; eickmans.com</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="62" t="inlineStr">
         <is>
           <t>Med-High</t>
         </is>
@@ -2161,7 +2178,7 @@
           <t>USDA FSIS MPI Directory + Establishment Demographic Data — fsis.usda.gov/inspection/establishments</t>
         </is>
       </c>
-      <c r="C21" s="60" t="inlineStr">
+      <c r="C21" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2183,7 +2200,7 @@
           <t>aphis.usda.gov/animal-product-export (IREGS); fsis.usda.gov/inspection/import-export</t>
         </is>
       </c>
-      <c r="C22" s="60" t="inlineStr">
+      <c r="C22" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2205,7 +2222,7 @@
           <t>EUR-Lex Reg (EC) 1069/2009; Reg (EU) 142/2011 (legislation.gov.uk consolidated); Annex XIV via Reg (EU) 2022/384</t>
         </is>
       </c>
-      <c r="C23" s="60" t="inlineStr">
+      <c r="C23" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2227,7 +2244,7 @@
           <t>MDR (EU) 2017/745 Annex I 13.1; Reg (EU) 722/2012 (legislation.gov.uk); ISO 22442 (practice)</t>
         </is>
       </c>
-      <c r="C24" s="60" t="inlineStr">
+      <c r="C24" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2249,7 +2266,7 @@
           <t>APHIS VS Field Operations / Veterinary Export Trade Services; EU importer; notified body</t>
         </is>
       </c>
-      <c r="C25" s="61" t="inlineStr">
+      <c r="C25" s="63" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -2271,7 +2288,7 @@
           <t>FSIS Quarterly Enforcement Reports &amp; NOS/NOIE PDFs; AWI Humane Slaughter suspension list; PETA/ASPCA releases; local news</t>
         </is>
       </c>
-      <c r="C26" s="60" t="inlineStr">
+      <c r="C26" s="62" t="inlineStr">
         <is>
           <t>Med-High</t>
         </is>
@@ -2293,7 +2310,7 @@
           <t>FSIS 'Eligible Establishments by Country' + EU page; FSIS MPI directory; APHIS Export-to-EU (VS); EU TRACES-NT; usda-eu.org</t>
         </is>
       </c>
-      <c r="C27" s="60" t="inlineStr">
+      <c r="C27" s="62" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2315,7 +2332,7 @@
           <t>Vendor sites (ISO/USDA claims); Reg (EC) 1069/2009 &amp; (EU) 142/2011; MDR Annex I 13.1 / ISO 22442</t>
         </is>
       </c>
-      <c r="C28" s="60" t="inlineStr">
+      <c r="C28" s="62" t="inlineStr">
         <is>
           <t>Med-High</t>
         </is>
@@ -2355,7 +2372,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="64" t="inlineStr">
+      <c r="A1" s="66" t="inlineStr">
         <is>
           <t>Deep Study — Multi-Agent Re-Research with Adversarial Verification</t>
         </is>
@@ -2369,7 +2386,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="65" t="inlineStr">
+      <c r="A4" s="67" t="inlineStr">
         <is>
           <t>KEY FINDINGS  (ranked by decision impact)</t>
         </is>
@@ -2453,7 +2470,7 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="65" t="inlineStr">
+      <c r="A17" s="67" t="inlineStr">
         <is>
           <t>WHAT THE VERIFICATION CHANGED  (vs. the first pass)</t>
         </is>
@@ -2580,7 +2597,7 @@
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="65" t="inlineStr">
+      <c r="A29" s="67" t="inlineStr">
         <is>
           <t>RECOMMENDED CONTACT ORDER  (post-verification)</t>
         </is>
@@ -2609,7 +2626,7 @@
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="57" t="n">
+      <c r="A31" s="59" t="n">
         <v>1</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -2629,7 +2646,7 @@
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="57" t="n">
+      <c r="A32" s="59" t="n">
         <v>2</v>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2649,7 +2666,7 @@
       </c>
     </row>
     <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="57" t="n">
+      <c r="A33" s="59" t="n">
         <v>3</v>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2669,7 +2686,7 @@
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="57" t="n">
+      <c r="A34" s="59" t="n">
         <v>4</v>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2689,7 +2706,7 @@
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="57" t="n">
+      <c r="A35" s="59" t="n">
         <v>5</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2709,7 +2726,7 @@
       </c>
     </row>
     <row r="36" ht="36" customHeight="1">
-      <c r="A36" s="57" t="n">
+      <c r="A36" s="59" t="n">
         <v>6</v>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2729,7 +2746,7 @@
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="57" t="n">
+      <c r="A37" s="59" t="n">
         <v>7</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2749,7 +2766,7 @@
       </c>
     </row>
     <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="57" t="n">
+      <c r="A38" s="59" t="n">
         <v>8</v>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2769,7 +2786,7 @@
       </c>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="57" t="n">
+      <c r="A39" s="59" t="n">
         <v>9</v>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2789,7 +2806,7 @@
       </c>
     </row>
     <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="57" t="n">
+      <c r="A40" s="59" t="n">
         <v>10</v>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2809,7 +2826,7 @@
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="65" t="inlineStr">
+      <c r="A42" s="67" t="inlineStr">
         <is>
           <t>VERIFIED FACILITY ROSTER</t>
         </is>
@@ -2858,7 +2875,7 @@
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="65" t="inlineStr">
+      <c r="A44" s="67" t="inlineStr">
         <is>
           <t>ADVERSARIALLY VERIFIED — these verdicts override the earlier tabs</t>
         </is>
@@ -2885,7 +2902,7 @@
           <t>NC STATE only (P-80A slaughter, swine-only; P-80 processing)</t>
         </is>
       </c>
-      <c r="E45" s="38" t="inlineStr">
+      <c r="E45" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -2925,7 +2942,7 @@
           <t>USDA Talmadge-Aiken TA-6720 (federal, exportable structure)</t>
         </is>
       </c>
-      <c r="E46" s="38" t="inlineStr">
+      <c r="E46" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -2965,7 +2982,7 @@
           <t>Talmadge-Aiken TA-19904 / M19904 — but 2 directories say CUSTOM EXEMPT</t>
         </is>
       </c>
-      <c r="E47" s="38" t="inlineStr">
+      <c r="E47" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3005,7 +3022,7 @@
           <t>USDA-FSIS M7975 / M7975A (V7975 = Voluntary, not poultry)</t>
         </is>
       </c>
-      <c r="E48" s="38" t="inlineStr">
+      <c r="E48" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3045,7 +3062,7 @@
           <t>USDA-FSIS M7420 + V7420</t>
         </is>
       </c>
-      <c r="E49" s="36" t="inlineStr">
+      <c r="E49" s="38" t="inlineStr">
         <is>
           <t>UNCERTAIN</t>
         </is>
@@ -3085,7 +3102,7 @@
           <t>USDA-FSIS M4005 + P4005 + V4005</t>
         </is>
       </c>
-      <c r="E50" s="38" t="inlineStr">
+      <c r="E50" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3125,7 +3142,7 @@
           <t>USDA-FSIS M9065 + P9065 + V9065</t>
         </is>
       </c>
-      <c r="E51" s="38" t="inlineStr">
+      <c r="E51" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3165,7 +3182,7 @@
           <t>USDA-FSIS M7455</t>
         </is>
       </c>
-      <c r="E52" s="38" t="inlineStr">
+      <c r="E52" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3205,7 +3222,7 @@
           <t>USDA-FSIS M8314 + V8314</t>
         </is>
       </c>
-      <c r="E53" s="38" t="inlineStr">
+      <c r="E53" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3245,7 +3262,7 @@
           <t>USDA-FSIS M21938</t>
         </is>
       </c>
-      <c r="E54" s="38" t="inlineStr">
+      <c r="E54" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN</t>
         </is>
@@ -3265,7 +3282,7 @@
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="65" t="inlineStr">
+      <c r="A55" s="67" t="inlineStr">
         <is>
           <t>NEWLY SURFACED — never in the earlier study (NOT yet adversarially verified)</t>
         </is>
@@ -3412,7 +3429,7 @@
           <t>unknown — establishment number not found by any public source</t>
         </is>
       </c>
-      <c r="E59" s="38" t="inlineStr">
+      <c r="E59" s="40" t="inlineStr">
         <is>
           <t>CONFIRMED OPEN (EPA permits)</t>
         </is>
@@ -3512,7 +3529,7 @@
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="65" t="inlineStr">
+      <c r="A63" s="67" t="inlineStr">
         <is>
           <t>COMPLETENESS CRITIC — what we still don't know / didn't cover</t>
         </is>
@@ -3589,7 +3606,7 @@
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="65" t="inlineStr">
+      <c r="A75" s="67" t="inlineStr">
         <is>
           <t>STRATEGIC READ  (given the 200-3,000/wk floor + EU export)</t>
         </is>
@@ -3652,42 +3669,42 @@
       </c>
     </row>
     <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="65" t="inlineStr">
+      <c r="A85" s="67" t="inlineStr">
         <is>
           <t>METHOD &amp; CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="86" ht="36" customHeight="1">
-      <c r="A86" s="66" t="inlineStr">
+      <c r="A86" s="68" t="inlineStr">
         <is>
           <t>•  Run as a 5-phase multi-agent workflow: Discover (6 parallel regional/national sweeps) → Compliance (3 sweeps: USDA/FSIS enforcement x2 + APHIS/EU export mechanics) → Verify (10 adversarial verifiers, high reasoning effort) → Completeness critic → Executive synthesis.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="66" t="inlineStr">
+      <c r="A87" s="68" t="inlineStr">
         <is>
           <t>•  21 agents · 121 raw facility records (see caveat on double-counting) · 10 candidates adversarially verified · ~2.0M tokens · 1,091 tool calls · 0 agent errors.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="48" customHeight="1">
-      <c r="A88" s="66" t="inlineStr">
+      <c r="A88" s="68" t="inlineStr">
         <is>
           <t>•  Verifiers were instructed to REFUTE rather than confirm, and were pointed at the specific failure modes that had already produced errors: identity confusion (the Martin's Falcon vs Martin's Abattoir Godwin case, supplied as a worked example), closure/operating status, cut-and-wrap vs on-site slaughter, capacity-vs-actual volume, inspection-type confusion, welfare branding vs enforcement record, and stale contact details.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="24" customHeight="1">
-      <c r="A89" s="66" t="inlineStr">
+      <c r="A89" s="68" t="inlineStr">
         <is>
           <t>•  Result: of 10 verified candidates, 2 were PROMOTED, 6 DOWNGRADED, and 2 KILLED — including both of the earlier pass's top picks in NC and VA. This tab's verdicts take precedence over the earlier tabs wherever they disagree.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="24" customHeight="1">
-      <c r="A90" s="66" t="inlineStr">
+      <c r="A90" s="68" t="inlineStr">
         <is>
           <t>•  Confidence vocabulary used throughout: VERIFIED (primary source cited) · INFERRED (reasoned from verified facts) · UNVERIFIED (asserted, not confirmed) · NONE FOUND (absence of public record, which is NOT proof of a clean record).</t>
         </is>
@@ -4419,11 +4436,11 @@
           <t>Subject:  Request for Quote / Proposal — Recurring Porcine Tissue Harvesting Partnership</t>
         </is>
       </c>
-      <c r="B31" s="63" t="n"/>
-      <c r="C31" s="63" t="n"/>
-      <c r="D31" s="63" t="n"/>
-      <c r="E31" s="63" t="n"/>
-      <c r="F31" s="62" t="n"/>
+      <c r="B31" s="65" t="n"/>
+      <c r="C31" s="65" t="n"/>
+      <c r="D31" s="65" t="n"/>
+      <c r="E31" s="65" t="n"/>
+      <c r="F31" s="64" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
@@ -4691,9 +4708,9 @@
           <t>WHY THIS IS ACTION #1: whether your models can use CULL-SOW anatomy decides the fate of roughly half the candidate pool, and NO amount of further research can answer it — it is a client-side clinical decision. A heavily parous sow has a REMODELLED BIRTH CANAL and a STRETCHED ABDOMINAL WALL: either disqualifying for pelvic and bariatric blocks, or a premium urogynaecology asset. Sow plants currently on the list: Gunnoe (VA), Kansas City Sausage (NC), Swaggerty (TN), Wampler's (TN), Williams/Tyson (TN). Fill this in BEFORE the first supplier call — it reorders the entire contact list.</t>
         </is>
       </c>
-      <c r="B4" s="63" t="n"/>
-      <c r="C4" s="63" t="n"/>
-      <c r="D4" s="62" t="n"/>
+      <c r="B4" s="65" t="n"/>
+      <c r="C4" s="65" t="n"/>
+      <c r="D4" s="64" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -4912,8 +4929,8 @@
           <t>Circle one:   MARKET HOG ONLY   /   SOW ACCEPTABLE   /   SOW PREFERRED (urogyn)   /   DEPENDS BY BLOCK (specify above)</t>
         </is>
       </c>
-      <c r="C27" s="63" t="n"/>
-      <c r="D27" s="62" t="n"/>
+      <c r="C27" s="65" t="n"/>
+      <c r="D27" s="64" t="n"/>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
@@ -4926,8 +4943,8 @@
           <t>Remove Gunnoe (VA), Kansas City Sausage (NC), Swaggerty (TN) and probably Wampler's and Williams/Tyson (TN) from the list. That leaves the NC Talmadge-Aiken swine plants (Martin's, Larry's, Bass Farms) plus Nahunta as essentially the entire realistic pool — and makes the eastern-NC cluster strategy close to mandatory.</t>
         </is>
       </c>
-      <c r="C28" s="63" t="n"/>
-      <c r="D28" s="62" t="n"/>
+      <c r="C28" s="65" t="n"/>
+      <c r="D28" s="64" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
@@ -4940,8 +4957,8 @@
           <t>The pool roughly doubles and several in-band plants come back: Gunnoe (~450-590/wk), Kansas City Sausage (~3,500-5,000/wk), plus the TN sow plants. Sow anatomy is also closer to ADULT HUMAN SCALE than a 250 lb market hog, which may be a product advantage.</t>
         </is>
       </c>
-      <c r="C29" s="63" t="n"/>
-      <c r="D29" s="62" t="n"/>
+      <c r="C29" s="65" t="n"/>
+      <c r="D29" s="64" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
@@ -4954,8 +4971,8 @@
           <t>Which blocks (if any) are destined for EUROPE?  EU-bound product cannot come from Nahunta (state-inspected, NC sales only) and requires a federally-inspected plant plus APHIS/TRACES listing. Domestic-only product has no such constraint.</t>
         </is>
       </c>
-      <c r="C30" s="63" t="n"/>
-      <c r="D30" s="62" t="n"/>
+      <c r="C30" s="65" t="n"/>
+      <c r="D30" s="64" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
@@ -4968,8 +4985,8 @@
           <t>If max warm ischemia is TIGHT (minutes), Model A on-site harvesting is effectively mandatory and buy-direct is out. If it is loose (hours), buy-direct and Model B both stay viable — which materially widens the supplier pool.</t>
         </is>
       </c>
-      <c r="C31" s="63" t="n"/>
-      <c r="D31" s="62" t="n"/>
+      <c r="C31" s="65" t="n"/>
+      <c r="D31" s="64" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="18" t="inlineStr">
@@ -5002,7 +5019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5090,7 +5107,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
         <is>
           <t>SMALL — 0-300 hogs/week</t>
@@ -5098,7 +5115,7 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>High-touch, family-scale, often the best welfare culture and the easiest to negotiate bespoke access with. Best for Model A (our harvesters on their floor) and for pilot/low-volume tissue programs. May need AGGREGATION across several plants to hit volume.</t>
+          <t>High-touch, family-scale, often the best welfare culture and the easiest to negotiate bespoke access with. Best for Model A (our harvesters on their floor) and for pilot / low-volume tissue programs. Usually needs AGGREGATION across several nearby plants to reach meaningful volume — which only works if they are close enough to share one crew.</t>
         </is>
       </c>
     </row>
@@ -5110,187 +5127,199 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>The sweet spot for a recurring single-plant program: enough throughput to matter, small enough to still be relationship-driven and to accommodate a third-party harvest crew. Both Model A and Model B are realistic here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
+          <t>The sweet spot for a recurring single-plant program: enough throughput to matter, small enough to stay relationship-driven and to accommodate a third-party harvest crew. Both Model A and Model B are realistic. Note this band is genuinely scarce in the US.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>HIGH — over 2,500 hogs/week</t>
+          <t>MEDIUM-HIGH — 2,500-5,000 hogs/week</t>
         </is>
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>Industrial scale. Volume is never the constraint; ACCESS is. Realistically Model B (they harvest to our spec) or a biologics/organ program. Worth pursuing where a plant already runs organ/tissue harvesting, or where sow anatomy is wanted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+          <t>Regional packers and CULL-SOW plants cluster here (~500-1,000 head/day). Volume is comfortable and sow anatomy is closer to adult human scale — potentially a product advantage for pelvic and bariatric blocks. Access is negotiable but more structured than at Medium: expect a formal agreement, scheduled harvest windows and their HACCP governing the floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="27" t="inlineStr">
         <is>
+          <t>HIGH — over 5,000 hogs/week</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Industrial scale. Volume is never the constraint; ACCESS is. Realistically Model B (they harvest to our spec) or a dedicated biologics / organ program. Worth pursuing where a plant ALREADY runs organ or tissue harvesting — that existing programme, not the head count, is the reason to be there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
           <t>unknown (confirm)</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>Weekly hog throughput is not published for most small/custom plants. Tier to be set on the qualifying call — ask 'how many hogs did you kill LAST WEEK?', not capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>NOTE — boundary</t>
-        </is>
-      </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>The tiers as specified leave 301-349/wk between Small and Medium; anything landing there is treated as the Small/Medium boundary and should be judged on its other merits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+          <t>Weekly hog throughput is not published for most small and custom plants. Set the tier on the qualifying call — ask 'how many hogs did you kill LAST WEEK?', not capacity, and not head across all species.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>NOTE — boundaries</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>301-349/wk sits between Small and Medium, and 2,500/wk is the Medium / Medium-High hinge. Anything landing on a boundary is judged on its other merits (welfare, certification, organ capability, model fit) rather than forced into a band.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>CERTIFICATION COLUMN CODES</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>USDA ✓</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>Federally inspected (FSIS) slaughter — grant of inspection.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>State ✓</t>
+          <t>USDA ✓</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>State meat-inspection program (equal-to FSIS for intrastate sale).</t>
+          <t>Federally inspected (FSIS) slaughter — grant of inspection.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Custom-exempt</t>
+          <t>State ✓</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Custom/exempt plant — NOT continuously inspected; product not for general commerce. FLAG for our use.</t>
+          <t>State meat-inspection program (equal-to FSIS for intrastate sale).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>APHIS ✓ / n/a</t>
+          <t>Custom-exempt</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>APHIS certification relates to animal-health/export programs; note where relevant. 'n/a' = not the applicable regime for this plant.</t>
+          <t>Custom/exempt plant — NOT continuously inspected; product not for general commerce. FLAG for our use.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
         <is>
+          <t>APHIS ✓ / n/a</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>APHIS certification relates to animal-health/export programs; note where relevant. 'n/a' = not the applicable regime for this plant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Not published / not confirmed — MUST verify by phone.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>HOW 'FIT' IS JUDGED  (weighting, not a hard formula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>Hog slaughter present</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>Hard gate — no hogs, out of scope.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>Weekly volume</t>
+          <t>Hog slaughter present</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>NOT a gate — capacity is open. Recorded as a TIER (Small / Medium / High) that shapes the operating model and whether aggregation is needed.</t>
+          <t>Hard gate — no hogs, out of scope.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>USDA / APHIS status</t>
+          <t>Weekly volume</t>
         </is>
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>Preferred; a gap is flagged, not always fatal (depends on our use + Model).</t>
+          <t>NOT a gate — capacity is open. Recorded as a TIER (Small / Medium / High) that shapes the operating model and whether aggregation is needed.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>Welfare &amp; culture</t>
+          <t>USDA / APHIS status</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Strong tie-breaker — the Nahunta differentiator.</t>
+          <t>Preferred; a gap is flagged, not always fatal (depends on our use + Model).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>Model A or B feasible</t>
+          <t>Welfare &amp; culture</t>
         </is>
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>At least one operating model must be plausible.</t>
+          <t>Strong tie-breaker — the Nahunta differentiator.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
+          <t>Model A or B feasible</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>At least one operating model must be plausible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
           <t>Organ/tissue capability</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>Bonus; especially valuable for pelvic/bariatric/thoracic blocks.</t>
         </is>
@@ -5298,10 +5327,10 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5467,7 +5496,7 @@
           <t>~400-500 (est.)</t>
         </is>
       </c>
-      <c r="E6" s="28" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>MEDIUM
 (350-2,500/wk)</t>
@@ -5520,7 +5549,7 @@
 nahuntapork.com</t>
         </is>
       </c>
-      <c r="O6" s="29" t="inlineStr">
+      <c r="O6" s="30" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
@@ -5557,7 +5586,7 @@
           <t>unknown — 'has volume' (est. mid-size)</t>
         </is>
       </c>
-      <c r="E7" s="28" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>MEDIUM
 (350-2,500/wk)</t>
@@ -5610,7 +5639,7 @@
 beth@martinspork.com · martinspork.com</t>
         </is>
       </c>
-      <c r="O7" s="29" t="inlineStr">
+      <c r="O7" s="30" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
@@ -5654,7 +5683,7 @@
           <t>unknown (5 days/wk)</t>
         </is>
       </c>
-      <c r="E9" s="30" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -5706,7 +5735,7 @@
 piedmontcustommeats.com</t>
         </is>
       </c>
-      <c r="O9" s="28" t="inlineStr">
+      <c r="O9" s="29" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -5743,7 +5772,7 @@
           <t>~400 (80 hogs/day cap)</t>
         </is>
       </c>
-      <c r="E10" s="30" t="inlineStr">
+      <c r="E10" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -5796,7 +5825,7 @@
 acrestationmeatfarm.com</t>
         </is>
       </c>
-      <c r="O10" s="31" t="inlineStr">
+      <c r="O10" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -5833,7 +5862,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E11" s="32" t="inlineStr">
+      <c r="E11" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -5884,7 +5913,7 @@
           <t>(252) 235-3558</t>
         </is>
       </c>
-      <c r="O11" s="31" t="inlineStr">
+      <c r="O11" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -5921,7 +5950,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E12" s="32" t="inlineStr">
+      <c r="E12" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -5972,7 +6001,7 @@
           <t>(252) 237-2982</t>
         </is>
       </c>
-      <c r="O12" s="31" t="inlineStr">
+      <c r="O12" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -6009,7 +6038,7 @@
           <t>unknown (small)</t>
         </is>
       </c>
-      <c r="E13" s="30" t="inlineStr">
+      <c r="E13" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -6025,7 +6054,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H13" s="33" t="inlineStr">
+      <c r="H13" s="34" t="inlineStr">
         <is>
           <t>⚠ Humane-handling NOS ~Aug 2020 (Est. M21848); PETA-documented pig shot 3× (2024). Recurring.</t>
         </is>
@@ -6061,7 +6090,7 @@
 maysmeats.net</t>
         </is>
       </c>
-      <c r="O13" s="31" t="inlineStr">
+      <c r="O13" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6098,7 +6127,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E14" s="32" t="inlineStr">
+      <c r="E14" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6114,7 +6143,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H14" s="33" t="inlineStr">
+      <c r="H14" s="34" t="inlineStr">
         <is>
           <t>⚠ Slaughter suspension Aug 2021 — egregious (failed goat stun, conscious throat-cut). PETA→DA.</t>
         </is>
@@ -6149,7 +6178,7 @@
           <t>(336) 591-7420</t>
         </is>
       </c>
-      <c r="O14" s="31" t="inlineStr">
+      <c r="O14" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6186,7 +6215,7 @@
           <t>unknown (small)</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -6239,7 +6268,7 @@
 keypackingcompany.com</t>
         </is>
       </c>
-      <c r="O15" s="31" t="inlineStr">
+      <c r="O15" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -6276,7 +6305,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E16" s="32" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6328,7 +6357,7 @@
           <t>(252) 332-2978</t>
         </is>
       </c>
-      <c r="O16" s="31" t="inlineStr">
+      <c r="O16" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -6365,7 +6394,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E17" s="32" t="inlineStr">
+      <c r="E17" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6381,7 +6410,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H17" s="33" t="inlineStr">
+      <c r="H17" s="34" t="inlineStr">
         <is>
           <t>⚠ REPEAT humane-handling suspensions 2009, 2015, 2018 (AWI list; Est. 19511M)</t>
         </is>
@@ -6416,7 +6445,7 @@
           <t>(336) 667-1346</t>
         </is>
       </c>
-      <c r="O17" s="31" t="inlineStr">
+      <c r="O17" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6453,7 +6482,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E18" s="32" t="inlineStr">
+      <c r="E18" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6504,7 +6533,7 @@
           <t>(704) 786-8616</t>
         </is>
       </c>
-      <c r="O18" s="31" t="inlineStr">
+      <c r="O18" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -6541,7 +6570,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E19" s="32" t="inlineStr">
+      <c r="E19" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6557,7 +6586,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="H19" s="33" t="inlineStr">
+      <c r="H19" s="34" t="inlineStr">
         <is>
           <t>⚠ FSIS suspension ~Dec 2025 (Est. M46085; cause unspecified in public snippets)</t>
         </is>
@@ -6592,7 +6621,7 @@
           <t>(336) 949-9696</t>
         </is>
       </c>
-      <c r="O19" s="31" t="inlineStr">
+      <c r="O19" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6629,7 +6658,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E20" s="32" t="inlineStr">
+      <c r="E20" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6680,7 +6709,7 @@
           <t>(828) 245-5544</t>
         </is>
       </c>
-      <c r="O20" s="31" t="inlineStr">
+      <c r="O20" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -6717,7 +6746,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E21" s="32" t="inlineStr">
+      <c r="E21" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -6770,7 +6799,7 @@
 riversidemeatsnc.com</t>
         </is>
       </c>
-      <c r="O21" s="31" t="inlineStr">
+      <c r="O21" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6814,10 +6843,10 @@
           <t>~28,000-32,000 / DAY</t>
         </is>
       </c>
-      <c r="E23" s="34" t="inlineStr">
+      <c r="E23" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -6865,7 +6894,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O23" s="31" t="inlineStr">
+      <c r="O23" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6902,10 +6931,10 @@
           <t>~1,000 sows/DAY (~5-6k/wk)</t>
         </is>
       </c>
-      <c r="E24" s="34" t="inlineStr">
-        <is>
-          <t>HIGH
-(&gt;2,500/wk)</t>
+      <c r="E24" s="36" t="inlineStr">
+        <is>
+          <t>MEDIUM-HIGH
+(2,500-5,000/wk)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -6953,7 +6982,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O24" s="31" t="inlineStr">
+      <c r="O24" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -6997,7 +7026,7 @@
           <t>unknown (small-mid est.)</t>
         </is>
       </c>
-      <c r="E26" s="32" t="inlineStr">
+      <c r="E26" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -7049,7 +7078,7 @@
 caughmans.com</t>
         </is>
       </c>
-      <c r="O26" s="31" t="inlineStr">
+      <c r="O26" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7086,7 +7115,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E27" s="32" t="inlineStr">
+      <c r="E27" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -7138,7 +7167,7 @@
 knockoutbutchery.com</t>
         </is>
       </c>
-      <c r="O27" s="31" t="inlineStr">
+      <c r="O27" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7175,7 +7204,7 @@
           <t>unknown (small)</t>
         </is>
       </c>
-      <c r="E28" s="30" t="inlineStr">
+      <c r="E28" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -7226,7 +7255,7 @@
           <t>864-374-3571</t>
         </is>
       </c>
-      <c r="O28" s="31" t="inlineStr">
+      <c r="O28" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7263,7 +7292,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E29" s="30" t="inlineStr">
+      <c r="E29" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -7315,7 +7344,7 @@
           <t>803-707-1040</t>
         </is>
       </c>
-      <c r="O29" s="31" t="inlineStr">
+      <c r="O29" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -7352,7 +7381,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E30" s="32" t="inlineStr">
+      <c r="E30" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -7369,7 +7398,7 @@
 SUSPENDED 2022</t>
         </is>
       </c>
-      <c r="H30" s="33" t="inlineStr">
+      <c r="H30" s="34" t="inlineStr">
         <is>
           <t>⚠ Humane-handling NOS Feb &amp; Mar 2022 (Est. M47715); PETA sought criminal probe. Also the slaughter suspension.</t>
         </is>
@@ -7404,7 +7433,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O30" s="35" t="inlineStr">
+      <c r="O30" s="37" t="inlineStr">
         <is>
           <t>OUT / FLAG</t>
         </is>
@@ -7448,7 +7477,7 @@
           <t>unknown (largest of TN group est.)</t>
         </is>
       </c>
-      <c r="E32" s="32" t="inlineStr">
+      <c r="E32" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -7464,7 +7493,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H32" s="33" t="inlineStr">
+      <c r="H32" s="34" t="inlineStr">
         <is>
           <t>⚠ Humane-handling NOS Apr 2023 (Est. M6555 — 4 stun attempts on a cow); held in abeyance.</t>
         </is>
@@ -7500,7 +7529,7 @@
 fayettepackingco.com</t>
         </is>
       </c>
-      <c r="O32" s="31" t="inlineStr">
+      <c r="O32" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7537,7 +7566,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E33" s="32" t="inlineStr">
+      <c r="E33" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -7588,7 +7617,7 @@
           <t>931-330-6328</t>
         </is>
       </c>
-      <c r="O33" s="31" t="inlineStr">
+      <c r="O33" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7625,7 +7654,7 @@
           <t>~18/wk (80/month verified)</t>
         </is>
       </c>
-      <c r="E34" s="30" t="inlineStr">
+      <c r="E34" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -7677,7 +7706,7 @@
 cherrymeat.com</t>
         </is>
       </c>
-      <c r="O34" s="31" t="inlineStr">
+      <c r="O34" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7714,7 +7743,7 @@
           <t>unknown (tens–low 100s/wk est.)</t>
         </is>
       </c>
-      <c r="E35" s="30" t="inlineStr">
+      <c r="E35" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -7730,7 +7759,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H35" s="33" t="inlineStr">
+      <c r="H35" s="34" t="inlineStr">
         <is>
           <t>⚠ Harris Country Meats (Greeneville, M20686): humane NOS 2024. Volunteer/412 (Lexington, M6561): humane NOS Nov 2024. Others: none found.</t>
         </is>
@@ -7765,7 +7794,7 @@
           <t>see notes →</t>
         </is>
       </c>
-      <c r="O35" s="31" t="inlineStr">
+      <c r="O35" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -7809,7 +7838,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E37" s="30" t="inlineStr">
+      <c r="E37" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -7861,7 +7890,7 @@
 ecofriendly.com</t>
         </is>
       </c>
-      <c r="O37" s="31" t="inlineStr">
+      <c r="O37" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -7898,7 +7927,7 @@
           <t>unknown (small)</t>
         </is>
       </c>
-      <c r="E38" s="30" t="inlineStr">
+      <c r="E38" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -7950,7 +7979,7 @@
 temeats.com</t>
         </is>
       </c>
-      <c r="O38" s="28" t="inlineStr">
+      <c r="O38" s="29" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -7987,7 +8016,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E39" s="32" t="inlineStr">
+      <c r="E39" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -8039,7 +8068,7 @@
 blueridgemeats.com</t>
         </is>
       </c>
-      <c r="O39" s="28" t="inlineStr">
+      <c r="O39" s="29" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -8076,7 +8105,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E40" s="32" t="inlineStr">
+      <c r="E40" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -8093,7 +8122,7 @@
 slaughter listed)</t>
         </is>
       </c>
-      <c r="H40" s="33" t="inlineStr">
+      <c r="H40" s="34" t="inlineStr">
         <is>
           <t>⚠ REPEAT humane-handling suspensions 2021 &amp; Dec 2024 (+ a 2018 violation). Est. M33940.</t>
         </is>
@@ -8129,7 +8158,7 @@
 finestbutcher.com</t>
         </is>
       </c>
-      <c r="O40" s="31" t="inlineStr">
+      <c r="O40" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -8166,7 +8195,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E41" s="32" t="inlineStr">
+      <c r="E41" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -8182,7 +8211,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H41" s="33" t="inlineStr">
+      <c r="H41" s="34" t="inlineStr">
         <is>
           <t>⚠ Donald's Meat Processing (Lexington, M39968): repeat humane suspension 2023 → 3-yr consent decision. Others: none found.</t>
         </is>
@@ -8217,7 +8246,7 @@
           <t>see notes →</t>
         </is>
       </c>
-      <c r="O41" s="31" t="inlineStr">
+      <c r="O41" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -8254,7 +8283,7 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="E42" s="30" t="inlineStr">
+      <c r="E42" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -8306,7 +8335,7 @@
           <t>see notes →</t>
         </is>
       </c>
-      <c r="O42" s="31" t="inlineStr">
+      <c r="O42" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -8350,7 +8379,7 @@
           <t>~385 (20k/yr)</t>
         </is>
       </c>
-      <c r="E44" s="28" t="inlineStr">
+      <c r="E44" s="29" t="inlineStr">
         <is>
           <t>MEDIUM
 (350-2,500/wk)</t>
@@ -8403,7 +8432,7 @@
 (phone via site)</t>
         </is>
       </c>
-      <c r="O44" s="28" t="inlineStr">
+      <c r="O44" s="29" t="inlineStr">
         <is>
           <t>STRONG FIT</t>
         </is>
@@ -8442,10 +8471,10 @@
 (organ exception)</t>
         </is>
       </c>
-      <c r="E45" s="34" t="inlineStr">
+      <c r="E45" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -8459,7 +8488,7 @@
 export-cert</t>
         </is>
       </c>
-      <c r="H45" s="33" t="inlineStr">
+      <c r="H45" s="34" t="inlineStr">
         <is>
           <t>⚠ REPEAT humane-handling: NOIE 2021 &amp; 2023; suspension 09/2024 (egregious). ASPCA line-speed concerns. Est. M717.</t>
         </is>
@@ -8494,7 +8523,7 @@
           <t>smithfieldbioscience.com</t>
         </is>
       </c>
-      <c r="O45" s="28" t="inlineStr">
+      <c r="O45" s="29" t="inlineStr">
         <is>
           <t>STRONG FIT
 (organ exc.)</t>
@@ -8539,7 +8568,7 @@
           <t>up to ~600 (120/day est.)</t>
         </is>
       </c>
-      <c r="E47" s="28" t="inlineStr">
+      <c r="E47" s="29" t="inlineStr">
         <is>
           <t>MEDIUM
 (350-2,500/wk)</t>
@@ -8591,7 +8620,7 @@
 lorentzmeats.com</t>
         </is>
       </c>
-      <c r="O47" s="31" t="inlineStr">
+      <c r="O47" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -8628,7 +8657,7 @@
           <t>unknown (small-mid)</t>
         </is>
       </c>
-      <c r="E48" s="32" t="inlineStr">
+      <c r="E48" s="33" t="inlineStr">
         <is>
           <t>unknown
 (confirm)</t>
@@ -8681,7 +8710,7 @@
 sigiowa.com</t>
         </is>
       </c>
-      <c r="O48" s="31" t="inlineStr">
+      <c r="O48" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -8718,7 +8747,7 @@
           <t>small (low-100s/wk est.)</t>
         </is>
       </c>
-      <c r="E49" s="30" t="inlineStr">
+      <c r="E49" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -8770,7 +8799,7 @@
 eickmans.com</t>
         </is>
       </c>
-      <c r="O49" s="31" t="inlineStr">
+      <c r="O49" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -8807,7 +8836,7 @@
           <t>low (very small)</t>
         </is>
       </c>
-      <c r="E50" s="30" t="inlineStr">
+      <c r="E50" s="31" t="inlineStr">
         <is>
           <t>SMALL
 (0-300/wk)</t>
@@ -8859,7 +8888,7 @@
           <t>(712) 837-5334</t>
         </is>
       </c>
-      <c r="O50" s="31" t="inlineStr">
+      <c r="O50" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -8903,10 +8932,10 @@
           <t>~4,500 / DAY</t>
         </is>
       </c>
-      <c r="E52" s="34" t="inlineStr">
+      <c r="E52" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -8920,7 +8949,7 @@
 organic</t>
         </is>
       </c>
-      <c r="H52" s="33" t="inlineStr">
+      <c r="H52" s="34" t="inlineStr">
         <is>
           <t>⚠ Humane-handling: NOIE 11/2020, suspension 04/2021 (Est. M5537); PETA sought charges (none filed on record).</t>
         </is>
@@ -8955,7 +8984,7 @@
           <t>(712) 722-2555</t>
         </is>
       </c>
-      <c r="O52" s="31" t="inlineStr">
+      <c r="O52" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -8992,10 +9021,10 @@
           <t>~10,000/DAY (up to 20-24k)</t>
         </is>
       </c>
-      <c r="E53" s="34" t="inlineStr">
+      <c r="E53" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -9043,7 +9072,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O53" s="31" t="inlineStr">
+      <c r="O53" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -9080,10 +9109,10 @@
           <t>~10,000-12,000/DAY</t>
         </is>
       </c>
-      <c r="E54" s="34" t="inlineStr">
+      <c r="E54" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -9096,7 +9125,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H54" s="33" t="inlineStr">
+      <c r="H54" s="34" t="inlineStr">
         <is>
           <t>⚠ REPEAT humane-handling suspensions 2020 &amp; 04/2022 (egregious). Est. M51340. PETA sought kill-floor cameras.</t>
         </is>
@@ -9131,7 +9160,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O54" s="31" t="inlineStr">
+      <c r="O54" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -9168,10 +9197,10 @@
           <t>~8,200/DAY (3M→5.6M/yr)</t>
         </is>
       </c>
-      <c r="E55" s="34" t="inlineStr">
+      <c r="E55" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -9184,7 +9213,7 @@
           <t>USDA ✓</t>
         </is>
       </c>
-      <c r="H55" s="33" t="inlineStr">
+      <c r="H55" s="34" t="inlineStr">
         <is>
           <t>⚠ Humane-handling NOIE 12/2019 (Est. M46491; captive bolt on a condemned hog).</t>
         </is>
@@ -9219,7 +9248,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O55" s="31" t="inlineStr">
+      <c r="O55" s="32" t="inlineStr">
         <is>
           <t>POSSIBLE</t>
         </is>
@@ -9256,10 +9285,10 @@
           <t>&gt;3,000/wk</t>
         </is>
       </c>
-      <c r="E56" s="34" t="inlineStr">
+      <c r="E56" s="35" t="inlineStr">
         <is>
           <t>HIGH
-(&gt;2,500/wk)</t>
+(&gt;5,000/wk)</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -9307,7 +9336,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O56" s="31" t="inlineStr">
+      <c r="O56" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -9351,7 +9380,7 @@
           <t>n/a (research minipigs)</t>
         </is>
       </c>
-      <c r="E58" s="32" t="inlineStr">
+      <c r="E58" s="33" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -9401,7 +9430,7 @@
           <t>sinclairbioresources.com</t>
         </is>
       </c>
-      <c r="O58" s="31" t="inlineStr">
+      <c r="O58" s="32" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
@@ -9560,7 +9589,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I5" s="36" t="inlineStr">
+      <c r="I5" s="38" t="inlineStr">
         <is>
           <t>RISKY — USDA-abattoir sourced but no ISO/APHIS/TRACES or export docs; must ask</t>
         </is>
@@ -9607,7 +9636,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I6" s="36" t="inlineStr">
+      <c r="I6" s="38" t="inlineStr">
         <is>
           <t>RISKY — USDA-inspected sourcing + Class B, but no ISO/APHIS/export docs published</t>
         </is>
@@ -9655,7 +9684,7 @@
 (prices)</t>
         </is>
       </c>
-      <c r="I7" s="37" t="inlineStr">
+      <c r="I7" s="39" t="inlineStr">
         <is>
           <t>LIKELY BLOCKER (device) — 'research use only, not for human/animal use' RUO labeling; no export docs</t>
         </is>
@@ -9702,7 +9731,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I8" s="38" t="inlineStr">
+      <c r="I8" s="40" t="inlineStr">
         <is>
           <t>OK (best) — ISO 13485 + 22442-2, USDA Class A, animal traceability; confirm establishment APHIS/TRACES listing</t>
         </is>
@@ -9749,7 +9778,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I9" s="38" t="inlineStr">
+      <c r="I9" s="40" t="inlineStr">
         <is>
           <t>OK (strong) — ISO 22442-2, USDA/SQF, PQA+ farms, full traceability; confirm ISO 13485 + TRACES</t>
         </is>
@@ -9796,7 +9825,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I10" s="38" t="inlineStr">
+      <c r="I10" s="40" t="inlineStr">
         <is>
           <t>OK (best) — vertically integrated, already exports heparin to EP; confirm they supply tissue blocks + VS certs</t>
         </is>
@@ -9843,7 +9872,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I11" s="36" t="inlineStr">
+      <c r="I11" s="38" t="inlineStr">
         <is>
           <t>RISKY — device-supply track record but multi-source broker; must document APHIS/TRACES</t>
         </is>
@@ -9890,7 +9919,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I12" s="36" t="inlineStr">
+      <c r="I12" s="38" t="inlineStr">
         <is>
           <t>RISKY — 'worldwide' supply but no ISO/APHIS/TRACES published; must ask</t>
         </is>
@@ -9938,7 +9967,7 @@
 (thyroid)</t>
         </is>
       </c>
-      <c r="I13" s="36" t="inlineStr">
+      <c r="I13" s="38" t="inlineStr">
         <is>
           <t>RISKY (porcine unverified) — documented USDA on-site inspection is for RABBIT; confirm porcine origin</t>
         </is>
@@ -9985,7 +10014,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I14" s="36" t="inlineStr">
+      <c r="I14" s="38" t="inlineStr">
         <is>
           <t>RISKY — US USDA sourcing but 'research/diagnostic/mfg only'; no export docs</t>
         </is>
@@ -10032,7 +10061,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I15" s="37" t="inlineStr">
+      <c r="I15" s="39" t="inlineStr">
         <is>
           <t>LIKELY BLOCKER / unknown — no published human-food-chain/APHIS basis; RUO-oriented</t>
         </is>
@@ -10079,7 +10108,7 @@
           <t>Med-High</t>
         </is>
       </c>
-      <c r="I16" s="36" t="inlineStr">
+      <c r="I16" s="38" t="inlineStr">
         <is>
           <t>RISKY — device customers worldwide but no published traceability/cert framework</t>
         </is>
@@ -10126,7 +10155,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I17" s="38" t="inlineStr">
+      <c r="I17" s="40" t="inlineStr">
         <is>
           <t>OK (strong) — ISO 13485 + 22442-2, USDA Class B/R, own harvest, ships internationally; confirm TRACES listing</t>
         </is>
@@ -10173,7 +10202,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I18" s="39" t="inlineStr">
+      <c r="I18" s="41" t="inlineStr">
         <is>
           <t>n/a — live animals, out of scope</t>
         </is>
@@ -10220,7 +10249,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I19" s="39" t="inlineStr">
+      <c r="I19" s="41" t="inlineStr">
         <is>
           <t>n/a — human tissue, out of scope</t>
         </is>
@@ -10267,7 +10296,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I20" s="39" t="inlineStr">
+      <c r="I20" s="41" t="inlineStr">
         <is>
           <t>n/a — rodent, out of scope</t>
         </is>
@@ -10312,13 +10341,13 @@
           <t>Smithfield BioScience · Tissue Source · Midwest Research Swine · SSR — device/pharma-grade, traceable, human-food-chain, not RUO-blocked. All still need ONE thing in writing: the slaughter establishment is APHIS-approved &amp; TRACES-listed and the vendor will furnish a VS-endorsed health certificate per consignment (none advertise TRACES listing).</t>
         </is>
       </c>
-      <c r="C27" s="63" t="n"/>
-      <c r="D27" s="63" t="n"/>
-      <c r="E27" s="63" t="n"/>
-      <c r="F27" s="63" t="n"/>
-      <c r="G27" s="63" t="n"/>
-      <c r="H27" s="63" t="n"/>
-      <c r="I27" s="62" t="n"/>
+      <c r="C27" s="65" t="n"/>
+      <c r="D27" s="65" t="n"/>
+      <c r="E27" s="65" t="n"/>
+      <c r="F27" s="65" t="n"/>
+      <c r="G27" s="65" t="n"/>
+      <c r="H27" s="65" t="n"/>
+      <c r="I27" s="64" t="n"/>
     </row>
     <row r="28" ht="34" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
@@ -10331,13 +10360,13 @@
           <t>ABI · WG Biomedical · LAMPIRE · Sierra · Animal Technologies — USDA-abattoir sourcing + device customers, but no published ISO/APHIS/TRACES/cert framework. Multi-source brokers (WG, Sierra, LAMPIRE) make single-establishment TRACES harder.</t>
         </is>
       </c>
-      <c r="C28" s="63" t="n"/>
-      <c r="D28" s="63" t="n"/>
-      <c r="E28" s="63" t="n"/>
-      <c r="F28" s="63" t="n"/>
-      <c r="G28" s="63" t="n"/>
-      <c r="H28" s="63" t="n"/>
-      <c r="I28" s="62" t="n"/>
+      <c r="C28" s="65" t="n"/>
+      <c r="D28" s="65" t="n"/>
+      <c r="E28" s="65" t="n"/>
+      <c r="F28" s="65" t="n"/>
+      <c r="G28" s="65" t="n"/>
+      <c r="H28" s="65" t="n"/>
+      <c r="I28" s="64" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
@@ -10350,13 +10379,13 @@
           <t>Innovative Research &amp; BioChemed (explicit RUO / 'not for human or animal use') · BioIVT (no published human-food-chain/APHIS basis) · Pel-Freez for porcine (their documented USDA on-site inspection is for rabbit). RUO labeling signals no export-doc support and conflicts with MDR Annex I 13.1 / ISO 22442.</t>
         </is>
       </c>
-      <c r="C29" s="63" t="n"/>
-      <c r="D29" s="63" t="n"/>
-      <c r="E29" s="63" t="n"/>
-      <c r="F29" s="63" t="n"/>
-      <c r="G29" s="63" t="n"/>
-      <c r="H29" s="63" t="n"/>
-      <c r="I29" s="62" t="n"/>
+      <c r="C29" s="65" t="n"/>
+      <c r="D29" s="65" t="n"/>
+      <c r="E29" s="65" t="n"/>
+      <c r="F29" s="65" t="n"/>
+      <c r="G29" s="65" t="n"/>
+      <c r="H29" s="65" t="n"/>
+      <c r="I29" s="64" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:I4"/>
@@ -10615,9 +10644,9 @@
           <t>•  Bottom line: for an operation that already harvests on-site, buying finished tissue from a national vendor is generally MORE expensive per tissue than self-harvest — but buying-direct wins in specific situations, not on unit cost.</t>
         </is>
       </c>
-      <c r="B15" s="63" t="n"/>
-      <c r="C15" s="63" t="n"/>
-      <c r="D15" s="62" t="n"/>
+      <c r="B15" s="65" t="n"/>
+      <c r="C15" s="65" t="n"/>
+      <c r="D15" s="64" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -10625,9 +10654,9 @@
           <t>•  One hog yields all three regions at once: self-harvest pulls pelvic + abdominal + thoracic from the same carcass in one session. Buying the equivalent separately (pelvic block ~$582 + a thoracic pluck + abdominal organs ~$141 each) stacks to roughly $1,000-2,000+ per animal-equivalent before shipping. Your marginal cost at the plant is mostly labor + consumables.</t>
         </is>
       </c>
-      <c r="B16" s="63" t="n"/>
-      <c r="C16" s="63" t="n"/>
-      <c r="D16" s="62" t="n"/>
+      <c r="B16" s="65" t="n"/>
+      <c r="C16" s="65" t="n"/>
+      <c r="D16" s="64" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -10635,9 +10664,9 @@
           <t>•  Custom dissection / processing fees: vendors charge for anything beyond base config (extra vessels, cannulation, specific trim, saline/PBS perfusion) — exactly the work you already do in-house.</t>
         </is>
       </c>
-      <c r="B17" s="63" t="n"/>
-      <c r="C17" s="63" t="n"/>
-      <c r="D17" s="62" t="n"/>
+      <c r="B17" s="65" t="n"/>
+      <c r="C17" s="65" t="n"/>
+      <c r="D17" s="64" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -10645,9 +10674,9 @@
           <t>•  Freshness / warm-ischemia: self-harvest is unbeatable (minutes). Vendors mitigate with overnight fresh-on-ice, but you still lose hours-to-a-day and pay cold-chain/dry-ice freight.</t>
         </is>
       </c>
-      <c r="B18" s="63" t="n"/>
-      <c r="C18" s="63" t="n"/>
-      <c r="D18" s="62" t="n"/>
+      <c r="B18" s="65" t="n"/>
+      <c r="C18" s="65" t="n"/>
+      <c r="D18" s="64" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -10655,9 +10684,9 @@
           <t>•  Minimums, lead times, shipping: published lead times run up to 2-4 weeks (Pel-Freez); custom collections longer.</t>
         </is>
       </c>
-      <c r="B19" s="63" t="n"/>
-      <c r="C19" s="63" t="n"/>
-      <c r="D19" s="62" t="n"/>
+      <c r="B19" s="65" t="n"/>
+      <c r="C19" s="65" t="n"/>
+      <c r="D19" s="64" t="n"/>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -10665,9 +10694,9 @@
           <t>•  Buy-direct is the better call despite higher unit cost when: volume is low/irregular; you lack USDA-inspected abattoir access or the QMS to document it and need traceability/certs (e.g. Tissue Source ISO 13485 + USDA Class A; ABI USDA-inspected); you need occasional organs outside your normal line, or specialized prep (perfused, snap-frozen, lyophilized — LAMPIRE).</t>
         </is>
       </c>
-      <c r="B20" s="63" t="n"/>
-      <c r="C20" s="63" t="n"/>
-      <c r="D20" s="62" t="n"/>
+      <c r="B20" s="65" t="n"/>
+      <c r="C20" s="65" t="n"/>
+      <c r="D20" s="64" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -10675,9 +10704,9 @@
           <t>•  Public price anchors to reason from: ~$141 per single porcine organ and ~$582 for a full regional (pelvic) block (Innovative Research, list). Exact self-harvest break-even depends on hog cost, labor rate, tissues-per-animal yield, and shipping — none public — so treat this as directional until real quotes are in hand.</t>
         </is>
       </c>
-      <c r="B21" s="63" t="n"/>
-      <c r="C21" s="63" t="n"/>
-      <c r="D21" s="62" t="n"/>
+      <c r="B21" s="65" t="n"/>
+      <c r="C21" s="65" t="n"/>
+      <c r="D21" s="64" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -10734,437 +10763,437 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="40" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Legend:  blue cells on pale-yellow = you edit  ·  black = calculated  ·  ★ = the answer.  Values shown are ILLUSTRATIVE placeholders — swap in your real numbers/quotes.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="41" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
         <is>
           <t>A.  HARVEST SESSION  (per visit)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="42" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>Blocks / organs harvested per visit</t>
         </is>
       </c>
-      <c r="C6" s="43" t="n">
+      <c r="C6" s="45" t="n">
         <v>40</v>
       </c>
-      <c r="D6" s="44" t="inlineStr">
+      <c r="D6" s="46" t="inlineStr">
         <is>
           <t>How many pieces you collect in one trip.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="44" t="inlineStr">
         <is>
           <t>Harvest time per block (minutes)</t>
         </is>
       </c>
-      <c r="C7" s="45" t="n">
+      <c r="C7" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="D7" s="44" t="inlineStr">
+      <c r="D7" s="46" t="inlineStr">
         <is>
           <t>Hands-on time to harvest one block/organ.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>Harvesters on site (#)</t>
         </is>
       </c>
-      <c r="C8" s="43" t="n">
+      <c r="C8" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="44" t="inlineStr">
+      <c r="D8" s="46" t="inlineStr">
         <is>
           <t>Your crew size. For Model B (plant harvests) set 0.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="42" t="inlineStr">
+      <c r="A9" s="44" t="inlineStr">
         <is>
           <t>Harvester labor rate ($/hr, loaded)</t>
         </is>
       </c>
-      <c r="C9" s="46" t="n">
+      <c r="C9" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="D9" s="44" t="inlineStr">
+      <c r="D9" s="46" t="inlineStr">
         <is>
           <t>Fully-loaded wage incl. burden.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>Session hours (wall-clock)</t>
         </is>
       </c>
-      <c r="C10" s="47">
+      <c r="C10" s="49">
         <f>C6*C7/60</f>
         <v/>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="46">
         <f> blocks × min/block ÷ 60.</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="42" t="inlineStr">
+      <c r="A11" s="44" t="inlineStr">
         <is>
           <t>Harvester labor per visit</t>
         </is>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="50">
         <f>C10*C8*C9</f>
         <v/>
       </c>
-      <c r="D11" s="44">
+      <c r="D11" s="46">
         <f> session hours × crew × rate.</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
+      <c r="A12" s="43" t="inlineStr">
         <is>
           <t>B.  FACILITY ACCESS  (per visit — varies by slaughterhouse)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="42" t="inlineStr">
+      <c r="A13" s="44" t="inlineStr">
         <is>
           <t>Space / line rental per visit ($)</t>
         </is>
       </c>
-      <c r="C13" s="46" t="n">
+      <c r="C13" s="48" t="n">
         <v>500</v>
       </c>
-      <c r="D13" s="44" t="inlineStr">
+      <c r="D13" s="46" t="inlineStr">
         <is>
           <t>Model A: rent floor/cooler access. 0 if none / relationship.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>Plant inspection / handling fee per visit ($)</t>
         </is>
       </c>
-      <c r="C14" s="46" t="n">
+      <c r="C14" s="48" t="n">
         <v>150</v>
       </c>
-      <c r="D14" s="44" t="inlineStr">
+      <c r="D14" s="46" t="inlineStr">
         <is>
           <t>Plant's charge for their staff/line time — OR the Model B per-visit harvest fee.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="42" t="inlineStr">
+      <c r="A15" s="44" t="inlineStr">
         <is>
           <t>Our inspector / trainer cost per visit ($)</t>
         </is>
       </c>
-      <c r="C15" s="46" t="n">
+      <c r="C15" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="44" t="inlineStr">
+      <c r="D15" s="46" t="inlineStr">
         <is>
           <t>Model B: amortized day-rate + travel of trainers/inspectors we send.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="42" t="inlineStr">
+      <c r="A16" s="44" t="inlineStr">
         <is>
           <t>Facility fixed subtotal</t>
         </is>
       </c>
-      <c r="C16" s="48">
+      <c r="C16" s="50">
         <f>C13+C14+C15</f>
         <v/>
       </c>
-      <c r="D16" s="44">
+      <c r="D16" s="46">
         <f> rental + plant fee + our inspector.</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="41" t="inlineStr">
+      <c r="A17" s="43" t="inlineStr">
         <is>
           <t>C.  LOGISTICS &amp; HOLDING</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="42" t="inlineStr">
+      <c r="A18" s="44" t="inlineStr">
         <is>
           <t>Transportation per visit ($)</t>
         </is>
       </c>
-      <c r="C18" s="46" t="n">
+      <c r="C18" s="48" t="n">
         <v>300</v>
       </c>
-      <c r="D18" s="44" t="inlineStr">
+      <c r="D18" s="46" t="inlineStr">
         <is>
           <t>Round-trip freight / vehicle / fuel / cold-chain for the trip.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="42" t="inlineStr">
+      <c r="A19" s="44" t="inlineStr">
         <is>
           <t>Inventory / holding cost per block ($)</t>
         </is>
       </c>
-      <c r="C19" s="46" t="n">
+      <c r="C19" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="44" t="inlineStr">
+      <c r="D19" s="46" t="inlineStr">
         <is>
           <t>Preservation, cold storage, holding per piece.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="41" t="inlineStr">
+      <c r="A20" s="43" t="inlineStr">
         <is>
           <t>D.  RESULT</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="42" t="inlineStr">
+      <c r="A21" s="44" t="inlineStr">
         <is>
           <t>Per-visit fixed + transport</t>
         </is>
       </c>
-      <c r="C21" s="48">
+      <c r="C21" s="50">
         <f>C16+C18</f>
         <v/>
       </c>
-      <c r="D21" s="44">
+      <c r="D21" s="46">
         <f> facility fixed + transportation.</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="42" t="inlineStr">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>Total cost per visit</t>
         </is>
       </c>
-      <c r="C22" s="48">
+      <c r="C22" s="50">
         <f>C21+C11+C19*C6</f>
         <v/>
       </c>
-      <c r="D22" s="44">
+      <c r="D22" s="46">
         <f> fixed+transport + harvester labor + inventory × blocks.</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="49" t="inlineStr">
+      <c r="A23" s="51" t="inlineStr">
         <is>
           <t>★ TOTAL COST PER BLOCK</t>
         </is>
       </c>
-      <c r="C23" s="50">
+      <c r="C23" s="52">
         <f>IF(C6&gt;0,C22/C6,0)</f>
         <v/>
       </c>
-      <c r="D23" s="44">
+      <c r="D23" s="46">
         <f> total cost per visit ÷ blocks. Your self-harvest unit cost.</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="A24" s="44" t="inlineStr">
         <is>
           <t>Memo: harvester labor per block</t>
         </is>
       </c>
-      <c r="C24" s="48">
+      <c r="C24" s="50">
         <f>IF(C6&gt;0,C11/C6,0)</f>
         <v/>
       </c>
-      <c r="D24" s="44">
+      <c r="D24" s="46">
         <f> (min/block ÷ 60) × crew × rate.</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="42" t="inlineStr">
+      <c r="A25" s="44" t="inlineStr">
         <is>
           <t>Memo: fixed+transport per block</t>
         </is>
       </c>
-      <c r="C25" s="48">
+      <c r="C25" s="50">
         <f>IF(C6&gt;0,C21/C6,0)</f>
         <v/>
       </c>
-      <c r="D25" s="44" t="inlineStr">
+      <c r="D25" s="46" t="inlineStr">
         <is>
           <t>Spread of per-visit fixed costs — falls as blocks/visit rises.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="41" t="inlineStr">
+      <c r="A26" s="43" t="inlineStr">
         <is>
           <t>E.  BUY-DIRECT BENCHMARK  (real published list prices)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="42" t="inlineStr">
+      <c r="A27" s="44" t="inlineStr">
         <is>
           <t>Buy-direct: single porcine organ ($)</t>
         </is>
       </c>
-      <c r="C27" s="46" t="n">
+      <c r="C27" s="48" t="n">
         <v>141</v>
       </c>
-      <c r="D27" s="44" t="inlineStr">
+      <c r="D27" s="46" t="inlineStr">
         <is>
           <t>Innovative Research list, base config (real published price).</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="42" t="inlineStr">
+      <c r="A28" s="44" t="inlineStr">
         <is>
           <t>Buy-direct: pelvic block ($)</t>
         </is>
       </c>
-      <c r="C28" s="46" t="n">
+      <c r="C28" s="48" t="n">
         <v>582</v>
       </c>
-      <c r="D28" s="44" t="inlineStr">
+      <c r="D28" s="46" t="inlineStr">
         <is>
           <t>Innovative Research list, base config (real published price).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="42" t="inlineStr">
+      <c r="A29" s="44" t="inlineStr">
         <is>
           <t>Δ self-harvest vs buy-direct (per organ)</t>
         </is>
       </c>
-      <c r="C29" s="48">
+      <c r="C29" s="50">
         <f>C23-C27</f>
         <v/>
       </c>
-      <c r="D29" s="44" t="inlineStr">
+      <c r="D29" s="46" t="inlineStr">
         <is>
           <t>Negative = self-harvest cheaper per organ.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="42" t="inlineStr">
+      <c r="A30" s="44" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C30" s="51">
+      <c r="C30" s="53">
         <f>IF(C23&lt;=C27,"Self-harvest cheaper / on par","Buying direct cheaper per organ")</f>
         <v/>
       </c>
-      <c r="D30" s="44" t="inlineStr">
+      <c r="D30" s="46" t="inlineStr">
         <is>
           <t>Rule of thumb; one visit yields many blocks, favoring self-harvest.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="41" t="inlineStr">
+      <c r="A32" s="43" t="inlineStr">
         <is>
           <t>PER-SLAUGHTERHOUSE COMPARISON  (illustrative placeholders — replace with real figures/quotes)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="52" t="inlineStr">
+      <c r="A33" s="54" t="inlineStr">
         <is>
           <t>Facility</t>
         </is>
       </c>
-      <c r="B33" s="52" t="inlineStr">
+      <c r="B33" s="54" t="inlineStr">
         <is>
           <t>Blocks/
 visit</t>
         </is>
       </c>
-      <c r="C33" s="52" t="inlineStr">
+      <c r="C33" s="54" t="inlineStr">
         <is>
           <t>Min/
 block</t>
         </is>
       </c>
-      <c r="D33" s="52" t="inlineStr">
+      <c r="D33" s="54" t="inlineStr">
         <is>
           <t>Crew</t>
         </is>
       </c>
-      <c r="E33" s="52" t="inlineStr">
+      <c r="E33" s="54" t="inlineStr">
         <is>
           <t>$/hr</t>
         </is>
       </c>
-      <c r="F33" s="52" t="inlineStr">
+      <c r="F33" s="54" t="inlineStr">
         <is>
           <t>Rental/
 visit</t>
         </is>
       </c>
-      <c r="G33" s="52" t="inlineStr">
+      <c r="G33" s="54" t="inlineStr">
         <is>
           <t>Plant fee /
 harvest fee</t>
         </is>
       </c>
-      <c r="H33" s="52" t="inlineStr">
+      <c r="H33" s="54" t="inlineStr">
         <is>
           <t>Our insp/
 visit</t>
         </is>
       </c>
-      <c r="I33" s="52" t="inlineStr">
+      <c r="I33" s="54" t="inlineStr">
         <is>
           <t>Transport/
 visit</t>
         </is>
       </c>
-      <c r="J33" s="52" t="inlineStr">
+      <c r="J33" s="54" t="inlineStr">
         <is>
           <t>Inv/
 block</t>
         </is>
       </c>
-      <c r="K33" s="52" t="inlineStr">
+      <c r="K33" s="54" t="inlineStr">
         <is>
           <t>⇒ Cost/
 block</t>
         </is>
       </c>
-      <c r="L33" s="52" t="inlineStr">
+      <c r="L33" s="54" t="inlineStr">
         <is>
           <t>vs $/organ
 direct</t>
@@ -11177,38 +11206,38 @@
           <t>Nahunta Pork Center (Pikeville, NC)</t>
         </is>
       </c>
-      <c r="B34" s="43" t="n">
+      <c r="B34" s="45" t="n">
         <v>40</v>
       </c>
-      <c r="C34" s="45" t="n">
+      <c r="C34" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="D34" s="43" t="n">
+      <c r="D34" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="46" t="n">
+      <c r="E34" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F34" s="46" t="n">
+      <c r="F34" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="46" t="n">
+      <c r="G34" s="48" t="n">
         <v>100</v>
       </c>
-      <c r="H34" s="46" t="n">
+      <c r="H34" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="46" t="n">
+      <c r="I34" s="48" t="n">
         <v>150</v>
       </c>
-      <c r="J34" s="46" t="n">
+      <c r="J34" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="K34" s="53">
+      <c r="K34" s="55">
         <f>IF(B34&gt;0,(F34+G34+H34+I34+(B34*C34/60)*D34*E34+J34*B34)/B34,0)</f>
         <v/>
       </c>
-      <c r="L34" s="48">
+      <c r="L34" s="50">
         <f>K34-$C$27</f>
         <v/>
       </c>
@@ -11219,38 +11248,38 @@
           <t>Martin's Pork Products (Falcon, NC)</t>
         </is>
       </c>
-      <c r="B35" s="43" t="n">
+      <c r="B35" s="45" t="n">
         <v>50</v>
       </c>
-      <c r="C35" s="45" t="n">
+      <c r="C35" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="D35" s="43" t="n">
+      <c r="D35" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="46" t="n">
+      <c r="E35" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F35" s="46" t="n">
+      <c r="F35" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="G35" s="46" t="n">
+      <c r="G35" s="48" t="n">
         <v>150</v>
       </c>
-      <c r="H35" s="46" t="n">
+      <c r="H35" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="46" t="n">
+      <c r="I35" s="48" t="n">
         <v>175</v>
       </c>
-      <c r="J35" s="46" t="n">
+      <c r="J35" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="K35" s="53">
+      <c r="K35" s="55">
         <f>IF(B35&gt;0,(F35+G35+H35+I35+(B35*C35/60)*D35*E35+J35*B35)/B35,0)</f>
         <v/>
       </c>
-      <c r="L35" s="48">
+      <c r="L35" s="50">
         <f>K35-$C$27</f>
         <v/>
       </c>
@@ -11261,38 +11290,38 @@
           <t>Piedmont Custom Meats (NC)</t>
         </is>
       </c>
-      <c r="B36" s="43" t="n">
+      <c r="B36" s="45" t="n">
         <v>45</v>
       </c>
-      <c r="C36" s="45" t="n">
+      <c r="C36" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="D36" s="43" t="n">
+      <c r="D36" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="46" t="n">
+      <c r="E36" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F36" s="46" t="n">
+      <c r="F36" s="48" t="n">
         <v>400</v>
       </c>
-      <c r="G36" s="46" t="n">
+      <c r="G36" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="46" t="n">
+      <c r="H36" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="I36" s="46" t="n">
+      <c r="I36" s="48" t="n">
         <v>200</v>
       </c>
-      <c r="J36" s="46" t="n">
+      <c r="J36" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="K36" s="53">
+      <c r="K36" s="55">
         <f>IF(B36&gt;0,(F36+G36+H36+I36+(B36*C36/60)*D36*E36+J36*B36)/B36,0)</f>
         <v/>
       </c>
-      <c r="L36" s="48">
+      <c r="L36" s="50">
         <f>K36-$C$27</f>
         <v/>
       </c>
@@ -11303,38 +11332,38 @@
           <t>Acre Station Meat Farm (NC)</t>
         </is>
       </c>
-      <c r="B37" s="43" t="n">
+      <c r="B37" s="45" t="n">
         <v>30</v>
       </c>
-      <c r="C37" s="45" t="n">
+      <c r="C37" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="D37" s="43" t="n">
+      <c r="D37" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E37" s="46" t="n">
+      <c r="E37" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F37" s="46" t="n">
+      <c r="F37" s="48" t="n">
         <v>350</v>
       </c>
-      <c r="G37" s="46" t="n">
+      <c r="G37" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="46" t="n">
+      <c r="H37" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="46" t="n">
+      <c r="I37" s="48" t="n">
         <v>220</v>
       </c>
-      <c r="J37" s="46" t="n">
+      <c r="J37" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="K37" s="53">
+      <c r="K37" s="55">
         <f>IF(B37&gt;0,(F37+G37+H37+I37+(B37*C37/60)*D37*E37+J37*B37)/B37,0)</f>
         <v/>
       </c>
-      <c r="L37" s="48">
+      <c r="L37" s="50">
         <f>K37-$C$27</f>
         <v/>
       </c>
@@ -11345,38 +11374,38 @@
           <t>EcoFriendly Foods (Moneta, VA)</t>
         </is>
       </c>
-      <c r="B38" s="43" t="n">
+      <c r="B38" s="45" t="n">
         <v>30</v>
       </c>
-      <c r="C38" s="45" t="n">
+      <c r="C38" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="D38" s="43" t="n">
+      <c r="D38" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E38" s="46" t="n">
+      <c r="E38" s="48" t="n">
         <v>48</v>
       </c>
-      <c r="F38" s="46" t="n">
+      <c r="F38" s="48" t="n">
         <v>400</v>
       </c>
-      <c r="G38" s="46" t="n">
+      <c r="G38" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="46" t="n">
+      <c r="H38" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="I38" s="46" t="n">
+      <c r="I38" s="48" t="n">
         <v>350</v>
       </c>
-      <c r="J38" s="46" t="n">
+      <c r="J38" s="48" t="n">
         <v>9</v>
       </c>
-      <c r="K38" s="53">
+      <c r="K38" s="55">
         <f>IF(B38&gt;0,(F38+G38+H38+I38+(B38*C38/60)*D38*E38+J38*B38)/B38,0)</f>
         <v/>
       </c>
-      <c r="L38" s="48">
+      <c r="L38" s="50">
         <f>K38-$C$27</f>
         <v/>
       </c>
@@ -11387,38 +11416,38 @@
           <t>Midwest Research Swine (MN) — Model B</t>
         </is>
       </c>
-      <c r="B39" s="43" t="n">
+      <c r="B39" s="45" t="n">
         <v>60</v>
       </c>
-      <c r="C39" s="45" t="n">
+      <c r="C39" s="47" t="n">
         <v>12</v>
       </c>
-      <c r="D39" s="43" t="n">
+      <c r="D39" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="E39" s="46" t="n">
+      <c r="E39" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F39" s="46" t="n">
+      <c r="F39" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="G39" s="46" t="n">
+      <c r="G39" s="48" t="n">
         <v>900</v>
       </c>
-      <c r="H39" s="46" t="n">
+      <c r="H39" s="48" t="n">
         <v>200</v>
       </c>
-      <c r="I39" s="46" t="n">
+      <c r="I39" s="48" t="n">
         <v>400</v>
       </c>
-      <c r="J39" s="46" t="n">
+      <c r="J39" s="48" t="n">
         <v>9</v>
       </c>
-      <c r="K39" s="53">
+      <c r="K39" s="55">
         <f>IF(B39&gt;0,(F39+G39+H39+I39+(B39*C39/60)*D39*E39+J39*B39)/B39,0)</f>
         <v/>
       </c>
-      <c r="L39" s="48">
+      <c r="L39" s="50">
         <f>K39-$C$27</f>
         <v/>
       </c>
@@ -11429,65 +11458,65 @@
           <t>Smithfield BioScience (IA) — Model B</t>
         </is>
       </c>
-      <c r="B40" s="43" t="n">
+      <c r="B40" s="45" t="n">
         <v>80</v>
       </c>
-      <c r="C40" s="45" t="n">
+      <c r="C40" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="D40" s="43" t="n">
+      <c r="D40" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="E40" s="46" t="n">
+      <c r="E40" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F40" s="46" t="n">
+      <c r="F40" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="46" t="n">
+      <c r="G40" s="48" t="n">
         <v>1200</v>
       </c>
-      <c r="H40" s="46" t="n">
+      <c r="H40" s="48" t="n">
         <v>150</v>
       </c>
-      <c r="I40" s="46" t="n">
+      <c r="I40" s="48" t="n">
         <v>300</v>
       </c>
-      <c r="J40" s="46" t="n">
+      <c r="J40" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="K40" s="53">
+      <c r="K40" s="55">
         <f>IF(B40&gt;0,(F40+G40+H40+I40+(B40*C40/60)*D40*E40+J40*B40)/B40,0)</f>
         <v/>
       </c>
-      <c r="L40" s="48">
+      <c r="L40" s="50">
         <f>K40-$C$27</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="54" t="inlineStr">
+      <c r="A42" s="56" t="inlineStr">
         <is>
           <t>•  For Model B (plant harvests): set Crew = 0 and enter the plant's per-visit harvest fee under 'Plant fee / harvest fee'.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="54" t="inlineStr">
+      <c r="A43" s="56" t="inlineStr">
         <is>
           <t>•  Cost/block = (rental + plant fee + our inspector + transport + harvester labor + inventory × blocks) ÷ blocks.  Harvester labor = (min/block ÷ 60) × blocks × crew × rate.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="54" t="inlineStr">
+      <c r="A44" s="56" t="inlineStr">
         <is>
           <t>•  Compare Cost/block (col ⇒) to buy-direct list prices: ~$141/organ and $582/pelvic block (Innovative Research). Self-harvest usually wins because one visit yields many blocks at once.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="54" t="inlineStr">
+      <c r="A45" s="56" t="inlineStr">
         <is>
           <t>•  Every blue number is an ILLUSTRATIVE placeholder to show the format — none are researched costs. Replace them with your real time-studies, rental terms, wages, freight, and holding costs.</t>
         </is>
@@ -11589,11 +11618,11 @@
           <t>BOTTOM LINE: The EU does NOT require your suppliers to hand you a standalone 'APHIS certificate.' It requires (1) the ORIGIN establishment (the slaughterhouse) to be APHIS-approved and LISTED on the EU TRACES establishment list for the correct animal-by-product category, and (2) an APHIS Veterinary Services-ENDORSED EU health certificate that YOUR company, as the exporter, carries with each shipment. Your instinct is right in substance — the supplier does need an APHIS eligibility/listing status — but it is a system tied to a specific product + destination, not a certificate on the wall.   ⚠ This tab is orientation, NOT legal advice: confirm the exact category and certificate with APHIS VS, your EU importer, and (if any product is a device) your notified body.</t>
         </is>
       </c>
-      <c r="B4" s="63" t="n"/>
-      <c r="C4" s="62" t="n"/>
+      <c r="B4" s="65" t="n"/>
+      <c r="C4" s="64" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="41" t="inlineStr">
+      <c r="A6" s="43" t="inlineStr">
         <is>
           <t>HOW TO CHECK APHIS / EXPORT STATUS YOURSELF  (the lookup sites)</t>
         </is>
@@ -11605,8 +11634,8 @@
           <t>There is NO single 'APHIS-certified slaughterhouse' lookup — the right source depends on WHAT is exported.</t>
         </is>
       </c>
-      <c r="B7" s="63" t="n"/>
-      <c r="C7" s="62" t="n"/>
+      <c r="B7" s="65" t="n"/>
+      <c r="C7" s="64" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -11619,7 +11648,7 @@
           <t>FSIS 'Eligible U.S. Establishments by Country' → the European Union page (plant must be in the FSIS 'Pork for the EU' / PFEU program).  fsis.usda.gov/inspection/import-export/import-export-library</t>
         </is>
       </c>
-      <c r="C8" s="62" t="n"/>
+      <c r="C8" s="64" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -11632,7 +11661,7 @@
           <t>FSIS Meat/Poultry/Egg (MPI) Directory — an establishment's 'Certification – Export' activity means it can issue export certs for SOME country; it does NOT mean EU-eligible.  fsis.usda.gov/inspection/establishments/meat-poultry-and-egg-product-inspection-directory</t>
         </is>
       </c>
-      <c r="C9" s="62" t="n"/>
+      <c r="C9" s="64" t="n"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -11645,7 +11674,7 @@
           <t>APHIS 'Export Animal Products to the European Union' — APHIS Veterinary Services (not FSIS) compiles the by-product establishment listing under Reg (EU) 142/2011. No public per-plant lookup; email vs.export.product.facilities@usda.gov.  aphis.usda.gov/animal-product-export/export-animal-products-european-union</t>
         </is>
       </c>
-      <c r="C10" s="62" t="n"/>
+      <c r="C10" s="64" t="n"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -11658,7 +11687,7 @@
           <t>EU TRACES-NT establishment search — filter Country = United States; FSIS edible plants appear under fresh-meat/meat-products, APHIS by-product plants under animal-by-products. Interactive only.  webgate.ec.europa.eu/tracesnt/directory/listing/establishment/publication  (US mirror: usda-eu.org/import-controls/approved-u-s-establishments)</t>
         </is>
       </c>
-      <c r="C11" s="62" t="n"/>
+      <c r="C11" s="64" t="n"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -11671,34 +11700,34 @@
           <t>Edible meat → FSIS list + TRACES fresh-meat section.  Non-food research tissue → APHIS VS listing + TRACES animal-by-products section.  FSIS 'Certification–Export' ≠ EU-eligible ≠ APHIS by-product listing.</t>
         </is>
       </c>
-      <c r="C12" s="62" t="n"/>
+      <c r="C12" s="64" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="41" t="inlineStr">
+      <c r="A14" s="43" t="inlineStr">
         <is>
           <t>THE THREE REGIMES — APHIS vs FSIS vs STATE  (not tiers of one thing)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="55" t="inlineStr">
+      <c r="A15" s="57" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="B15" s="55" t="inlineStr">
+      <c r="B15" s="57" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C15" s="55" t="inlineStr">
+      <c r="C15" s="57" t="inlineStr">
         <is>
           <t>What it means for you</t>
         </is>
       </c>
     </row>
     <row r="16" ht="62" customHeight="1">
-      <c r="A16" s="56" t="inlineStr">
+      <c r="A16" s="58" t="inlineStr">
         <is>
           <t>USDA FSIS
 (Food Safety &amp; Inspection Service)</t>
@@ -11716,7 +11745,7 @@
       </c>
     </row>
     <row r="17" ht="62" customHeight="1">
-      <c r="A17" s="56" t="inlineStr">
+      <c r="A17" s="58" t="inlineStr">
         <is>
           <t>USDA APHIS Veterinary Services (VS)</t>
         </is>
@@ -11733,7 +11762,7 @@
       </c>
     </row>
     <row r="18" ht="62" customHeight="1">
-      <c r="A18" s="56" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>State meat inspection</t>
         </is>
@@ -11750,7 +11779,7 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="41" t="inlineStr">
+      <c r="A20" s="43" t="inlineStr">
         <is>
           <t>WHAT THE EU ACTUALLY REQUIRES  (the practical spine)</t>
         </is>
@@ -11767,7 +11796,7 @@
           <t>Regulation (EC) No 1069/2009 (the parent 'animal by-products' regulation — health rules for animal by-products NOT for human consumption) + Commission Regulation (EU) No 142/2011 (the implementing rules: categories, permitted uses, import conditions, model health certificates).</t>
         </is>
       </c>
-      <c r="C21" s="62" t="n"/>
+      <c r="C21" s="64" t="n"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
@@ -11780,7 +11809,7 @@
           <t>Porcine slaughter byproducts for technical/research/manufacturing use are typically CATEGORY 3 (lowest risk) — but classification is use-dependent, so confirm it. Common CN codes 0511 91 / 0511 99 / 3001. 142/2011 has special rules for research/diagnostic samples (Art. 11) and an 'Intermediate Products – Chapter 20' pathway for material used to manufacture medicinal products / medical devices.</t>
         </is>
       </c>
-      <c r="C22" s="62" t="n"/>
+      <c r="C22" s="64" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -11788,8 +11817,8 @@
           <t>The four-step import spine</t>
         </is>
       </c>
-      <c r="B23" s="63" t="n"/>
-      <c r="C23" s="62" t="n"/>
+      <c r="B23" s="65" t="n"/>
+      <c r="C23" s="64" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -11797,8 +11826,8 @@
           <t>•  1. APPROVED THIRD COUNTRY — the US must be listed for that ABP category (country lists in Annex XIV of Reg (EU) 142/2011, amended e.g. by Reg (EU) 2022/384). The US is listed for many ABP categories.</t>
         </is>
       </c>
-      <c r="B24" s="63" t="n"/>
-      <c r="C24" s="62" t="n"/>
+      <c r="B24" s="65" t="n"/>
+      <c r="C24" s="64" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -11806,8 +11835,8 @@
           <t>•  2. LISTED ESTABLISHMENT — the origin plant must be APHIS-approved and appear on the EU TRACES establishment list for the category. (APHIS: 'Facilities must be listed by APHIS in compliance with Reg (EU) 142/2011 to export.')</t>
         </is>
       </c>
-      <c r="B25" s="63" t="n"/>
-      <c r="C25" s="62" t="n"/>
+      <c r="B25" s="65" t="n"/>
+      <c r="C25" s="64" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -11815,8 +11844,8 @@
           <t>•  3. ENDORSED HEALTH CERTIFICATE — a model veterinary health certificate (matching the category/use, from the 142/2011 annexes) accompanies the consignment, endorsed by APHIS Veterinary Services.</t>
         </is>
       </c>
-      <c r="B26" s="63" t="n"/>
-      <c r="C26" s="62" t="n"/>
+      <c r="B26" s="65" t="n"/>
+      <c r="C26" s="64" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -11824,8 +11853,8 @@
           <t>•  4. BORDER ENTRY via TRACES — entry through an EU Border Control Post with prior notification in TRACES (the CHED). APHIS endorses the certificate but does NOT prepare the EU entry document — that is the importer's side.</t>
         </is>
       </c>
-      <c r="B27" s="63" t="n"/>
-      <c r="C27" s="62" t="n"/>
+      <c r="B27" s="65" t="n"/>
+      <c r="C27" s="64" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -11838,10 +11867,10 @@
           <t>Slaughterhouse → exporter (facility listing status, species/origin, inspection records, traceability) → APHIS endorses the certificate → EU importer lodges the CHED in TRACES.</t>
         </is>
       </c>
-      <c r="C28" s="62" t="n"/>
+      <c r="C28" s="64" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="41" t="inlineStr">
+      <c r="A29" s="43" t="inlineStr">
         <is>
           <t>MEDICAL-DEVICE ANGLE  (only if the end product is actually a device)</t>
         </is>
@@ -11853,8 +11882,8 @@
           <t>•  A surgical-training / anatomical 'model' is OFTEN NOT a medical device (not intended to diagnose/treat a patient). If so, MDR does not apply — but the tissue is still an animal by-product, so the ABP rules above still govern EU entry. Whether a given 'model' is a device is a classification call for a regulatory specialist / notified body.</t>
         </is>
       </c>
-      <c r="B30" s="63" t="n"/>
-      <c r="C30" s="62" t="n"/>
+      <c r="B30" s="65" t="n"/>
+      <c r="C30" s="64" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -11862,8 +11891,8 @@
           <t>•  If it IS a device: Regulation (EU) 2017/745 (MDR), Annex I GSPR 13.1 governs devices manufactured using animal tissue.</t>
         </is>
       </c>
-      <c r="B31" s="63" t="n"/>
-      <c r="C31" s="62" t="n"/>
+      <c r="B31" s="65" t="n"/>
+      <c r="C31" s="64" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -11871,8 +11900,8 @@
           <t>•  KEY: Regulation (EU) No 722/2012 (the special TSE regime) does NOT cover porcine — it is limited to bovine, ovine, caprine, deer, elk, mink and cats. So porcine devices sit under MDR's GENERAL animal-origin requirements (13.1), NOT the 722/2012 procedure.</t>
         </is>
       </c>
-      <c r="B32" s="63" t="n"/>
-      <c r="C32" s="62" t="n"/>
+      <c r="B32" s="65" t="n"/>
+      <c r="C32" s="64" t="n"/>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -11880,11 +11909,11 @@
           <t>•  MDR 13.1 expectations (good practice for porcine too): animals subject to veterinary controls adapted to intended use; retain geographical-origin records; sourcing/processing/testing to the ISO 22442 series; source from healthy animals fit for human consumption, EXCLUDING fallen stock, emergency-slaughtered, and diseased animals.</t>
         </is>
       </c>
-      <c r="B33" s="63" t="n"/>
-      <c r="C33" s="62" t="n"/>
+      <c r="B33" s="65" t="n"/>
+      <c r="C33" s="64" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="41" t="inlineStr">
+      <c r="A34" s="43" t="inlineStr">
         <is>
           <t>DOES THE SUPPLIER NEED 'APHIS CERTIFICATION'?  (direct answer)</t>
         </is>
@@ -11896,8 +11925,8 @@
           <t>•  'APHIS certification' is not one credential on the wall — it is a SYSTEM: (i) APHIS approves/lists a specific facility for a specific export certificate/category, and (ii) APHIS VS endorses the actual health certificate per shipment.</t>
         </is>
       </c>
-      <c r="B35" s="63" t="n"/>
-      <c r="C35" s="62" t="n"/>
+      <c r="B35" s="65" t="n"/>
+      <c r="C35" s="64" t="n"/>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -11905,8 +11934,8 @@
           <t>•  WHO NEEDS WHAT: the EXPORTER (your company) obtains and presents the APHIS-endorsed health certificate. But for APHIS to endorse it and the EU to accept the consignment, the SOURCE establishment usually must be APHIS-approved and on the EU/TRACES list for that category. So the supplier DOES need an eligibility/listing status — the grain of truth in what you were told.</t>
         </is>
       </c>
-      <c r="B36" s="63" t="n"/>
-      <c r="C36" s="62" t="n"/>
+      <c r="B36" s="65" t="n"/>
+      <c r="C36" s="64" t="n"/>
     </row>
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -11914,18 +11943,18 @@
           <t>•  A small, humane, STATE-inspected family plant that has never exported will NOT have this yet and must apply — via APHIS VS Field Operations / Veterinary Export Trade Services — and get placed on the EU TRACES list. Confirm with APHIS whether the plant's state-inspection status is acceptable for the EXACT certificate you'll use (some certs require ante-/post-mortem inspection or 'fit for human consumption'; state inspection typically satisfies this, but the certificate wording controls).</t>
         </is>
       </c>
-      <c r="B37" s="63" t="n"/>
-      <c r="C37" s="62" t="n"/>
+      <c r="B37" s="65" t="n"/>
+      <c r="C37" s="64" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="41" t="inlineStr">
+      <c r="A39" s="43" t="inlineStr">
         <is>
           <t>SUPPLIER CHECKLIST — require in writing (also in the Call Question Sheet, section G)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="57" t="n">
+      <c r="A40" s="59" t="n">
         <v>1</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -11933,10 +11962,10 @@
           <t>APHIS export eligibility / facility approval — is the establishment already APHIS-approved and on the EU TRACES establishment list for the relevant ABP category? If not, willing to apply via APHIS VS?</t>
         </is>
       </c>
-      <c r="C40" s="62" t="n"/>
+      <c r="C40" s="64" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="57" t="n">
+      <c r="A41" s="59" t="n">
         <v>2</v>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -11944,10 +11973,10 @@
           <t>Inspection status — USDA-FSIS or state-inspected? Can it document ante-mortem AND post-mortem veterinary inspection of the source animals? (Needed for many EU certificates and for MDR 13.1.)</t>
         </is>
       </c>
-      <c r="C41" s="62" t="n"/>
+      <c r="C41" s="64" t="n"/>
     </row>
     <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="57" t="n">
+      <c r="A42" s="59" t="n">
         <v>3</v>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -11955,10 +11984,10 @@
           <t>Veterinary health certificates / affidavits — can it supply the source declarations/affidavits APHIS VS needs to endorse the EU model health certificate, and per-lot documentation?</t>
         </is>
       </c>
-      <c r="C42" s="62" t="n"/>
+      <c r="C42" s="64" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="57" t="n">
+      <c r="A43" s="59" t="n">
         <v>4</v>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -11966,10 +11995,10 @@
           <t>Species, herd health &amp; country/region of origin — porcine only; US origin; herd-health assurances; animals healthy and fit for human consumption, with fallen stock / emergency-slaughtered / diseased animals excluded.</t>
         </is>
       </c>
-      <c r="C43" s="62" t="n"/>
+      <c r="C43" s="64" t="n"/>
     </row>
     <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="57" t="n">
+      <c r="A44" s="59" t="n">
         <v>5</v>
       </c>
       <c r="B44" s="5" t="inlineStr">
@@ -11977,10 +12006,10 @@
           <t>Traceability — lot-level traceability from live animal → tissue → shipment, and retention of geographical-origin records (required under MDR Annex I 13.1 if the end product is a device).</t>
         </is>
       </c>
-      <c r="C44" s="62" t="n"/>
+      <c r="C44" s="64" t="n"/>
     </row>
     <row r="45" ht="36" customHeight="1">
-      <c r="A45" s="57" t="n">
+      <c r="A45" s="59" t="n">
         <v>6</v>
       </c>
       <c r="B45" s="5" t="inlineStr">
@@ -11988,10 +12017,10 @@
           <t>Records retention &amp; audit access — inspection, sourcing, and lot records; willingness to support APHIS facility audits and (if a device) notified-body / ISO 22442 documentation requests.</t>
         </is>
       </c>
-      <c r="C45" s="62" t="n"/>
+      <c r="C45" s="64" t="n"/>
     </row>
     <row r="46" ht="36" customHeight="1">
-      <c r="A46" s="57" t="n">
+      <c r="A46" s="59" t="n">
         <v>7</v>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -11999,10 +12028,10 @@
           <t>Category/use agreement — align on the ABP category (likely Cat 3) and intended use so the correct 142/2011 model certificate (research/diagnostic sample, commercial sample, technical product, or intermediate-product Chapter 20) can be identified.</t>
         </is>
       </c>
-      <c r="C46" s="62" t="n"/>
+      <c r="C46" s="64" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="41" t="inlineStr">
+      <c r="A48" s="43" t="inlineStr">
         <is>
           <t>WHO TO LOOP IN  (this tab is orientation, not final legal advice)</t>
         </is>
@@ -12014,8 +12043,8 @@
           <t>•  APHIS VS Field Operations / Veterinary Export Trade Services — the authority on facility listing and which EU certificate applies to your exact product; they endorse the certificate.</t>
         </is>
       </c>
-      <c r="B49" s="63" t="n"/>
-      <c r="C49" s="62" t="n"/>
+      <c r="B49" s="65" t="n"/>
+      <c r="C49" s="64" t="n"/>
     </row>
     <row r="50" ht="26" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -12023,8 +12052,8 @@
           <t>•  Your EU importer — lodges the TRACES/CHED entry and knows the receiving Member State's border-control expectations.</t>
         </is>
       </c>
-      <c r="B50" s="63" t="n"/>
-      <c r="C50" s="62" t="n"/>
+      <c r="B50" s="65" t="n"/>
+      <c r="C50" s="64" t="n"/>
     </row>
     <row r="51" ht="26" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -12032,8 +12061,8 @@
           <t>•  A customs / regulatory specialist — to fix the ABP category, CN code, and correct 142/2011 model certificate per product line.</t>
         </is>
       </c>
-      <c r="B51" s="63" t="n"/>
-      <c r="C51" s="62" t="n"/>
+      <c r="B51" s="65" t="n"/>
+      <c r="C51" s="64" t="n"/>
     </row>
     <row r="52" ht="26" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
@@ -12041,60 +12070,60 @@
           <t>•  A notified body — only if any product is actually a medical device (MDR Annex I 13.1; porcine is outside 722/2012 but still scrutinized).</t>
         </is>
       </c>
-      <c r="B52" s="63" t="n"/>
-      <c r="C52" s="62" t="n"/>
+      <c r="B52" s="65" t="n"/>
+      <c r="C52" s="64" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="41" t="inlineStr">
+      <c r="A54" s="43" t="inlineStr">
         <is>
           <t>KEY SOURCES</t>
         </is>
       </c>
     </row>
     <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="58" t="inlineStr">
+      <c r="A55" s="60" t="inlineStr">
         <is>
           <t>•  APHIS — International Animal Product Export Regulations (IREGS): aphis.usda.gov/animal-product-export/international-animal-product-export-regulations</t>
         </is>
       </c>
-      <c r="B55" s="63" t="n"/>
-      <c r="C55" s="62" t="n"/>
+      <c r="B55" s="65" t="n"/>
+      <c r="C55" s="64" t="n"/>
     </row>
     <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="58" t="inlineStr">
+      <c r="A56" s="60" t="inlineStr">
         <is>
           <t>•  APHIS — Export Animal Products to the EU: aphis.usda.gov/animal-product-export/export-animal-products-european-union</t>
         </is>
       </c>
-      <c r="B56" s="63" t="n"/>
-      <c r="C56" s="62" t="n"/>
+      <c r="B56" s="65" t="n"/>
+      <c r="C56" s="64" t="n"/>
     </row>
     <row r="57" ht="24" customHeight="1">
-      <c r="A57" s="58" t="inlineStr">
+      <c r="A57" s="60" t="inlineStr">
         <is>
           <t>•  EU ABP — Reg (EC) 1069/2009 (EUR-Lex summary) &amp; Reg (EU) 142/2011 (legislation.gov.uk consolidated); country lists Annex XIV via Reg (EU) 2022/384</t>
         </is>
       </c>
-      <c r="B57" s="63" t="n"/>
-      <c r="C57" s="62" t="n"/>
+      <c r="B57" s="65" t="n"/>
+      <c r="C57" s="64" t="n"/>
     </row>
     <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="58" t="inlineStr">
+      <c r="A58" s="60" t="inlineStr">
         <is>
           <t>•  EU devices — MDR (EU) 2017/745 (EUR-Lex); Reg (EU) 722/2012 (legislation.gov.uk) — porcine NOT covered; ISO 22442 series (industry practice)</t>
         </is>
       </c>
-      <c r="B58" s="63" t="n"/>
-      <c r="C58" s="62" t="n"/>
+      <c r="B58" s="65" t="n"/>
+      <c r="C58" s="64" t="n"/>
     </row>
     <row r="59" ht="24" customHeight="1">
-      <c r="A59" s="58" t="inlineStr">
+      <c r="A59" s="60" t="inlineStr">
         <is>
           <t>•  USDA-EU approved U.S. establishments: usda-eu.org/import-controls/approved-u-s-establishments  ·  Third-country establishment lists explained: agrinfo.eu</t>
         </is>
       </c>
-      <c r="B59" s="63" t="n"/>
-      <c r="C59" s="62" t="n"/>
+      <c r="B59" s="65" t="n"/>
+      <c r="C59" s="64" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="48">

</xml_diff>

<commit_message>
Record two client corrections: Villari tissue gate is hard; Parks is Model B-T
Client-stated 2026-09-03, applied to the roster, comparison tab and Overview:

- Villari / The Pork Company: the tissue gate is HARD. Leaf fat only; no organ
  planning through Villari. The 2026-08-17 "negotiable wedge" reading is
  superseded and kept only as background should Villari ever reopen the topic.
- Parks Family Meats: their OWN people harvest, trained by us (Model B-T) - the
  working template for supervised-harvest partnerships. The play reframed to
  program pricing on a committed window harvested by their trained crew.

Also restates the base's operating models: Nahunta / Martin's / CQP = our techs
on site (Model A); Parks = B-T; Villari = leaf fat only.

Formatting reapplied; audit clean (0 under-height rows, 0 empty-anchor merges).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvB48tbAk8juvoi9bxkFTf
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
+++ b/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11760" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview &amp; Method" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meeting Notes 2026-08" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anatomical Spec" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Scoring" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Roster" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NC Comparison 2026-08-17" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="National Direct Suppliers" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Models &amp; Make-vs-Buy" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TCO Calculator" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APHIS &amp; EU Export" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Question Sheet" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Confidence" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deep Study (Verified)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Overview &amp; Method" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Meeting Notes 2026-08" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Action Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Anatomical Spec" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Legend &amp; Scoring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Supplier Roster" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NC Comparison 2026-08-17" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="National Direct Suppliers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Models &amp; Make-vs-Buy" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TCO Calculator" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="APHIS &amp; EU Export" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Call Question Sheet" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sources &amp; Confidence" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Deep Study (Verified)" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Supplier Roster'!$A$4:$R$4</definedName>
@@ -1760,10 +1760,10 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="152.4" customHeight="1" s="59">
+    <row r="30" ht="165.8" customHeight="1" s="59">
       <c r="A30" s="68" t="inlineStr">
         <is>
-          <t>★ FOCUS-REGION PASS (2026-08-17, client-directed) — CURRENT BASE RE-VERIFIED + WEST / NORTH-OF-RALEIGH / EAST SWEPT. Ground truth recorded: we currently work with Nahunta and Martin's and CQP (our harvesters on site), Parks (small, BBQ pigs, a bit expensive) and Villari (LEAF FAT ONLY — no organs). Headlines: (1) all three cat-3 market-hog floors in NC/SC/VA are ALREADY ours (Martin's, Parks, CQP) — there is no second Martin's; dependence is reduced by contract, not discovery. (2) Villari's 'no organs' is negotiable but hard near-term — a $3.27M wastewater project (county loan 3/2026) blocks new offal handling until ~2027; the wedge is a paid client-crewed viscera-table pilot, and their $800K NCAMPI award (7/7/2026) is the leverage moment. (3) Larry's Sausage promoted to the #6 call: the east's only established sow-class organ lane. (4) NEW FINDS: McLamb's Abattoir (Benson P-247, 37 mi) and Gale McLamb (Dunn P-221, 44 mi) — unworked state-inspected floors closer than any current supplier except Nahunta. (5) North of Raleigh is a confirmed desert (3 kill floors in 13 counties — and they're our Sims cluster); the west has NO volume play but holds Piedmont (AWA/Temple Grandin, all four hog classes, actually INSIDE the radius at 116 mi) and three Nahunta-structure state plants. (6) CQP carries a 2018-2020 humane-handling history (PETA attention) the file lacked — audit before scaling. (7) Kansas City Sausage/Godwin is RESOLVED DEAD; 8 nearby closures in 20 months say: lock in survivors. See the 'NC Comparison 2026-08-17' tab.</t>
+          <t>★ FOCUS-REGION PASS (2026-08-17, client-directed) — CURRENT BASE RE-VERIFIED + WEST / NORTH-OF-RALEIGH / EAST SWEPT. Ground truth recorded: we currently work with Nahunta and Martin's and CQP (our harvesters on site), Parks (small, BBQ pigs, a bit expensive) and Villari (LEAF FAT ONLY — no organs). Headlines: (1) all three cat-3 market-hog floors in NC/SC/VA are ALREADY ours (Martin's, Parks, CQP) — there is no second Martin's; dependence is reduced by contract, not discovery. (2) VILLARI — CORRECTED 2026-09-03: the tissue gate is HARD (client-stated); no organ planning through Villari; keep leaf fat flowing and revisit only if they reopen it (background: wastewater project to ~2027; $800K NCAMPI award 7/7/2026). (3) Larry's Sausage promoted to the #6 call: the east's only established sow-class organ lane. (4) NEW FINDS: McLamb's Abattoir (Benson P-247, 37 mi) and Gale McLamb (Dunn P-221, 44 mi) — unworked state-inspected floors closer than any current supplier except Nahunta. (5) North of Raleigh is a confirmed desert (3 kill floors in 13 counties — and they're our Sims cluster); the west has NO volume play but holds Piedmont (AWA/Temple Grandin, all four hog classes, actually INSIDE the radius at 116 mi) and three Nahunta-structure state plants. (6) CQP carries a 2018-2020 humane-handling history (PETA attention) the file lacked — audit before scaling. (7) Kansas City Sausage/Godwin is RESOLVED DEAD; 8 nearby closures in 20 months say: lock in survivors. See the 'NC Comparison 2026-08-17' tab. ★ ALSO CORRECTED 2026-09-03: PARKS harvests with THEIR OWN people under OUR training (Model B-T) — the base already runs both operating models, and candidate ratings now score A-fit (host our techs) and B-fit (their crew, our training) separately — see Supplier_Outreach_Plan.xlsx.</t>
         </is>
       </c>
       <c r="B30" s="65" t="n"/>
@@ -2151,7 +2151,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="31.8" customHeight="1" s="59">
+    <row r="11" ht="18.4" customHeight="1" s="59">
       <c r="A11" s="74" t="inlineStr">
         <is>
           <t>Harvester labor per visit</t>
@@ -2218,7 +2218,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="31.8" customHeight="1" s="59">
+    <row r="16" ht="18.4" customHeight="1" s="59">
       <c r="A16" s="74" t="inlineStr">
         <is>
           <t>Facility fixed subtotal</t>
@@ -2292,7 +2292,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="31.8" customHeight="1" s="59">
+    <row r="22" ht="18.4" customHeight="1" s="59">
       <c r="A22" s="74" t="inlineStr">
         <is>
           <t>Total cost per visit</t>
@@ -2307,7 +2307,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="31.8" customHeight="1" s="59">
+    <row r="23" ht="18.4" customHeight="1" s="59">
       <c r="A23" s="78" t="inlineStr">
         <is>
           <t>★ TOTAL COST PER BLOCK</t>
@@ -2322,7 +2322,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="31.8" customHeight="1" s="59">
+    <row r="24" ht="18.4" customHeight="1" s="59">
       <c r="A24" s="74" t="inlineStr">
         <is>
           <t>Memo: harvester labor per block</t>
@@ -2337,7 +2337,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="31.8" customHeight="1" s="59">
+    <row r="25" ht="18.4" customHeight="1" s="59">
       <c r="A25" s="74" t="inlineStr">
         <is>
           <t>Memo: fixed+transport per block</t>
@@ -2406,7 +2406,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="125.6" customHeight="1" s="59">
+    <row r="30" ht="18.4" customHeight="1" s="59">
       <c r="A30" s="74" t="inlineStr">
         <is>
           <t>Verdict</t>
@@ -2501,7 +2501,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="72" customHeight="1" s="59">
+    <row r="34" ht="31.8" customHeight="1" s="59">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Nahunta Pork Center (Pikeville, NC)</t>
@@ -2543,7 +2543,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="72" customHeight="1" s="59">
+    <row r="35" ht="31.8" customHeight="1" s="59">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Martin's Pork Products (Falcon, NC)</t>
@@ -2585,7 +2585,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="72" customHeight="1" s="59">
+    <row r="36" ht="18.4" customHeight="1" s="59">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Piedmont Custom Meats (NC)</t>
@@ -2627,7 +2627,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="72" customHeight="1" s="59">
+    <row r="37" ht="18.4" customHeight="1" s="59">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>Acre Station Meat Farm (NC)</t>
@@ -2669,7 +2669,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="72" customHeight="1" s="59">
+    <row r="38" ht="18.4" customHeight="1" s="59">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>EcoFriendly Foods (Moneta, VA)</t>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="72" customHeight="1" s="59">
+    <row r="39" ht="31.8" customHeight="1" s="59">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Midwest Research Swine (MN) — Model B</t>
@@ -2753,7 +2753,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="72" customHeight="1" s="59">
+    <row r="40" ht="31.8" customHeight="1" s="59">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Smithfield BioScience (IA) — Model B</t>
@@ -4230,7 +4230,7 @@
     <col width="30" customWidth="1" style="59" min="1" max="1"/>
     <col width="52" customWidth="1" style="59" min="2" max="2"/>
     <col width="13" customWidth="1" style="59" min="3" max="3"/>
-    <col width="60" customWidth="1" style="59" min="4" max="4"/>
+    <col width="90" customWidth="1" style="59" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.1" customHeight="1" s="59">
@@ -4270,7 +4270,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="139" customHeight="1" s="59">
+    <row r="5" ht="98.8" customHeight="1" s="59">
       <c r="A5" s="138" t="inlineStr">
         <is>
           <t>★ FOCUS-REGION PASS
@@ -4293,7 +4293,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="192.6" customHeight="1" s="59">
+    <row r="6" ht="125.6" customHeight="1" s="59">
       <c r="A6" s="138" t="inlineStr">
         <is>
           <t>★ FULL ROSTER RE-VERIFICATION
@@ -4316,7 +4316,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="125.6" customHeight="1" s="59">
+    <row r="7" ht="85.40000000000001" customHeight="1" s="59">
       <c r="A7" s="138" t="inlineStr">
         <is>
           <t>Volume categories → weekly ceilings</t>
@@ -4338,7 +4338,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="139" customHeight="1" s="59">
+    <row r="8" ht="98.8" customHeight="1" s="59">
       <c r="A8" s="138" t="inlineStr">
         <is>
           <t>Enforcement — what was actually checked</t>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="9" ht="58.6" customHeight="1" s="59">
       <c r="A9" s="138" t="inlineStr">
         <is>
           <t>Road distances (120-mile Model A test)</t>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="152.4" customHeight="1" s="59">
+    <row r="10" ht="98.8" customHeight="1" s="59">
       <c r="A10" s="138" t="inlineStr">
         <is>
           <t>⚠ Claims withdrawn for lack of a source</t>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="31.8" customHeight="1" s="59">
+    <row r="12" ht="18.4" customHeight="1" s="59">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Pel-Freez thyroid price</t>
@@ -4580,7 +4580,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="31.8" customHeight="1" s="59">
+    <row r="19" ht="18.4" customHeight="1" s="59">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Cross-off leads</t>
@@ -4624,7 +4624,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="58.6" customHeight="1" s="59">
+    <row r="21" ht="45.2" customHeight="1" s="59">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Martin's Pork Products (incumbent)</t>
@@ -4646,7 +4646,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="31.8" customHeight="1" s="59">
+    <row r="22" ht="18.4" customHeight="1" s="59">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Nahunta</t>
@@ -4668,7 +4668,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="45.2" customHeight="1" s="59">
+    <row r="23" ht="31.8" customHeight="1" s="59">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>SC facilities</t>
@@ -4756,7 +4756,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="72" customHeight="1" s="59">
+    <row r="27" ht="58.6" customHeight="1" s="59">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Authoritative confirmation source</t>
@@ -4778,7 +4778,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="45.2" customHeight="1" s="59">
+    <row r="28" ht="31.8" customHeight="1" s="59">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>APHIS vs FSIS vs state inspection</t>
@@ -4800,7 +4800,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="58.6" customHeight="1" s="59">
+    <row r="29" ht="45.2" customHeight="1" s="59">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>EU animal by-products law</t>
@@ -4822,7 +4822,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="58.6" customHeight="1" s="59">
+    <row r="30" ht="45.2" customHeight="1" s="59">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>EU medical-device angle</t>
@@ -4844,7 +4844,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="45.2" customHeight="1" s="59">
+    <row r="31" ht="31.8" customHeight="1" s="59">
       <c r="A31" s="4" t="inlineStr">
         <is>
           <t>APHIS / EU — caveat</t>
@@ -4866,7 +4866,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="58.6" customHeight="1" s="59">
+    <row r="32" ht="45.2" customHeight="1" s="59">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>USDA/FSIS enforcement (per facility)</t>
@@ -4888,7 +4888,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="58.6" customHeight="1" s="59">
+    <row r="33" ht="45.2" customHeight="1" s="59">
       <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Export / APHIS lookup sites</t>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="45.2" customHeight="1" s="59">
+    <row r="34" ht="31.8" customHeight="1" s="59">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>National vendors × EU export</t>
@@ -6780,10 +6780,10 @@
   <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="30" customWidth="1" style="59" min="1" max="1"/>
-    <col width="62" customWidth="1" style="59" min="2" max="2"/>
+    <col width="34" customWidth="1" style="59" min="1" max="1"/>
+    <col width="88" customWidth="1" style="59" min="2" max="2"/>
     <col width="28" customWidth="1" style="59" min="3" max="3"/>
-    <col width="16" customWidth="1" style="59" min="4" max="4"/>
+    <col width="18" customWidth="1" style="59" min="4" max="4"/>
     <col width="12" customWidth="1" style="59" min="5" max="6"/>
     <col width="12" customWidth="1" style="59" min="6" max="6"/>
   </cols>
@@ -6795,7 +6795,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="31.8" customHeight="1" s="59">
+    <row r="2" ht="18.4" customHeight="1" s="59">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>Sequenced: hold the internal strategy meeting FIRST, then send RFQ/Ps to the priority plants. The reach-first list was re-reviewed against volume, welfare/enforcement, certifications, and model fit.</t>
@@ -6842,7 +6842,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58.6" customHeight="1" s="59">
+    <row r="6" ht="45.2" customHeight="1" s="59">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>0a. WRITE THE ANATOMICAL SPEC  (do this FIRST)</t>
@@ -6870,7 +6870,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="179.2" customHeight="1" s="59">
+    <row r="7" ht="139" customHeight="1" s="59">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>0b. EMAIL APHIS VS — settle the EU-export question</t>
@@ -6900,7 +6900,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="246.2" customHeight="1" s="59">
+    <row r="8" ht="165.8" customHeight="1" s="59">
       <c r="A8" s="51" t="inlineStr">
         <is>
           <t>0c. ★★ INTERVIEW THE TISSUE COLLECTORS  (PRIORITY — client flagged)</t>
@@ -6932,7 +6932,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="72" customHeight="1" s="59">
+    <row r="9" ht="58.6" customHeight="1" s="59">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>1. Strategy &amp; requirements alignment  (COMPANY stakeholders — NOT slaughterhouses)</t>
@@ -6960,7 +6960,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="10" ht="58.6" customHeight="1" s="59">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>2. Outreach kickoff</t>
@@ -6988,7 +6988,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="11" ht="58.6" customHeight="1" s="59">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>3. Shortlist review &amp; scoring</t>
@@ -7016,7 +7016,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="165.8" customHeight="1" s="59">
+    <row r="12" ht="112.2" customHeight="1" s="59">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>4. FSIS FOIA on shortlist establishments</t>
@@ -7044,7 +7044,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="58.6" customHeight="1" s="59">
+    <row r="13" ht="45.2" customHeight="1" s="59">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>5. Site visits / audits  (top 2-3)</t>
@@ -7112,7 +7112,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="17" ht="72" customHeight="1" s="59">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>1. Nahunta Slaughter House  (NC state P-80A)
@@ -7143,7 +7143,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="98.8" customHeight="1" s="59">
+    <row r="18" ht="72" customHeight="1" s="59">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>2. Parks Family Meats, LLC  (M18296A, Talmadge-Aiken)
@@ -7174,7 +7174,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="72" customHeight="1" s="59">
+    <row r="19" ht="58.6" customHeight="1" s="59">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>3. Martin's Pork Products, Inc.  (M6720, Talmadge-Aiken)
@@ -7205,7 +7205,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="165.8" customHeight="1" s="59">
+    <row r="20" ht="112.2" customHeight="1" s="59">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>4. Custom Quality Packers, LLC  (M20129)
@@ -7234,7 +7234,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="21" ht="58.6" customHeight="1" s="59">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>5. Smithfield BioScience
@@ -7263,7 +7263,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="125.6" customHeight="1" s="59">
+    <row r="22" ht="85.40000000000001" customHeight="1" s="59">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>6. Larry's Sausage Co. (M8305)  ★ PROMOTED
@@ -7294,7 +7294,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="72" customHeight="1" s="59">
+    <row r="23" ht="58.6" customHeight="1" s="59">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>7. Wampler's Farm Sausage Co.  (M9065)
@@ -7323,7 +7323,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="24" ht="58.6" customHeight="1" s="59">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>8. EcoFriendly Foods, LLC  (M21938)
@@ -7352,7 +7352,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="58.6" customHeight="1" s="59">
+    <row r="25" ht="45.2" customHeight="1" s="59">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>9. Underground Slaughter LLC  (M51351)
@@ -7381,7 +7381,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="85.40000000000001" customHeight="1" s="59">
+    <row r="26" ht="58.6" customHeight="1" s="59">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>10. Flowers Slaughter House  (M21747)
@@ -7410,7 +7410,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="112.2" customHeight="1" s="59">
+    <row r="27" ht="72" customHeight="1" s="59">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>11. McLamb's Abattoir (P-247) + Gale McLamb Meats (P-221)
@@ -7440,7 +7440,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="72" customHeight="1" s="59">
+    <row r="28" ht="45.2" customHeight="1" s="59">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>12. Williamsburg Packing  (M4005)
@@ -7469,14 +7469,14 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="53.2" customHeight="1" s="59">
+    <row r="29" ht="41.2" customHeight="1" s="59">
       <c r="A29" s="60" t="inlineStr">
         <is>
           <t>•  SECONDARY (parallel track): get 1-2 buy-direct BENCHMARK quotes to price-check self-harvest — Tissue Source and Smithfield BioScience. AVOID Innovative Research for EU-bound product (research-use-only labelling is a likely EU blocker). Note that MIDWEST RESEARCH SWINE resolves to Est. M40110, Collagen Solutions (US) LLC DBA Evergen, Glencoe MN — FSIS category 2, so a ~192/wk ceiling, not the ~385/wk the roster carried. Its value is as a comparator and a make-vs-buy price check, not as a volume lane. Also call SIG INTERNATIONAL (Boyden IA, M20748 + V20748) — market hogs, FSIS category 3, and it carries a Certification-Export activity, which matters for anything EU-bound.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="101.5" customHeight="1" s="59">
+    <row r="30" ht="89.40000000000001" customHeight="1" s="59">
       <c r="A30" s="60" t="inlineStr">
         <is>
           <t>•  REMOVED FROM THE CONTACT ORDER BY THE FSIS PRIMARY-DATA SWEEP (do NOT reach): GUNNOE SAUSAGE CO. (Goode VA) — was #5. No establishment named 'Gunnoe' exists anywhere in the FSIS MPI directory and nothing is listed at Goode VA; the '~450/wk dedicated sow slaughterhouse since 1965' profile cannot be attached to an inspected establishment. BASS FARMS, INC. (M3521, Spring Hope NC) — was #4. Three claims refuted: it is federal M3521 not 'TA-3521' (and the grant IS live, which closes that open question); it is NOT 'slaughter only' — FSIS records slaughter AND processing, processing category 4, DBA 'Bass Farm Sausage', i.e. a sausage business with a small kill floor, not the 'purest Model A structure in the state'; and slaughter_volume_category = 1 = FEWER THAN 1,000 HEAD PER YEAR, under ~19/wk. It is also sow-only. Its value, if any, is as a PROCESSOR. TRIAD MEAT CUSTOM PROCESSING (Madison NC) — the only FSIS slaughter establishment at Madison is Triad Halal Meats (M46085), with NO swine flags of any kind. CAUGHMAN'S MEAT PLANT (Lexington SC) and SESSOMS PACKING (Ahoskie NC) — both carried USDA labels with nothing behind them; neither appears in the FSIS MPI directory. ⚠ 2026-08-17 FINAL: the Godwin question is CLOSED — KCS's own establishment M760A went inactive 9/3/2024 and no establishment exists at the site in the active or inactive directories. Also closed: Country Slaughter &amp; Meats (M32012 inactive 6/24/2025) and Assured Community Processing (M2123 inactive 11/10/2025) — the earlier 'number not found' mysteries were both closures.</t>
@@ -13386,7 +13386,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="219.4" customHeight="1" s="59">
+    <row r="62" ht="165.8" customHeight="1" s="59">
       <c r="A62" s="82" t="inlineStr">
         <is>
           <t>The Pork Company (Villari Food Group)</t>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="K62" s="83" t="inlineStr">
         <is>
-          <t>CLIENT GROUND TRUTH (2026-08-17): we buy LEAF FAT only — 'they can't do organs'. Research verdict: that wall is NEGOTIABLE BUT HARD NEAR-TERM. No regulatory or contractual blocker found (no third party holds the viscera; no organ SKUs in their catalog — viscera go inedible/rendering, inferred outlet Darling Ingredients Rose Hill ~10 mi). The real obstacle is the WASTEWATER crisis: a $3.27M pre-treatment project (Duplin County approved a $200K loan 3/2/2026; friction with the town of Warsaw documented) makes NEW offal handling unattractive until upgrades land (~2027).</t>
+          <t>CLIENT GROUND TRUTH — CORRECTED 2026-09-03: the tissue gate is HARD. We buy LEAF FAT only; Villari cannot / will not do organs, and this is not currently negotiable. The 2026-08-17 research reading ('negotiable but hard near-term', wastewater timing, viscera-table wedge) is SUPERSEDED as a plan — retained below only as background should VILLARI ever reopen the topic themselves.</t>
         </is>
       </c>
       <c r="L62" s="83" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="N62" s="83" t="inlineStr">
         <is>
-          <t>Model B candidate on volume</t>
+          <t>No — hard gate on tissue</t>
         </is>
       </c>
       <c r="O62" s="83" t="inlineStr">
@@ -13480,11 +13480,11 @@
       </c>
       <c r="R62" s="83" t="inlineStr">
         <is>
-          <t>★ CURRENT SUPPLIER — LEAF FAT ONLY; cannot do organs (client-stated 2026-08-17). VERIFIED 2026-08-17: the leaf-fat program is itself the proof point — the plant already segregates a per-head by-product for us at line speed, so organs at the viscera table are the ADJACENT operation, not a new concept. THE WEDGE: pitch a paid, CLIENT-CREWED viscera-table pilot (Model A — our crew, zero plant labor, zero new SKUs, zero line-speed impact; organs currently leave at rendering value) to GM Cory Johnson / Plant Mgr Rickie Purnell now, and time the big-volume ask for AFTER the wastewater Phase I/II upgrades land (~2027) — organ/gut-room handling is precisely the high-BOD activity the $3.27M project must reduce, so expect 'no organs' to harden until then. LEVERAGE MOMENT: Villari won the single largest NCAMPI award of the 2026-07-07 round — $800,000 for meat processing — and county support cites 1,000 existing + 75 new jobs; a revenue-from-byproduct pitch lands well while they invest. SIZE OF THE PRIZE: at ~1,500 hd/day this is the ONLY current supplier whose scale could cover the entire organ need from a low-single-digit share of the kill. GATE any deepening on the humane record: same egregious failure mode twice (2022, 2025) — a third event could suspend slaughter mid-program; re-check when the Q3/Q4 FY2026 QERs publish.  [2026-08-17 focus-region pass: FSIS MPI + Demographic datasets and NCDA&amp;CS directories (dated 2026-08-10) retrieved fresh 2026-08-17; adversarially verified.]</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="219.4" customHeight="1" s="59">
+          <t>★ CURRENT SUPPLIER — LEAF FAT ONLY, and the tissue gate is HARD (client-corrected 2026-09-03; supersedes the 2026-08-17 'negotiable wedge' framing — plan NO organ volume through Villari). What stays true and useful: the leaf-fat program itself (they segregate a per-head by-product for us at line speed, reliably, at industrial scale); keep it flowing. BACKGROUND ONLY (if they ever reopen the topic): no regulatory blocker exists — M20608 is federally inspected; no third party holds the viscera (renders out, inferred outlet Darling Rose Hill ~10 mi); the $3.27M wastewater pre-treatment project (county loan 3/2026, friction with Warsaw) runs to ~2027 and made new offal handling unattractive; $800K NCAMPI award 7/7/2026. Humane record: same egregious bleed-rail failure mode twice (suspension 2022; NOIE 5/6/2025 deferred 5/15) — clean through Mar 2026, Apr 2026+ unverified until later QERs. GM Cory Johnson / Plant Mgr Rickie Purnell / CEO Joe Villari.  [Client correction 2026-09-03.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="125.6" customHeight="1" s="59">
       <c r="A63" s="82" t="inlineStr">
         <is>
           <t>Parks Family Meats, LLC</t>
@@ -13550,7 +13550,8 @@
       </c>
       <c r="L63" s="83" t="inlineStr">
         <is>
-          <t>STRONG — 20 staff, single 15,000 sq ft floor, one decision-maker</t>
+          <t>Their floor hosts THEIR crew —
+see Model B column (B-T live)</t>
         </is>
       </c>
       <c r="M63" s="109" t="inlineStr">
@@ -13560,7 +13561,9 @@
       </c>
       <c r="N63" s="83" t="inlineStr">
         <is>
-          <t>Only if juvenile tissue acceptable</t>
+          <t>★ MODEL B-T LIVE — THEIR people
+harvest, trained by US
+(client-corrected 2026-09-03)</t>
         </is>
       </c>
       <c r="O63" s="83" t="inlineStr">
@@ -13584,7 +13587,7 @@
       </c>
       <c r="R63" s="83" t="inlineStr">
         <is>
-          <t>★ CURRENT SUPPLIER — small, focuses on barbecue pigs, works at low quantities, a bit expensive (client-stated 2026-08-17; a third-party review independently calls pricing 'a little expensive'). VERIFIED 2026-08-17: PARKS IS STRUCTURALLY BIGGER THAN OUR MENTAL MODEL. It is one unit of THE PARKS COMPANIES — 29 facilities in 11 states + 2 Canadian provinces, with its own livestock-marketing arm and trucking fleet. The Warsaw floor is slaughter-only (the exact Model A shape), flagged for BOTH market hogs AND roasters, stated 400/day capacity that cat-3 actuals confirm is not fully used, clean in every checkable enforcement quarter FY2024-FY2026Q2. READ: the 'small, expensive, barbecue-pig' experience is most plausibly a PRICING-AND-PRIORITY ARTIFACT of small spot lots of a premium roaster product — not a structural ceiling. THE PLAY: (1) ask Kevin Krum — newly COO, formerly the plant's own contact — what share of the week is market-weight and whether a contracted client kill day (our crew on-site) can be scheduled; (2) convert spot pricing to PROGRAM pricing against committed weekly volume; (3) the unique lever: use the parent as a PROCUREMENT ARM — they can source market hogs to our spec across 11 states and truck them to their own floor, a supply+harvest bundle nobody else in the base offers. If Krum won't sell a dedicated market-hog window, Parks stays what it is today. NOTE: plant contacts changed — Krum + Albino Cardoso now run the floor; Maxwell is corporate sales in Danville IL.  [2026-08-17 focus-region pass: FSIS MPI + Demographic datasets and NCDA&amp;CS directories (dated 2026-08-10) retrieved fresh 2026-08-17; adversarially verified.]</t>
+          <t>★ CURRENT SUPPLIER — OPERATING MODEL CORRECTED 2026-09-03: Parks harvests with THEIR OWN PEOPLE under OUR TRAINING (Model B-T) — the working template for supervised-harvest partnerships; we do not put our own techs on this floor. Still true (client + 3rd-party): small lots, roaster focus, 'a bit expensive' — most plausibly spot pricing on a premium niche, not a structural ceiling. VERIFIED 2026-08-17: slaughter-only floor, market + roaster flags, stated 400/day capacity not fully used, clean every checkable enforcement quarter; parent THE PARKS COMPANIES (29 facilities, 11 states, own trucking) can source hogs to spec and truck them in. THE PLAY: ask COO Kevin Krum ((910) 290-0075) for PROGRAM pricing on a committed market-hog window harvested by their trained crew, and use the parent as a procurement arm. Their crew's training is OUR asset — protect it in any renegotiation.  [Client correction 2026-09-03.]</t>
         </is>
       </c>
     </row>
@@ -19102,7 +19105,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="112.2" customHeight="1" s="59">
+    <row r="9" ht="139" customHeight="1" s="59">
       <c r="A9" s="153" t="inlineStr">
         <is>
           <t>PARKS FAMILY MEATS
@@ -19112,7 +19115,7 @@
       </c>
       <c r="B9" s="154" t="inlineStr">
         <is>
-          <t>Small; barbecue pigs; low quantities; a bit expensive. (Client-stated; 3rd-party review echoes 'a little expensive'.)</t>
+          <t>THEIR people harvest, trained by US — Model B-T live (client-corrected 2026-09-03). Small lots; roaster focus; 'a bit expensive' (3rd-party review agrees).</t>
         </is>
       </c>
       <c r="C9" s="154" t="inlineStr">
@@ -19137,11 +19140,11 @@
       </c>
       <c r="G9" s="154" t="inlineStr">
         <is>
-          <t>'Small and expensive' is most plausibly SPOT PRICING on a premium roaster niche, not a ceiling. Ask Krum: market-weight share of the week + a contracted client kill day at PROGRAM pricing. Unique lever: the parent can SOURCE hogs to our spec across 11 states and truck them to its own floor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="125.6" customHeight="1" s="59">
+          <t>'Small and expensive' is most plausibly SPOT PRICING on a premium roaster niche, not a ceiling. Ask Krum for PROGRAM pricing on a committed market-hog window harvested by their trained crew (B-T); use the parent to source hogs to our spec across 11 states. Their trained crew is our asset — protect it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="112.2" customHeight="1" s="59">
       <c r="A10" s="153" t="inlineStr">
         <is>
           <t>VILLARI / THE PORK CO.
@@ -19151,12 +19154,12 @@
       </c>
       <c r="B10" s="154" t="inlineStr">
         <is>
-          <t>LEAF FAT ONLY — 'they can't do organs.' (Client-stated.)</t>
+          <t>LEAF FAT ONLY — the tissue gate is HARD (client-corrected 2026-09-03). No organ planning through Villari.</t>
         </is>
       </c>
       <c r="C10" s="154" t="inlineStr">
         <is>
-          <t>'No organs' is NEGOTIABLE BUT HARD NEAR-TERM: no regulatory/contractual blocker, no third party holds the viscera (goes to rendering; Darling Rose Hill ~10 mi inferred). Real obstacle = the WASTEWATER crisis: $3.27M pre-treatment project, county loan 3/2026, friction with Warsaw.</t>
+          <t>HARD GATE confirmed by the client 2026-09-03 — supersedes the research 'negotiable wedge' reading. Background if THEY ever reopen it: no regulatory blocker; viscera render out; $3.27M wastewater project to ~2027; $800K NCAMPI award 7/7/2026.</t>
         </is>
       </c>
       <c r="D10" s="154" t="inlineStr">
@@ -19176,7 +19179,7 @@
       </c>
       <c r="G10" s="154" t="inlineStr">
         <is>
-          <t>THE WEDGE: paid, client-crewed viscera-table pilot NOW (our crew, zero plant labor — leaf-fat segregation already proves per-head diversion works here); big-volume ask AFTER wastewater Phase I/II lands (~2027).</t>
+          <t>Keep leaf fat flowing; do NOT pitch organs. Revisit only if Villari reopens the topic (earliest realistically after the wastewater project lands, ~2027). Gate any deepening on the humane record (Q3/Q4 FY2026 QERs).</t>
         </is>
       </c>
     </row>
@@ -19197,7 +19200,7 @@
     <row r="13" ht="45.2" customHeight="1" s="59">
       <c r="A13" s="157" t="inlineStr">
         <is>
-          <t>ORGANS AT VOLUME, WITH LOW FRICTION. Villari has the volume but no organs (until the wedge lands); Martin's has the volume but the friction; Nahunta has the quality but a ~150/day ceiling; Parks and CQP work but are small and priced as spot business. Everything below is judged against that gap. One structural fact frames it all (adversarially confirmed): ALL THREE cat-3 market-hog floors in NC/SC/VA are already in this base — growth comes from working the base better and from sow-class / state-inspected / cluster plays, not from finding a new Martin's.</t>
+          <t>ORGANS AT VOLUME, WITH LOW FRICTION. Villari has the volume but a HARD tissue gate (client-corrected 2026-09-03 — no organ path); Martin's has the volume but the friction; Nahunta has the quality but a ~150/day ceiling; Parks and CQP work but are small and priced as spot business. Everything below is judged against that gap. One structural fact frames it all (adversarially confirmed): ALL THREE cat-3 market-hog floors in NC/SC/VA are already in this base — growth comes from working the base better and from sow-class / state-inspected / cluster plays, not from finding a new Martin's.</t>
         </is>
       </c>
       <c r="B13" s="171" t="n"/>
@@ -19719,7 +19722,7 @@
     <row r="34" ht="72" customHeight="1" s="59">
       <c r="A34" s="168" t="inlineStr">
         <is>
-          <t>THE SEQUENCED MOVES — (1) CALL LARRY'S: the single best structural organ add; gate on the sow-vs-market-hog spec decision (Anatomical Spec tab — still the #1 internal action). (2) CALL THE I-95 STATE PAIR (McLamb's Benson + Gale McLamb Dunn): two Nahunta-playbook floors at 37-44 mi nobody has ever worked. (3) BUY A DEDICATED CQP KILL DAY and pilot Bass + Flowers as the Sims cluster (one crew, three floors) — after the CQP welfare audit. (4) PITCH THE VILLARI VISCERA-TABLE PILOT to Johnson/Purnell while the $800K NCAMPI award is warm; big-volume ask ~2027 post-wastewater. (5) RESET MARTIN'S WITH BETH HOLMES on economics (bench fee + per-head; optionally fund a harvest bay for a multi-year agreement) — it is irreplaceable and clean on paper. (6) ASK KRUM AT PARKS for program pricing on a contracted market-hog window + parent-company hog sourcing to spec. (7) PIEDMONT MODEL A PILOT as the EU-facing welfare showcase (116 mi, borderline inside the radius). West beyond Piedmont: park until a western crew exists.</t>
+          <t>THE SEQUENCED MOVES — (1) CALL LARRY'S: the single best structural organ add; gate on the sow-vs-market-hog spec decision (Anatomical Spec tab — still the #1 internal action). (2) CALL THE I-95 STATE PAIR (McLamb's Benson + Gale McLamb Dunn): two Nahunta-playbook floors at 37-44 mi nobody has ever worked. (3) BUY A DEDICATED CQP KILL DAY and pilot Bass + Flowers as the Sims cluster (one crew, three floors) — after the CQP welfare audit. (4) VILLARI: keep leaf fat flowing and do NOT pitch organs — the gate is hard (client, 2026-09-03); revisit only if they reopen it (~2027 at the earliest). (5) RESET MARTIN'S WITH BETH HOLMES on economics (bench fee + per-head; optionally fund a harvest bay for a multi-year agreement) — it is irreplaceable and clean on paper. (6) ASK KRUM AT PARKS for program pricing on a committed market-hog window harvested by THEIR trained crew (Model B-T — how Parks already works) + parent-company hog sourcing to spec. (7) PIEDMONT MODEL A PILOT as the EU-facing welfare showcase (116 mi, borderline inside the radius). West beyond Piedmont: park until a western crew exists.</t>
         </is>
       </c>
       <c r="B34" s="171" t="n"/>

</xml_diff>

<commit_message>
Fold Beebop v2.1: convergent call order, EcoFriendly as a B-T gate call
Beebop's v2.1 recommendations (commit f9d4dd7) re-rank on evidence of
fit and now match the Rated Candidates order for the first ten.

- Column W carries the v2.1 ranks (Easternview, Cool Springs, Mitchell's
  as follow-ups; Larry's and Bass out on the sow class).
- EcoFriendly restored from Tier 3 to Tier 2 with an explicit gate: a
  Model B-T harvesting-service call, not a volume play (its scores sit
  at Tier-2 level; the NASS demotion over-corrected).
- Call question 2 now asks for weekly hogs IN the 140-220 lb range.
- Legend notes Beebop's radius-vs-road reading; the workbook keeps road
  miles as the Model A screen.
- Sources & Confidence row for v2.1.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvB48tbAk8juvoi9bxkFTf
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
+++ b/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11760" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Overview &amp; Method" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Meeting Notes 2026-08" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Current Base (benchmarks)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Supplier Roster" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rated Candidates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Call Questionnaire" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Visit Agenda" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Anatomical Spec" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TCO Calculator" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Models &amp; Make-vs-Buy" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="APHIS &amp; EU Export" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="National Direct Suppliers" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Sources &amp; Confidence" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview &amp; Method" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meeting Notes 2026-08" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Base (benchmarks)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Roster" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rated Candidates" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call Questionnaire" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visit Agenda" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anatomical Spec" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TCO Calculator" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Models &amp; Make-vs-Buy" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APHIS &amp; EU Export" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="National Direct Suppliers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Confidence" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Supplier Roster'!$A$4:$T$4</definedName>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="58.6" customHeight="1" s="59">
+    <row r="29" ht="98.8" customHeight="1" s="59">
       <c r="A29" s="160" t="inlineStr">
         <is>
           <t>Distance column</t>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B29" s="154" t="inlineStr">
         <is>
-          <t>'YES/NO · ~nn mi' = real ROAD miles from the DURHAM origin (101 City Hall Plaza placeholder; OSRM driving routes, not straight-line) — the figure from the study's earlier Pikeville anchor is kept underneath in parentheses. '≈' = geocoded at city level (±5 mi); no mark = exact street address. YES = inside the 120-mile Model A radius; 'borderline' = 110-130. 'n/m' = not measured (multi-site, out of region, or not a plant).</t>
+          <t>'YES/NO · ~nn mi' = real ROAD miles from the DURHAM origin (101 City Hall Plaza placeholder; OSRM driving routes, not straight-line) — the figure from the study's earlier Pikeville anchor is kept underneath in parentheses. '≈' = geocoded at city level (±5 mi); no mark = exact street address. YES = inside the 120-mile Model A radius; 'borderline' = 110-130. 'n/m' = not measured (multi-site, out of region, or not a plant). NOTE (Beebop v2.1): the ChatGPT brief reads '120 miles' as a RADIUS (straight-line) with road miles as logistics only — under that reading EcoFriendly (92.6 radial) is inside. This workbook keeps ROAD miles as the Model A screen because the crew drives it; radial figures are shown where Beebop supplied them. For Model B-T candidates distance is a sub-score, not a gate.</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" style="59" min="1" max="1"/>
@@ -6071,6 +6071,28 @@
       <c r="D49" s="68" t="inlineStr">
         <is>
           <t>Ladder applied to every roster row: company figure &gt; FSIS band × species flags × HACCP size (MPI directory 'size' field) &gt; NASS state caps &gt; business-type class for NC state plants &gt; FOIA / NCDA / the call. Effects: EcoFriendly and Williamsburg drop to Tier 3 (VOL 5→2, 4→2); federal rows now show HACCP size; the eight NC state rows carry a class-based range instead of 'unknown'. Checked and found empty: CEFS/NC Choices processor directories (services only, no capacity), NMPAN profiles (Acre Station only: 80 hogs/day capacity), plant websites (no throughput statements), NC DEQ permits (not indexed by throughput).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="125.6" customHeight="1" s="59">
+      <c r="A50" s="138" t="inlineStr">
+        <is>
+          <t>Beebop v2.1 (2026-09-28, commit f9d4dd7)</t>
+        </is>
+      </c>
+      <c r="B50" s="68" t="inlineStr">
+        <is>
+          <t>Beebop/round2-2026-09-28/RECOMMENDATIONS_FOR_ROCKSTEADY.md + updated cross-reference workbook (26 fact reviews)</t>
+        </is>
+      </c>
+      <c r="C50" s="46" t="inlineStr">
+        <is>
+          <t>High (convergent)</t>
+        </is>
+      </c>
+      <c r="D50" s="68" t="inlineStr">
+        <is>
+          <t>Beebop re-ranked on evidence of fit after reviewing commits a403954 and 1cb841f; its first ten now match this tab's order exactly (Piedmont, McLamb's, Gale McLamb, EcoFriendly, Flowers, Select, Key Packing, Quaqua, Farmington, Contentnea), with Easternview and Cool Springs as follow-ups. It independently confirmed the NASS state totals against the official text file. ADOPTED: EcoFriendly back to Tier 2 as a Model B-T harvesting-service call with a gate; its sharper opening question (hogs per week IN the 140-220 lb range) folded into call question 2; the radius-vs-road distinction noted in the legend; the complementary-pick idea noted on Rated Candidates. KEPT: road miles as the Model A screen. Two agents working from the same primary data now agree on the call order — that agreement is the useful output of this round.</t>
         </is>
       </c>
     </row>
@@ -20610,10 +20632,10 @@
       <c r="V1" s="171" t="n"/>
       <c r="W1" s="172" t="n"/>
     </row>
-    <row r="2" ht="18.4" customHeight="1" s="59">
+    <row r="2" ht="31.8" customHeight="1" s="59">
       <c r="A2" s="180" t="inlineStr">
         <is>
-          <t>Codes, scoring definitions and weights: see the INSTRUCTIONS tab (sections 5-6). Yellow weight cells below are editable; scores recompute on open. 2026-09-28: PROX measured from the DURHAM origin, ANAT against the 140-220 lb target; column W shows the Beebop (ChatGPT) round-2 call rank for comparison.</t>
+          <t>Codes, scoring definitions and weights: see the INSTRUCTIONS tab (sections 5-6). Yellow weight cells below are editable; scores recompute on open. 2026-09-28: PROX measured from the DURHAM origin, ANAT against the 140-220 lb target; column W shows Beebop's v2.1 call rank — it now matches this tab's order for the first ten. Beebop's complementary-pick idea for step 1: if Purchasing picks the local Tier-1 trio (Piedmont, McLamb's, Gale), the Supplier Engineer picks the different-model / different-region set (EcoFriendly, Select, Farmington).</t>
         </is>
       </c>
       <c r="B2" s="171" t="n"/>
@@ -20815,7 +20837,7 @@
       <c r="W5" s="152" t="inlineStr">
         <is>
           <t>Beebop rank
-(round 2, 9-28)</t>
+(v2.1, 9-28)</t>
         </is>
       </c>
     </row>
@@ -20919,7 +20941,7 @@
       </c>
       <c r="W6" s="198" t="inlineStr">
         <is>
-          <t>— (r1 #19)</t>
+          <t>— (sow)</t>
         </is>
       </c>
     </row>
@@ -21123,7 +21145,7 @@
         </is>
       </c>
       <c r="W8" s="198" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" ht="219.4" customHeight="1" s="59">
@@ -21325,7 +21347,7 @@
         </is>
       </c>
       <c r="W10" s="199" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" ht="58.6" customHeight="1" s="59">
@@ -21531,7 +21553,7 @@
       </c>
       <c r="W12" s="199" t="inlineStr">
         <is>
-          <t>— (r1 #16)</t>
+          <t>— (sow)</t>
         </is>
       </c>
     </row>
@@ -21737,7 +21759,7 @@
         </is>
       </c>
       <c r="W14" s="200" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" ht="125.6" customHeight="1" s="59">
@@ -21837,10 +21859,8 @@
 The western sleeper — one phone call resolves it, but at 190 mi it needs a western crew or Model B-T to matter. (704) 202-9340 / (704) 933-7550.</t>
         </is>
       </c>
-      <c r="W15" s="200" t="inlineStr">
-        <is>
-          <t>— (r1 #17)</t>
-        </is>
+      <c r="W15" s="200" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="16" ht="72" customHeight="1" s="59">
@@ -22146,7 +22166,7 @@
         </is>
       </c>
       <c r="W18" s="200" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" ht="112.2" customHeight="1" s="59">
@@ -22444,7 +22464,7 @@
       </c>
       <c r="V21" s="154" t="n"/>
       <c r="W21" s="200" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" ht="45.2" customHeight="1" s="59">
@@ -22538,8 +22558,10 @@
         </is>
       </c>
       <c r="V22" s="154" t="n"/>
-      <c r="W22" s="200" t="n">
-        <v>10</v>
+      <c r="W22" s="200" t="inlineStr">
+        <is>
+          <t>follow-up</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="58.6" customHeight="1" s="59">
@@ -22635,11 +22657,11 @@
       <c r="V23" s="154" t="n"/>
       <c r="W23" s="200" t="inlineStr">
         <is>
-          <t>— (r1 #9; dropped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="206" customHeight="1" s="59">
+          <t>follow-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="250" customHeight="1" s="59">
       <c r="A24" s="153" t="inlineStr">
         <is>
           <t>EcoFriendly Foods, LLC
@@ -22724,20 +22746,18 @@
         <f>ROUND(SUMPRODUCT($K$4:$R$4,K24:R24),1)</f>
         <v/>
       </c>
-      <c r="U24" s="188" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="U24" s="187" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="V24" s="154" t="inlineStr">
         <is>
-          <t>9-28 VOLUME: Tier 2 → 3. NASS 2025 shows Virginia's 16 federal plants killed 7,841 hogs all year; the cat-3 band here is poultry-driven. Welfare-branded pilot candidate, not a volume lane. 9-28 r2: exact-address routing puts it at 120.4 road / 92.6 radial miles — a boundary case; PROX held at 4 pending the real departure point. 9-28 NEW ON THE SHORTLIST: the Durham origin brings it to ~112 road miles (city-level estimate — it was 198 from Pikeville). Cat 3 with all four hog classes and Certified Humane branding; Tier 2 with one gate — is it operating today, and is the real departure point Durham? Model B-T fits best at this distance.</t>
-        </is>
-      </c>
-      <c r="W24" s="200" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>9-28 v2.1: Tier 3 → 2, with a GATE. Beebop's point stands — this is a Model B-T harvesting-service call, not a volume play; its A/B scores (3.6 / 3.5) sit at Tier-2 level and parking it contradicted them. Gate on the call: is it operating today, and how many hogs in the 140-220 lb range per week (expect tens, not hundreds — Virginia's whole federal total is 7,841/yr). 9-28 VOLUME: Tier 2 → 3. NASS 2025 shows Virginia's 16 federal plants killed 7,841 hogs all year; the cat-3 band here is poultry-driven. Welfare-branded pilot candidate, not a volume lane. 9-28 r2: exact-address routing puts it at 120.4 road / 92.6 radial miles — a boundary case; PROX held at 4 pending the real departure point. 9-28 NEW ON THE SHORTLIST: the Durham origin brings it to ~112 road miles (city-level estimate — it was 198 from Pikeville). Cat 3 with all four hog classes and Certified Humane branding; Tier 2 with one gate — is it operating today, and is the real departure point Durham? Model B-T fits best at this distance.</t>
+        </is>
+      </c>
+      <c r="W24" s="200" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="25" ht="45.2" customHeight="1" s="59">
@@ -22832,7 +22852,7 @@
       </c>
       <c r="V25" s="154" t="n"/>
       <c r="W25" s="200" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" ht="45.2" customHeight="1" s="59">
@@ -22926,8 +22946,10 @@
         </is>
       </c>
       <c r="V26" s="154" t="n"/>
-      <c r="W26" s="200" t="n">
-        <v>6</v>
+      <c r="W26" s="200" t="inlineStr">
+        <is>
+          <t>follow-up</t>
+        </is>
       </c>
     </row>
     <row r="27" ht="45.2" customHeight="1" s="59">
@@ -23122,13 +23144,13 @@
       </c>
       <c r="C7" s="191" t="n"/>
     </row>
-    <row r="8" ht="18.4" customHeight="1" s="59">
+    <row r="8" ht="31.8" customHeight="1" s="59">
       <c r="A8" s="193" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="154" t="inlineStr">
         <is>
-          <t>How many pigs do you kill in a WEEK? (which days; steady or seasonal?)</t>
+          <t>How many pigs do you kill in a WEEK — and how many of those are in the 140-220 lb live range? (which days; steady or seasonal?)</t>
         </is>
       </c>
       <c r="C8" s="191" t="n"/>

</xml_diff>

<commit_message>
Apply the boar/stag rule; keep the owner's final plan slide
- Client rule (2026-09-28): avoid plants that also kill boars/stags - no
  mixing with our hogs. Implemented as gate G4 (soft; the call can clear
  a plant if boars/stags never run with our hogs), an ANAT cap of 2, a
  visible flag on the roster class column, and call question 1 asking
  about boars/stags. Flagged in reach: Piedmont, Flowers, Contentnea,
  EcoFriendly, Mitchell's, Wilkes, Williamsburg, Easternview, Butcher's
  Block; incumbents Martin's and Villari carry the flag too.
- Tiers: Piedmont 1->2, EcoFriendly 2->3, flagged others 3; Select Meats
  (market-only flags) 2->1. State plants marked "ask".
- Tissue_Supplier_Qualification_Plan.pptx is the owner's final slide;
  the earlier Supplier_Qualification_Plan.pptx is removed. README updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvB48tbAk8juvoi9bxkFTf
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
+++ b/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
@@ -1762,7 +1762,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="58.6" customHeight="1" s="59">
+    <row r="16" ht="98.8" customHeight="1" s="59">
       <c r="A16" s="160" t="inlineStr">
         <is>
           <t>Hard gates (pass/fail)</t>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="B16" s="154" t="inlineStr">
         <is>
-          <t>G1 INSPECTION: USDA federal grant (M / Talmadge-Aiken) or NORTH CAROLINA state grant (P-number) = fully eligible — NC state is APHIS-accepted as equivalent for material WE harvest and assemble at ATM. SC/VA/TN state programmes are NOT accepted → domestic lane only. Custom-exempt = ineligible, full stop.  ·  G2 OPERATING: verified operating on primary data as of the date in the row.  ·  G3 SWINE: actually kills hogs per USDA species flags or state species code.</t>
+          <t>G1 INSPECTION: USDA federal grant (M / Talmadge-Aiken) or NORTH CAROLINA state grant (P-number) = fully eligible — NC state is APHIS-accepted as equivalent for material WE harvest and assemble at ATM. SC/VA/TN state programmes are NOT accepted → domestic lane only. Custom-exempt = ineligible, full stop.  ·  G2 OPERATING: verified operating on primary data as of the date in the row.  ·  G3 SWINE: actually kills hogs per USDA species flags or state species code.  ·  G4 BOAR / STAG (client rule, 2026-09-28): plants whose FSIS species flags include boar/stag slaughter are AVOIDED — we do not want boars mixed with our hogs. Soft gate: the call can clear a plant if boars/stags are never run with our designated hogs (separate days or lines). State plants: the NCDA species code (C = swine) does not distinguish boars — ask. Note that two incumbents (Martin's, Villari) carry the flag; confirm current practice there.</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="B23" s="154" t="inlineStr">
         <is>
-          <t>PROX proximity — road miles from the DURHAM origin (5 ≤60 · 4 ≤120 · 2 ≤160 · 1 beyond; boundary cases within ±5 mi of 120 scored 4 pending the confirmed origin) · ACCESS how hostable the floor is for OUR techs · CREW their crew's ability to harvest to spec under our training · ANAT anatomy match against the 140-220 lb live-weight target (5 market/light hogs · 4 market flag, confirm a lighter pull · 3 mixed or unknown class · 1 sow-only, 400+ lb) · VOL volume standing (5 = federal band cat 3+ · 3 = cat 2 · 1 = cat 1/unknown-small — kept on USDA bands so it stays source-verifiable) · WELF welfare &amp; enforcement (5 clean · 3 historic-resolved · 1 repeat/recent) · EXPORT path (5 = federal or NC state · 2 = domestic-only) · RELN approachability (named decision-maker, family culture, warm path in).</t>
+          <t>PROX proximity — road miles from the DURHAM origin (5 ≤60 · 4 ≤120 · 2 ≤160 · 1 beyond; boundary cases within ±5 mi of 120 scored 4 pending the confirmed origin) · ACCESS how hostable the floor is for OUR techs · CREW their crew's ability to harvest to spec under our training · ANAT anatomy match against the 140-220 lb live-weight target (5 market/light hogs · 4 market flag, confirm a lighter pull · 3 mixed or unknown class · 1 sow-only, 400+ lb; CAPPED AT 2 where boar/stag slaughter is flagged — gate G4) · VOL volume standing (5 = federal band cat 3+ · 3 = cat 2 · 1 = cat 1/unknown-small — kept on USDA bands so it stays source-verifiable) · WELF welfare &amp; enforcement (5 clean · 3 historic-resolved · 1 repeat/recent) · EXPORT path (5 = federal or NC state · 2 = domestic-only) · RELN approachability (named decision-maker, family culture, warm path in).</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="45.2" customHeight="1" s="59">
+    <row r="31" ht="58.6" customHeight="1" s="59">
       <c r="A31" s="160" t="inlineStr">
         <is>
           <t>Animal class column</t>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B31" s="154" t="inlineStr">
         <is>
-          <t>USDA's own species flags: MARKET = market-weight butcher hogs (~230-290 lb — the standard for most blocks) · SOW = cull breeding females (mature anatomy; internal spec decision pending) · ROASTER = juvenile pigs · BOAR/STAG = intact/castrated males · 'NO SWINE FLAGS' = hog slaughter unsupported by the primary data — confirm species before calling.</t>
+          <t>USDA's own species flags: MARKET = market-weight butcher hogs (~230-290 lb — the standard for most blocks) · SOW = cull breeding females (mature anatomy; internal spec decision pending) · ROASTER = juvenile pigs · BOAR/STAG = intact/castrated males — '⚠ BOAR/STAG flagged' marks plants the client avoids (gate G4) · 'NO SWINE FLAGS' = hog slaughter unsupported by the primary data — confirm species before calling.</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" style="59" min="1" max="1"/>
@@ -6093,6 +6093,28 @@
       <c r="D50" s="68" t="inlineStr">
         <is>
           <t>Beebop re-ranked on evidence of fit after reviewing commits a403954 and 1cb841f; its first ten now match this tab's order exactly (Piedmont, McLamb's, Gale McLamb, EcoFriendly, Flowers, Select, Key Packing, Quaqua, Farmington, Contentnea), with Easternview and Cool Springs as follow-ups. It independently confirmed the NASS state totals against the official text file. ADOPTED: EcoFriendly back to Tier 2 as a Model B-T harvesting-service call with a gate; its sharper opening question (hogs per week IN the 140-220 lb range) folded into call question 2; the radius-vs-road distinction noted in the legend; the complementary-pick idea noted on Rated Candidates. KEPT: road miles as the Model A screen. Two agents working from the same primary data now agree on the call order — that agreement is the useful output of this round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="165.8" customHeight="1" s="59">
+      <c r="A51" s="138" t="inlineStr">
+        <is>
+          <t>Boar / stag rule (client, 2026-09-28)</t>
+        </is>
+      </c>
+      <c r="B51" s="68" t="inlineStr">
+        <is>
+          <t>FSIS Establishment Demographic Data, boar_stag_swine_slaughter flag (pull 2026-09-03); NCDA directory species codes (no boar distinction)</t>
+        </is>
+      </c>
+      <c r="C51" s="46" t="inlineStr">
+        <is>
+          <t>High (flag) / Ask (state plants)</t>
+        </is>
+      </c>
+      <c r="D51" s="68" t="inlineStr">
+        <is>
+          <t>The client does not want boars/stags mixed with our hogs. Flagged in NC/SC/VA/TN: Martin's Pork Products, Inc., Piedmont Custom Meats, Wayne Mays Meat Processing, M.L. Mitchell &amp; Son, Wilkes Abattoir, LLC dba Apple Bra, Wells, Jenkins &amp; Wells Abattoir, Williamsburg Packing Company, Inc., Fayette Packing Co., Inc., EcoFriendly Foods, LLC, T&amp;E Meats (True &amp; Essential), Blue Ridge Meats of Front Royal, The Pork Company (Villari Food Gro, Contentnea Farms, LLC, Flowers Slaughter House (George Fl, Fauquier's Finest — DATA ANOMALY, Easternview Farms LLC, The Butcher's Block. Effects: '⚠ BOAR/STAG flagged' on the roster class column; STRONG FIT / POSSIBLE → CAUTION for flagged non-incumbents; ANAT capped at 2 on Rated Candidates; Piedmont Tier 1 → 2, Flowers stays 2, EcoFriendly 2 → 3, the rest 3; Select Meats (market-only flags) Tier 2 → 1. The flag means the plant slaughtered boars/stags in the data period, not that they share a day with market hogs — hence a SOFT gate cleared by the call (question 1 now asks). Two incumbents carry the flag (Martin's, Villari): mixing already occurs at a plant we harvest at, so 'separate days' is the practical standard.</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7430,8 @@
       </c>
       <c r="G7" s="134" t="inlineStr">
         <is>
-          <t>MARKET HOG + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET HOG + boar/stag
 (sow: No)</t>
         </is>
       </c>
@@ -7464,7 +7487,8 @@
       </c>
       <c r="Q7" s="178" t="inlineStr">
         <is>
-          <t>CURRENT — Model A volume anchor: the only cat-3 market-hog floor we run crews on; clean record; irreplaceable in NC/SC/VA. Friction is relational — reset with Beth Holmes.</t>
+          <t>BOAR/STAG RULE 9-28 (incumbent): FSIS flags boar/stag slaughter here — the client does not want boars mixed with our hogs; confirm current practice (separate days / never with our designated hogs).
+CURRENT — Model A volume anchor: the only cat-3 market-hog floor we run crews on; clean record; irreplaceable in NC/SC/VA. Friction is relational — reset with Beth Holmes.</t>
         </is>
       </c>
       <c r="R7" s="179" t="inlineStr">
@@ -7530,7 +7554,8 @@
       </c>
       <c r="G9" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + ROASTER + boar/stag
 (M7975, Gibsonville)</t>
         </is>
       </c>
@@ -7578,14 +7603,15 @@
 piedmontcustommeats.com</t>
         </is>
       </c>
-      <c r="P9" s="20" t="inlineStr">
-        <is>
-          <t>STRONG FIT</t>
+      <c r="P9" s="23" t="inlineStr">
+        <is>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q9" s="178" t="inlineStr">
         <is>
-          <t>★ TIER 1 — best host structure + best welfare story (AWA / Temple Grandin), all four hog classes, inside the radius at 116 mi. Their disposal fee suggests viscera are discarded today — confirm which organs, and who owns them. Cat-2 ceiling.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). ★ TIER 1 — best host structure + best welfare story (AWA / Temple Grandin), all four hog classes, inside the radius at 116 mi. Their disposal fee suggests viscera are discarded today — confirm which organs, and who owns them. Cat-2 ceiling.</t>
         </is>
       </c>
       <c r="R9" s="179" t="inlineStr">
@@ -7939,7 +7965,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="58.6" customHeight="1" s="59">
+    <row r="13" ht="72" customHeight="1" s="59">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Wayne Mays Meat Processing</t>
@@ -7975,7 +8001,8 @@
       </c>
       <c r="G13" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + boar/stag</t>
         </is>
       </c>
       <c r="H13" s="68" t="inlineStr">
@@ -8026,7 +8053,7 @@
       </c>
       <c r="Q13" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R13" s="179" t="inlineStr">
@@ -8083,7 +8110,8 @@
       </c>
       <c r="G14" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + boar/stag</t>
         </is>
       </c>
       <c r="H14" s="68" t="inlineStr">
@@ -8134,7 +8162,7 @@
       </c>
       <c r="Q14" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R14" s="179" t="inlineStr">
@@ -8407,7 +8435,8 @@
       </c>
       <c r="G17" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + boar/stag</t>
         </is>
       </c>
       <c r="H17" s="68" t="inlineStr">
@@ -8460,7 +8489,7 @@
       </c>
       <c r="Q17" s="178" t="inlineStr">
         <is>
-          <t>TIER 3 — highest hog share in the west (~half the kill), real cut-to-spec crew; 209 mi and prior-owner welfare history → B-T only.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER 3 — highest hog share in the west (~half the kill), real cut-to-spec crew; 209 mi and prior-owner welfare history → B-T only.</t>
         </is>
       </c>
       <c r="R17" s="179" t="inlineStr">
@@ -8730,7 +8759,8 @@
       </c>
       <c r="G20" s="68" t="inlineStr">
         <is>
-          <t>MARKET + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + boar/stag
 (sow: No, roaster: No)</t>
         </is>
       </c>
@@ -8776,12 +8806,13 @@
       </c>
       <c r="P20" s="23" t="inlineStr">
         <is>
-          <t>POSSIBLE</t>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q20" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R20" s="179" t="inlineStr">
@@ -9936,7 +9967,8 @@
       </c>
       <c r="G33" s="68" t="inlineStr">
         <is>
-          <t>ALL FOUR hog classes
+          <t>⚠ BOAR/STAG flagged (FSIS)
+ALL FOUR hog classes
 (market+sow+roaster+boar/stag,
 FSIS flags 2026-09-03)</t>
         </is>
@@ -9983,14 +10015,15 @@
           <t>(843) 355-6447</t>
         </is>
       </c>
-      <c r="P33" s="140" t="inlineStr">
-        <is>
-          <t>POSSIBLE</t>
+      <c r="P33" s="23" t="inlineStr">
+        <is>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q33" s="178" t="inlineStr">
         <is>
-          <t>TIER 2 — the ONLY non-incumbent cat-3 floor within ~200 mi, now showing all four swine classes. ONE call decides it: actual hogs/week (the cat-3 band is multi-species, so the hog number could disappoint).</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER 2 — the ONLY non-incumbent cat-3 floor within ~200 mi, now showing all four swine classes. ONE call decides it: actual hogs/week (the cat-3 band is multi-species, so the hog number could disappoint).</t>
         </is>
       </c>
       <c r="R33" s="179" t="inlineStr">
@@ -10162,7 +10195,8 @@
       </c>
       <c r="G36" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + ROASTER + boar/stag
 (all four classes)</t>
         </is>
       </c>
@@ -10209,12 +10243,13 @@
       </c>
       <c r="P36" s="23" t="inlineStr">
         <is>
-          <t>POSSIBLE</t>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q36" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R36" s="179" t="inlineStr">
@@ -10592,7 +10627,8 @@
       </c>
       <c r="G41" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + ROASTER + boar/stag
 (all four classes)</t>
         </is>
       </c>
@@ -10637,14 +10673,15 @@
 ecofriendly.com</t>
         </is>
       </c>
-      <c r="P41" s="140" t="inlineStr">
-        <is>
-          <t>POSSIBLE</t>
+      <c r="P41" s="23" t="inlineStr">
+        <is>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q41" s="178" t="inlineStr">
         <is>
-          <t>TIER-2-ADJACENT (VA) — all four hog classes at cat-3 volume, the strongest VA option and welfare-branded; 198 mi → Model B-T only. Site live 2026-09-03 (contradicts the old 'ceased ~2020' rumor again).</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER-2-ADJACENT (VA) — all four hog classes at cat-3 volume, the strongest VA option and welfare-branded; 198 mi → Model B-T only. Site live 2026-09-03 (contradicts the old 'ceased ~2020' rumor again).</t>
         </is>
       </c>
       <c r="R41" s="179" t="inlineStr">
@@ -10702,7 +10739,8 @@
       </c>
       <c r="G42" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + ROASTER + boar/stag
 (all four classes)</t>
         </is>
       </c>
@@ -10748,14 +10786,15 @@
 temeats.com</t>
         </is>
       </c>
-      <c r="P42" s="20" t="inlineStr">
-        <is>
-          <t>STRONG FIT</t>
+      <c r="P42" s="23" t="inlineStr">
+        <is>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q42" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R42" s="179" t="inlineStr">
@@ -10811,7 +10850,8 @@
       </c>
       <c r="G43" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + boar/stag</t>
         </is>
       </c>
       <c r="H43" s="68" t="inlineStr">
@@ -10855,14 +10895,15 @@
 blueridgemeats.com</t>
         </is>
       </c>
-      <c r="P43" s="20" t="inlineStr">
-        <is>
-          <t>STRONG FIT</t>
+      <c r="P43" s="23" t="inlineStr">
+        <is>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q43" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R43" s="179" t="inlineStr">
@@ -12546,7 +12587,8 @@
       </c>
       <c r="G64" s="83" t="inlineStr">
         <is>
-          <t>MARKET + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + boar/stag
 (sow: No, roaster: No)</t>
         </is>
       </c>
@@ -12601,7 +12643,8 @@
       </c>
       <c r="Q64" s="178" t="inlineStr">
         <is>
-          <t>CURRENT — leaf fat ONLY; tissue gate is HARD (client 2026-09-03). Not an organ candidate; keep the leaf-fat lane healthy.</t>
+          <t>BOAR/STAG RULE 9-28 (incumbent): FSIS flags boar/stag slaughter here — the client does not want boars mixed with our hogs; confirm current practice (separate days / never with our designated hogs).
+CURRENT — leaf fat ONLY; tissue gate is HARD (client 2026-09-03). Not an organ candidate; keep the leaf-fat lane healthy.</t>
         </is>
       </c>
       <c r="R64" s="179" t="inlineStr">
@@ -12780,7 +12823,8 @@
       </c>
       <c r="G66" s="68" t="inlineStr">
         <is>
-          <t>Yes — SWINE-ONLY</t>
+          <t>Yes — SWINE-ONLY
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H66" s="68" t="inlineStr">
@@ -12887,7 +12931,8 @@
       </c>
       <c r="G67" s="68" t="inlineStr">
         <is>
-          <t>Yes — SWINE-ONLY</t>
+          <t>Yes — SWINE-ONLY
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H67" s="68" t="inlineStr">
@@ -12995,7 +13040,8 @@
       </c>
       <c r="G68" s="68" t="inlineStr">
         <is>
-          <t>Yes — SWINE-ONLY</t>
+          <t>Yes — SWINE-ONLY
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H68" s="68" t="inlineStr">
@@ -13104,7 +13150,8 @@
       </c>
       <c r="G69" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + boar/stag</t>
         </is>
       </c>
       <c r="H69" s="68" t="inlineStr">
@@ -13151,12 +13198,13 @@
       </c>
       <c r="P69" s="23" t="inlineStr">
         <is>
-          <t>POSSIBLE</t>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q69" s="178" t="inlineStr">
         <is>
-          <t>TIER 3 — closest plant on the list (35 mi) but &lt;19/wk; overflow/pilot for odd-lot sow or boar needs.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER 3 — closest plant on the list (35 mi) but &lt;19/wk; overflow/pilot for odd-lot sow or boar needs.</t>
         </is>
       </c>
       <c r="R69" s="179" t="inlineStr">
@@ -13423,7 +13471,8 @@
       </c>
       <c r="G72" s="68" t="inlineStr">
         <is>
-          <t>MARKET + boar/stag
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + boar/stag
 (sow: No, roaster: No)</t>
         </is>
       </c>
@@ -13473,12 +13522,13 @@
       </c>
       <c r="P72" s="23" t="inlineStr">
         <is>
-          <t>POSSIBLE</t>
+          <t>CAUTION
+(boar/stag)</t>
         </is>
       </c>
       <c r="Q72" s="178" t="inlineStr">
         <is>
-          <t>TIER 2 — Sims cluster redundancy 3 mi from CQP + the region's only boar/stag access. Not a standalone lane (cat 2).</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER 2 — Sims cluster redundancy 3 mi from CQP + the region's only boar/stag access. Not a standalone lane (cat 2).</t>
         </is>
       </c>
       <c r="R72" s="179" t="inlineStr">
@@ -14065,7 +14115,8 @@
       <c r="G79" s="134" t="inlineStr">
         <is>
           <t>Multi-species incl. HOGS
-(state species A,B,C,D,E)</t>
+(state species A,B,C,D,E)
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H79" s="83" t="inlineStr">
@@ -14177,7 +14228,8 @@
       <c r="G80" s="134" t="inlineStr">
         <is>
           <t>Cattle + HOGS
-(state species A,B,C)</t>
+(state species A,B,C)
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H80" s="83" t="inlineStr">
@@ -14617,7 +14669,8 @@
       <c r="G84" s="134" t="inlineStr">
         <is>
           <t>HOGS + goats/sheep
-(state species C, D, E)</t>
+(state species C, D, E)
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H84" s="83" t="inlineStr">
@@ -18358,7 +18411,8 @@
       </c>
       <c r="G126" s="68" t="inlineStr">
         <is>
-          <t>Yes — MKT+SOW+boar+beef</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+Yes — MKT+SOW+boar+beef</t>
         </is>
       </c>
       <c r="H126" s="68" t="inlineStr">
@@ -18409,7 +18463,7 @@
       </c>
       <c r="Q126" s="178" t="inlineStr">
         <is>
-          <t>Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Back-pool — passes no current tier; see Fit and notes for what a call would need to change.</t>
         </is>
       </c>
       <c r="R126" s="179" t="inlineStr">
@@ -18686,7 +18740,8 @@
       <c r="G131" s="68" t="inlineStr">
         <is>
           <t>Calves, cattle, SWINE, sheep, goats
-(NCDA species A,B,C,D,E)</t>
+(NCDA species A,B,C,D,E)
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H131" s="68" t="inlineStr">
@@ -20141,7 +20196,8 @@
       <c r="G145" s="68" t="inlineStr">
         <is>
           <t>Calves, cattle, SWINE, sheep, goats
-(NCDA species A,B,C,D,E)</t>
+(NCDA species A,B,C,D,E)
+(boar/stag: ask — the NCDA species code does not distinguish boars)</t>
         </is>
       </c>
       <c r="H145" s="68" t="inlineStr">
@@ -20247,7 +20303,8 @@
       </c>
       <c r="G146" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag (FSIS flags); custom-exempt slaughter also = Yes</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + boar/stag (FSIS flags); custom-exempt slaughter also = Yes</t>
         </is>
       </c>
       <c r="H146" s="68" t="inlineStr">
@@ -20298,7 +20355,7 @@
       </c>
       <c r="Q146" s="178" t="inlineStr">
         <is>
-          <t>Beebop r2 ranks it #6: the closest Virginia plant to Durham (76 road mi) with its own site describing on-site slaughter and M1908. Verified in the FSIS pull: federal slaughter, cat 1, market + sow flags, plus a V (voluntary/non-amenable) grant — the research-species mechanism. Pilot scale; cheap call.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Beebop r2 ranks it #6: the closest Virginia plant to Durham (76 road mi) with its own site describing on-site slaughter and M1908. Verified in the FSIS pull: federal slaughter, cat 1, market + sow flags, plus a V (voluntary/non-amenable) grant — the research-species mechanism. Pilot scale; cheap call.</t>
         </is>
       </c>
       <c r="R146" s="179" t="inlineStr">
@@ -20353,7 +20410,8 @@
       </c>
       <c r="G147" s="68" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag (all four FSIS classes); custom-exempt also = Yes</t>
+          <t>⚠ BOAR/STAG flagged (FSIS)
+MARKET + SOW + ROASTER + boar/stag (all four FSIS classes); custom-exempt also = Yes</t>
         </is>
       </c>
       <c r="H147" s="68" t="inlineStr">
@@ -20404,7 +20462,7 @@
       </c>
       <c r="Q147" s="178" t="inlineStr">
         <is>
-          <t>Beebop r2 lead: 74 road miles from Durham with all four hog classes flagged in the FSIS pull — but cat 1 (&lt;19 animals/week). Namesake shops elsewhere are different businesses. A one-call scale check.</t>
+          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). Beebop r2 lead: 74 road miles from Durham with all four hog classes flagged in the FSIS pull — but cat 1 (&lt;19 animals/week). Namesake shops elsewhere are different businesses. A one-call scale check.</t>
         </is>
       </c>
       <c r="R147" s="179" t="inlineStr">
@@ -20635,7 +20693,7 @@
     <row r="2" ht="31.8" customHeight="1" s="59">
       <c r="A2" s="180" t="inlineStr">
         <is>
-          <t>Codes, scoring definitions and weights: see the INSTRUCTIONS tab (sections 5-6). Yellow weight cells below are editable; scores recompute on open. 2026-09-28: PROX measured from the DURHAM origin, ANAT against the 140-220 lb target; column W shows Beebop's v2.1 call rank — it now matches this tab's order for the first ten. Beebop's complementary-pick idea for step 1: if Purchasing picks the local Tier-1 trio (Piedmont, McLamb's, Gale), the Supplier Engineer picks the different-model / different-region set (EcoFriendly, Select, Farmington).</t>
+          <t>Codes, scoring definitions and weights: see the INSTRUCTIONS tab (sections 5-6). Yellow weight cells below are editable; scores recompute on open. 2026-09-28: PROX measured from the DURHAM origin, ANAT against the 140-220 lb target and CAPPED AT 2 where FSIS flags boar/stag slaughter (client rule: no mixing) — Piedmont, Flowers and EcoFriendly moved down on that rule; column W shows Beebop's v2.1 call rank (set before the rule).</t>
         </is>
       </c>
       <c r="B2" s="171" t="n"/>
@@ -20971,7 +21029,7 @@
       <c r="E7" s="154" t="inlineStr">
         <is>
           <t>Multi-species incl. hogs
-(state species A,B,C,D,E)</t>
+(state species A,B,C,D,E) — boar/stag: ASK (state code does not distinguish)</t>
         </is>
       </c>
       <c r="F7" s="154" t="inlineStr">
@@ -21047,7 +21105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="45.2" customHeight="1" s="59">
+    <row r="8" ht="58.6" customHeight="1" s="59">
       <c r="A8" s="153" t="inlineStr">
         <is>
           <t>Gale McLamb Meats
@@ -21073,7 +21131,7 @@
       <c r="E8" s="154" t="inlineStr">
         <is>
           <t>Cattle + hogs
-(state species A,B,C)</t>
+(state species A,B,C) — boar/stag: ASK (state code does not distinguish)</t>
         </is>
       </c>
       <c r="F8" s="154" t="inlineStr">
@@ -21148,7 +21206,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="219.4" customHeight="1" s="59">
+    <row r="9" ht="250" customHeight="1" s="59">
       <c r="A9" s="153" t="inlineStr">
         <is>
           <t>Piedmont Custom Meats
@@ -21173,7 +21231,7 @@
       </c>
       <c r="E9" s="154" t="inlineStr">
         <is>
-          <t>ALL FOUR hog classes —
+          <t>⚠ BOAR/STAG flagged — ALL FOUR hog classes —
 only NC plant so flagged</t>
         </is>
       </c>
@@ -21213,7 +21271,7 @@
         <v>4</v>
       </c>
       <c r="N9" s="185" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O9" s="185" t="n">
         <v>3</v>
@@ -21235,14 +21293,14 @@
         <f>ROUND(SUMPRODUCT($K$4:$R$4,K9:R9),1)</f>
         <v/>
       </c>
-      <c r="U9" s="186" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="U9" s="187" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="V9" s="154" t="inlineStr">
         <is>
-          <t>9-28: Beebop's #1 too. New facts — 150 lb live minimum published (fits the target), NC Farm Bureau capacity-expansion grant, and service-processing of customer-owned animals → ask who owns the organs. 48 road mi from Durham.
+          <t>9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 5); tier 2. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. 9-28: Beebop's #1 too. New facts — 150 lb live minimum published (fits the target), NC Farm Bureau capacity-expansion grant, and service-processing of customer-owned animals → ask who owns the organs. 48 road mi from Durham.
 The strongest all-round candidate outside the current base. Limit: cat-2 ceiling (~194/wk all species). ⚠ PROTOCOL QUESTION FOR THE CALL: their FAQ (2026-09-03) says hogs get an electric stun 'and a second time to stop their hearts' (occasionally a rifle for heavy hogs) — ask whether OUR designated hogs can skip the second/cardiac stun to protect thoracic organs and aortas. Scheduling line (336) 628-4949.</t>
         </is>
       </c>
@@ -21250,7 +21308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" ht="58.6" customHeight="1" s="59">
+    <row r="10" ht="139" customHeight="1" s="59">
       <c r="A10" s="153" t="inlineStr">
         <is>
           <t>Flowers Slaughter House
@@ -21275,7 +21333,7 @@
       </c>
       <c r="E10" s="154" t="inlineStr">
         <is>
-          <t>Market + BOAR/STAG
+          <t>⚠ BOAR/STAG flagged — Market + BOAR/STAG
 (largest male anatomy in region)</t>
         </is>
       </c>
@@ -21314,7 +21372,7 @@
         <v>3</v>
       </c>
       <c r="N10" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" s="185" t="n">
         <v>3</v>
@@ -21343,7 +21401,7 @@
       </c>
       <c r="V10" s="154" t="inlineStr">
         <is>
-          <t>Cluster play, not a standalone lane: redundancy for Sims + the region's only boar/stag access. Contacts Alan Sharp / Tim Boswell, (252) 237-2982.</t>
+          <t>9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 2. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. Cluster play, not a standalone lane: redundancy for Sims + the region's only boar/stag access. Contacts Alan Sharp / Tim Boswell, (252) 237-2982.</t>
         </is>
       </c>
       <c r="W10" s="199" t="n">
@@ -21557,7 +21615,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="125.6" customHeight="1" s="59">
+    <row r="13" ht="206" customHeight="1" s="59">
       <c r="A13" s="153" t="inlineStr">
         <is>
           <t>Williamsburg Packing Co.
@@ -21582,7 +21640,7 @@
       </c>
       <c r="E13" s="154" t="inlineStr">
         <is>
-          <t>ALL FOUR hog classes
+          <t>⚠ BOAR/STAG flagged — ALL FOUR hog classes
 (market + sow + roaster + boar/stag —
 fresh FSIS flags 2026-09-03)</t>
         </is>
@@ -21623,7 +21681,7 @@
         <v>3</v>
       </c>
       <c r="N13" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O13" s="185" t="n">
         <v>2</v>
@@ -21652,7 +21710,7 @@
       </c>
       <c r="V13" s="154" t="inlineStr">
         <is>
-          <t>9-28 VOLUME: Tier 2 → 3. NASS 2025: South Carolina's 8 federal plants killed 14,070 hogs all year — the 'only non-incumbent cat-3' was an all-species artifact. ONE call decides it: actual hogs/week (the cat-3 band is a multi-species aggregate, so the hog number could disappoint). If the hog share is real, this is the only outside-the-base volume play in reach — as Model B-T. (843) 355-6447.</t>
+          <t>9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. 9-28 VOLUME: Tier 2 → 3. NASS 2025: South Carolina's 8 federal plants killed 14,070 hogs all year — the 'only non-incumbent cat-3' was an all-species artifact. ONE call decides it: actual hogs/week (the cat-3 band is a multi-species aggregate, so the hog number could disappoint). If the hog share is real, this is the only outside-the-base volume play in reach — as Model B-T. (843) 355-6447.</t>
         </is>
       </c>
       <c r="W13" s="199" t="inlineStr">
@@ -21661,7 +21719,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="98.8" customHeight="1" s="59">
+    <row r="14" ht="179.2" customHeight="1" s="59">
       <c r="A14" s="153" t="inlineStr">
         <is>
           <t>Contentnea Farms
@@ -21687,7 +21745,7 @@
       </c>
       <c r="E14" s="154" t="inlineStr">
         <is>
-          <t>Market + sow + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged — Market + sow + boar/stag</t>
         </is>
       </c>
       <c r="F14" s="154" t="inlineStr">
@@ -21725,7 +21783,7 @@
         <v>3</v>
       </c>
       <c r="N14" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O14" s="185" t="n">
         <v>1</v>
@@ -21754,7 +21812,7 @@
       </c>
       <c r="V14" s="154" t="inlineStr">
         <is>
-          <t>9-28: Beebop ranks it #4 (active booking site, TA-2583) — but its FSIS band is cat 1 (&lt;19/wk): a cheap call, pilot-scale at best. Tier unchanged.
+          <t>9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. 9-28: Beebop ranks it #4 (active booking site, TA-2583) — but its FSIS band is cat 1 (&lt;19/wk): a cheap call, pilot-scale at best. Tier unchanged.
 Closest plant on the list (35 mi) but &lt;19/wk: overflow/pilot for odd-lot sow or boar needs only. (252) 717-9229.</t>
         </is>
       </c>
@@ -21762,7 +21820,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" ht="125.6" customHeight="1" s="59">
+    <row r="15" ht="192.6" customHeight="1" s="59">
       <c r="A15" s="153" t="inlineStr">
         <is>
           <t>Select Meats
@@ -21848,14 +21906,14 @@
         <f>ROUND(SUMPRODUCT($K$4:$R$4,K15:R15),1)</f>
         <v/>
       </c>
-      <c r="U15" s="187" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U15" s="186" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="V15" s="154" t="inlineStr">
         <is>
-          <t>9-28 UPDATE: Tier 3 → 2. From the Durham origin it is ~115 road miles — INSIDE the radius (it was ~190 from Pikeville). Market-only, cat 2, one call resolves it; Beebop ranks it #17 with the same boundary caveat.
+          <t>9-28 BOAR/STAG RULE: Tier 2 → 1. The cleanest class profile in reach — FSIS flags MARKET hogs only (no sow, no roaster, no boar/stag), federal, cat 2, ~115 road mi from Durham. One call resolves volume. 9-28 UPDATE: Tier 3 → 2. From the Durham origin it is ~115 road miles — INSIDE the radius (it was ~190 from Pikeville). Market-only, cat 2, one call resolves it; Beebop ranks it #17 with the same boundary caveat.
 The western sleeper — one phone call resolves it, but at 190 mi it needs a western crew or Model B-T to matter. (704) 202-9340 / (704) 933-7550.</t>
         </is>
       </c>
@@ -21863,7 +21921,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" ht="72" customHeight="1" s="59">
+    <row r="16" ht="125.6" customHeight="1" s="59">
       <c r="A16" s="153" t="inlineStr">
         <is>
           <t>Wilkes Abattoir (Apple Brandy)
@@ -21888,7 +21946,7 @@
       </c>
       <c r="E16" s="154" t="inlineStr">
         <is>
-          <t>Market + sow + boar/stag</t>
+          <t>⚠ BOAR/STAG flagged — Market + sow + boar/stag</t>
         </is>
       </c>
       <c r="F16" s="154" t="inlineStr">
@@ -21927,7 +21985,7 @@
         <v>4</v>
       </c>
       <c r="N16" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O16" s="185" t="n">
         <v>3</v>
@@ -21956,7 +22014,7 @@
       </c>
       <c r="V16" s="154" t="inlineStr">
         <is>
-          <t>Highest confirmed hog share in the west (~half the kill) — but 209 mi. Model B-T only. (336) 667-1346.</t>
+          <t>9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. Highest confirmed hog share in the west (~half the kill) — but 209 mi. Model B-T only. (336) 667-1346.</t>
         </is>
       </c>
       <c r="W16" s="200" t="inlineStr">
@@ -22069,7 +22127,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="45.2" customHeight="1" s="59">
+    <row r="18" ht="58.6" customHeight="1" s="59">
       <c r="A18" s="153" t="inlineStr">
         <is>
           <t>Key Packing Co.
@@ -22095,7 +22153,7 @@
       <c r="E18" s="154" t="inlineStr">
         <is>
           <t>Multi-species incl. hogs
-(A,B,C,D,E)</t>
+(A,B,C,D,E) — boar/stag: ASK (state code does not distinguish)</t>
         </is>
       </c>
       <c r="F18" s="154" t="inlineStr">
@@ -22372,7 +22430,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="45.2" customHeight="1" s="59">
+    <row r="21" ht="72" customHeight="1" s="59">
       <c r="A21" s="153" t="inlineStr">
         <is>
           <t>Quaqua Creek Farm
@@ -22397,7 +22455,7 @@
       </c>
       <c r="E21" s="154" t="inlineStr">
         <is>
-          <t>Species A-E incl. swine (state code C); hog share unknown</t>
+          <t>Species A-E incl. swine (state code C); hog share unknown — boar/stag: ASK (state code does not distinguish)</t>
         </is>
       </c>
       <c r="F21" s="154" t="inlineStr">
@@ -22564,7 +22622,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="58.6" customHeight="1" s="59">
+    <row r="23" ht="85.40000000000001" customHeight="1" s="59">
       <c r="A23" s="153" t="inlineStr">
         <is>
           <t>Mitchell's Butchery (M.L. Mitchell &amp; Son)
@@ -22589,7 +22647,7 @@
       </c>
       <c r="E23" s="154" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag (FSIS)</t>
+          <t>⚠ BOAR/STAG flagged — MARKET + SOW + boar/stag (FSIS)</t>
         </is>
       </c>
       <c r="F23" s="154" t="inlineStr">
@@ -22627,7 +22685,7 @@
         <v>3</v>
       </c>
       <c r="N23" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O23" s="185" t="n">
         <v>1</v>
@@ -22654,7 +22712,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="V23" s="154" t="n"/>
+      <c r="V23" s="154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. </t>
+        </is>
+      </c>
       <c r="W23" s="200" t="inlineStr">
         <is>
           <t>follow-up</t>
@@ -22686,7 +22748,7 @@
       </c>
       <c r="E24" s="154" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag (all four FSIS classes)</t>
+          <t>⚠ BOAR/STAG flagged — MARKET + SOW + ROASTER + boar/stag (all four FSIS classes)</t>
         </is>
       </c>
       <c r="F24" s="154" t="inlineStr">
@@ -22724,7 +22786,7 @@
         <v>3</v>
       </c>
       <c r="N24" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O24" s="185" t="n">
         <v>2</v>
@@ -22746,21 +22808,21 @@
         <f>ROUND(SUMPRODUCT($K$4:$R$4,K24:R24),1)</f>
         <v/>
       </c>
-      <c r="U24" s="187" t="inlineStr">
-        <is>
-          <t>2</t>
+      <c r="U24" s="188" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="V24" s="154" t="inlineStr">
         <is>
-          <t>9-28 v2.1: Tier 3 → 2, with a GATE. Beebop's point stands — this is a Model B-T harvesting-service call, not a volume play; its A/B scores (3.6 / 3.5) sit at Tier-2 level and parking it contradicted them. Gate on the call: is it operating today, and how many hogs in the 140-220 lb range per week (expect tens, not hundreds — Virginia's whole federal total is 7,841/yr). 9-28 VOLUME: Tier 2 → 3. NASS 2025 shows Virginia's 16 federal plants killed 7,841 hogs all year; the cat-3 band here is poultry-driven. Welfare-branded pilot candidate, not a volume lane. 9-28 r2: exact-address routing puts it at 120.4 road / 92.6 radial miles — a boundary case; PROX held at 4 pending the real departure point. 9-28 NEW ON THE SHORTLIST: the Durham origin brings it to ~112 road miles (city-level estimate — it was 198 from Pikeville). Cat 3 with all four hog classes and Certified Humane branding; Tier 2 with one gate — is it operating today, and is the real departure point Durham? Model B-T fits best at this distance.</t>
+          <t>9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. 9-28 v2.1: Tier 3 → 2, with a GATE. Beebop's point stands — this is a Model B-T harvesting-service call, not a volume play; its A/B scores (3.6 / 3.5) sit at Tier-2 level and parking it contradicted them. Gate on the call: is it operating today, and how many hogs in the 140-220 lb range per week (expect tens, not hundreds — Virginia's whole federal total is 7,841/yr). 9-28 VOLUME: Tier 2 → 3. NASS 2025 shows Virginia's 16 federal plants killed 7,841 hogs all year; the cat-3 band here is poultry-driven. Welfare-branded pilot candidate, not a volume lane. 9-28 r2: exact-address routing puts it at 120.4 road / 92.6 radial miles — a boundary case; PROX held at 4 pending the real departure point. 9-28 NEW ON THE SHORTLIST: the Durham origin brings it to ~112 road miles (city-level estimate — it was 198 from Pikeville). Cat 3 with all four hog classes and Certified Humane branding; Tier 2 with one gate — is it operating today, and is the real departure point Durham? Model B-T fits best at this distance.</t>
         </is>
       </c>
       <c r="W24" s="200" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="25" ht="45.2" customHeight="1" s="59">
+    <row r="25" ht="72" customHeight="1" s="59">
       <c r="A25" s="153" t="inlineStr">
         <is>
           <t>Farmington Meat Processing
@@ -22785,7 +22847,7 @@
       </c>
       <c r="E25" s="154" t="inlineStr">
         <is>
-          <t>Species A-E incl. swine (state code C); hog share unknown</t>
+          <t>Species A-E incl. swine (state code C); hog share unknown — boar/stag: ASK (state code does not distinguish)</t>
         </is>
       </c>
       <c r="F25" s="154" t="inlineStr">
@@ -22855,7 +22917,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" ht="45.2" customHeight="1" s="59">
+    <row r="26" ht="85.40000000000001" customHeight="1" s="59">
       <c r="A26" s="153" t="inlineStr">
         <is>
           <t>Easternview Farms
@@ -22880,7 +22942,7 @@
       </c>
       <c r="E26" s="154" t="inlineStr">
         <is>
-          <t>MARKET + SOW + boar/stag (FSIS)</t>
+          <t>⚠ BOAR/STAG flagged — MARKET + SOW + boar/stag (FSIS)</t>
         </is>
       </c>
       <c r="F26" s="154" t="inlineStr">
@@ -22918,7 +22980,7 @@
         <v>3</v>
       </c>
       <c r="N26" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O26" s="185" t="n">
         <v>1</v>
@@ -22945,14 +23007,18 @@
           <t>3</t>
         </is>
       </c>
-      <c r="V26" s="154" t="n"/>
+      <c r="V26" s="154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. </t>
+        </is>
+      </c>
       <c r="W26" s="200" t="inlineStr">
         <is>
           <t>follow-up</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="45.2" customHeight="1" s="59">
+    <row r="27" ht="85.40000000000001" customHeight="1" s="59">
       <c r="A27" s="153" t="inlineStr">
         <is>
           <t>The Butcher's Block
@@ -22977,7 +23043,7 @@
       </c>
       <c r="E27" s="154" t="inlineStr">
         <is>
-          <t>MARKET + SOW + ROASTER + boar/stag (all four FSIS classes)</t>
+          <t>⚠ BOAR/STAG flagged — MARKET + SOW + ROASTER + boar/stag (all four FSIS classes)</t>
         </is>
       </c>
       <c r="F27" s="154" t="inlineStr">
@@ -23015,7 +23081,7 @@
         <v>3</v>
       </c>
       <c r="N27" s="185" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O27" s="185" t="n">
         <v>1</v>
@@ -23042,7 +23108,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="V27" s="154" t="n"/>
+      <c r="V27" s="154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. </t>
+        </is>
+      </c>
       <c r="W27" s="200" t="inlineStr">
         <is>
           <t>—</t>
@@ -23133,13 +23203,13 @@
       <c r="B6" s="171" t="n"/>
       <c r="C6" s="172" t="n"/>
     </row>
-    <row r="7" ht="31.8" customHeight="1" s="59">
+    <row r="7" ht="45.2" customHeight="1" s="59">
       <c r="A7" s="193" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="154" t="inlineStr">
         <is>
-          <t>Are you a slaughterhouse — do you slaughter HOGS on site? (which classes — market weight, sows, roasters? anything in the 140-220 lb live range?)</t>
+          <t>Are you a slaughterhouse — do you slaughter HOGS on site? (which classes — market weight, sows, roasters? Any BOARS or STAGS — and are they ever run with the market hogs, or only on separate days?)</t>
         </is>
       </c>
       <c r="C7" s="191" t="n"/>

</xml_diff>

<commit_message>
Record the owner's decisions: scores stand, road miles only, EcoFriendly kept
- Scoring: Beebop's Part C caps declined; sub-scores unchanged.
- Distance: road miles only from the Durham origin. The radial
  reading is dropped; radial figures removed from the roster's distance
  column and the Rated Candidates distance cell; Instructions distance
  legend restated as an owner decision.
- EcoFriendly Foods stays on the list with its disputed-status note
  (moved to the "why" column on Rated Candidates; fit note on the
  roster).
- Instructions change log 2026-09-30 c; Sources & Confidence and the
  change register updated. Still open: boar gate hard vs soft, sow and
  aorta.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JvB48tbAk8juvoi9bxkFTf
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
+++ b/Tissue Supplier Research/Tissue_Supplier_Study.xlsx
@@ -1635,7 +1635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="59" min="1" max="1"/>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="98.8" customHeight="1" s="59">
+    <row r="29" ht="85.40000000000001" customHeight="1" s="59">
       <c r="A29" s="160" t="inlineStr">
         <is>
           <t>Distance column</t>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B29" s="154" t="inlineStr">
         <is>
-          <t>'YES/NO · ~nn mi' = real ROAD miles from the DURHAM origin (101 City Hall Plaza placeholder; OSRM driving routes, not straight-line) — the figure from the study's earlier Pikeville anchor is kept underneath in parentheses. '≈' = geocoded at city level (±5 mi); no mark = exact street address. YES = inside the 120-mile Model A radius; 'borderline' = 110-130. 'n/m' = not measured (multi-site, out of region, or not a plant). NOTE (Beebop v2.1): the ChatGPT brief reads '120 miles' as a RADIUS (straight-line) with road miles as logistics only — under that reading EcoFriendly (92.6 radial) is inside. This workbook keeps ROAD miles as the Model A screen because the crew drives it; radial figures are shown where Beebop supplied them. For Model B-T candidates distance is a sub-score, not a gate.</t>
+          <t>'YES/NO · ~nn mi' = real ROAD miles from the DURHAM origin (101 City Hall Plaza placeholder; OSRM driving routes, not straight-line) — the figure from the study's earlier Pikeville anchor is kept underneath in parentheses. '≈' = geocoded at city level (±5 mi); no mark = exact street address. YES = inside the 120-mile Model A radius; 'borderline' = 110-130. 'n/m' = not measured (multi-site, out of region, or not a plant). OWNER DECISION 2026-09-30: ROAD miles ONLY. The 'radius' (straight-line) reading of the brief is not used and radial figures are not carried; road miles from the Durham origin are the Model A screen because the crew drives them. For Model B-T candidates distance is a sub-score, not a gate.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,19 @@
       </c>
       <c r="B56" s="205" t="inlineStr">
         <is>
-          <t>Owner direction + Beebop instruction 23: three context tabs retired (export essentials folded into §6); change-register Part A facts applied (Gilbert Key d. 2026-04-06; Piedmont cut sheet disproves the 'viscera discarded' inference and J9 now cites M7975; TissueSource/LAMPIRE export statements recorded as company claims; Cool Springs 1976; McLaughlin's note repaired and its leadership-change signal downgraded to unverified; McLamb's ownership labelled as an interview claim; EcoFriendly status DISPUTED) and Part B repairs (TCO prose-as-formula cells, 'n/a' at zero production, cost-per-ACCEPTED-block block; full filters; western trio split; Anatomical Spec weight/sow/aorta fields, B28 and B31 wording; stunning ask removed). The roster was rebuilt into six priority sections with Priority IDs; duplicate rows marked. Part C scoring treatment and Part D decisions remain OPEN for the owner.</t>
+          <t>Owner direction + Beebop instruction 23: three context tabs retired (export essentials folded into §6); change-register Part A facts applied (Gilbert Key d. 2026-04-06; Piedmont cut sheet disproves the 'viscera discarded' inference and J9 now cites M7975; TissueSource/LAMPIRE export statements recorded as company claims; Cool Springs 1976; McLaughlin's note repaired and its leadership-change signal downgraded to unverified; McLamb's ownership labelled as an interview claim; EcoFriendly status DISPUTED) and Part B repairs (TCO prose-as-formula cells, 'n/a' at zero production, cost-per-ACCEPTED-block block; full filters; western trio split; Anatomical Spec weight/sow/aorta fields, B28 and B31 wording; stunning ask removed). The roster was rebuilt into six priority sections with Priority IDs; duplicate rows marked. Part C and Part D were put to the owner (see 2026-09-30 c).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="85.40000000000001" customHeight="1" s="59">
+      <c r="A57" s="204" t="inlineStr">
+        <is>
+          <t>2026-09-30 c</t>
+        </is>
+      </c>
+      <c r="B57" s="205" t="inlineStr">
+        <is>
+          <t>OWNER DECISIONS on the change register: (1) Scoring stays as built — Beebop's Part C caps (WELF 5 only with positive evidence, ACCESS ≤4 before a visit, RELN trims) are DECLINED; the sub-scores keep their 'bounded' wording where evidence is thin. (2) Distance: ROAD miles only from the Durham origin; the radial reading is dropped and radial figures removed from the distance column (§ distance legend updated). (3) EcoFriendly Foods stays on the list with its disputed-status note; the call settles it. Still open for the owner: boar/stag gate hard vs soft (currently soft, clearable on the call), sow acceptability and the aorta under the 140–220 lb target (Anatomical Spec B12/B14/D7).</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4345,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="98.8" customHeight="1" s="59">
+    <row r="53" ht="125.6" customHeight="1" s="59">
       <c r="A53" s="138" t="inlineStr">
         <is>
           <t>Retired tabs + restructure (2026-09-30)</t>
@@ -4351,7 +4363,7 @@
       </c>
       <c r="D53" s="68" t="inlineStr">
         <is>
-          <t>On the owner's direction the workbook was narrowed to the supplier list: 'Overview &amp; Method', 'Meeting Notes 2026-08' and 'APHIS &amp; EU Export' were retired (decisions and export essentials now live on Instructions §3/§6; the verbatim notes and the August narrative survive in git and in Deep_Study_Synthesis.pdf). The Supplier Roster's old region banners were replaced by six priority sections; every row got a Priority ID (column U); duplicate entries (Swaggerty, Leidy's, Fauquier's) were marked DUPLICATE in favour of the later row. Beebop's instruction 23 change register (Reviews/2026-09-30-rocksteady-change-register.md) Parts A and B were applied; Parts C and D await the owner.</t>
+          <t>On the owner's direction the workbook was narrowed to the supplier list: 'Overview &amp; Method', 'Meeting Notes 2026-08' and 'APHIS &amp; EU Export' were retired (decisions and export essentials now live on Instructions §3/§6; the verbatim notes and the August narrative survive in git and in Deep_Study_Synthesis.pdf). The Supplier Roster's old region banners were replaced by six priority sections; every row got a Priority ID (column U); duplicate entries (Swaggerty, Leidy's, Fauquier's) were marked DUPLICATE in favour of the later row. Beebop's instruction 23 change register (Reviews/2026-09-30-rocksteady-change-register.md) Parts A and B were applied; Owner decisions (same day): Part C declined — scores stand as built; road miles only (radial dropped); EcoFriendly kept with its note. Boar-gate hardness and the sow/aorta questions remain open.</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5984,7 @@
       <c r="E15" s="88" t="inlineStr">
         <is>
           <t>NO (boundary) · ~120 mi
-(120.4 exact road · 92.6 radial; Pikeville: ~198 mi)</t>
+(120.4 exact road; Pikeville: ~198 mi)</t>
         </is>
       </c>
       <c r="F15" s="143" t="inlineStr">
@@ -6037,7 +6049,7 @@
       </c>
       <c r="Q15" s="178" t="inlineStr">
         <is>
-          <t>BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER-2-ADJACENT (VA) — all four hog classes at cat-3 volume, the strongest VA option and welfare-branded; 120 road mi from Durham (198 from Pikeville) → Model B-T only. Site live 2026-09-03 (contradicts the old 'ceased ~2020' rumor again).</t>
+          <t>KEPT (owner decision 9-30) with the status note: confirm it is slaughtering before anything else. BOAR/STAG RULE 9-28: FSIS flags boar/stag slaughter at this plant — AVOID unless the call confirms boars/stags are never run with our hogs (gate G4). TIER-2-ADJACENT (VA) — all four hog classes at cat-3 volume, the strongest VA option and welfare-branded; 120 road mi from Durham (198 from Pikeville) → Model B-T only. Site live 2026-09-03 (contradicts the old 'ceased ~2020' rumor again).</t>
         </is>
       </c>
       <c r="R15" s="179" t="inlineStr">
@@ -6219,7 +6231,7 @@
       <c r="E17" s="88" t="inlineStr">
         <is>
           <t>YES · ~103 mi
-(91.7 radial; Pikeville: n/m)</t>
+(Pikeville: n/m)</t>
         </is>
       </c>
       <c r="F17" s="143" t="inlineStr">
@@ -6342,7 +6354,7 @@
       <c r="E18" s="88" t="inlineStr">
         <is>
           <t>YES · ~74 mi
-(60.5 radial; Pikeville: n/m)</t>
+(Pikeville: n/m)</t>
         </is>
       </c>
       <c r="F18" s="139" t="inlineStr">
@@ -6463,7 +6475,7 @@
       <c r="E19" s="88" t="inlineStr">
         <is>
           <t>YES · ~76 mi
-(65.2 radial; Pikeville: n/m)</t>
+(Pikeville: n/m)</t>
         </is>
       </c>
       <c r="F19" s="139" t="inlineStr">
@@ -7540,7 +7552,7 @@
       <c r="E28" s="88" t="inlineStr">
         <is>
           <t>YES · ~117 mi (borderline)
-(90.8 radial; Pikeville: n/m)</t>
+(Pikeville: n/m)</t>
         </is>
       </c>
       <c r="F28" s="139" t="inlineStr">
@@ -8286,7 +8298,7 @@
       <c r="E35" s="88" t="inlineStr">
         <is>
           <t>NO · ~141 mi
-(119.7 radial; Pikeville: ~88 mi)</t>
+(Pikeville: ~88 mi)</t>
         </is>
       </c>
       <c r="F35" s="139" t="inlineStr">
@@ -21614,7 +21626,7 @@
       </c>
       <c r="F24" s="154" t="inlineStr">
         <is>
-          <t>OPERATING STATUS DISPUTED (undated 'closed' directory flag vs live site) · cat 3 is ALL SPECIES incl. poultry — NASS caps all of VA at 7,841 hogs/yr; realistically tens/wk</t>
+          <t>cat 3 is ALL SPECIES incl. poultry — NASS caps all of VA at 7,841 hogs/yr; realistically tens/wk</t>
         </is>
       </c>
       <c r="G24" s="154" t="inlineStr">
@@ -21676,7 +21688,7 @@
       </c>
       <c r="V24" s="154" t="inlineStr">
         <is>
-          <t>9-30 SOCIAL: YellowPages lists it CLOSED and the phone conflicts across listings — operating status is the first call question. 9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. 9-28 v2.1: Tier 3 → 2, with a GATE. Beebop's point stands — this is a Model B-T harvesting-service call, not a volume play; its A/B scores (3.6 / 3.5) sit at Tier-2 level and parking it contradicted them. Gate on the call: is it operating today, and how many hogs in the 140-220 lb range per week (expect tens, not hundreds — Virginia's whole federal total is 7,841/yr). 9-28 VOLUME: Tier 2 → 3. NASS 2025 shows Virginia's 16 federal plants killed 7,841 hogs all year; the cat-3 band here is poultry-driven. Welfare-branded pilot candidate, not a volume lane. 9-28 r2: exact-address routing puts it at 120.4 road / 92.6 radial miles — a boundary case; PROX held at 4 pending the real departure point. 9-28 NEW ON THE SHORTLIST: the Durham origin brings it to ~112 road miles (city-level estimate — it was 198 from Pikeville). Cat 3 with all four hog classes and Certified Humane branding; Tier 2 with one gate — is it operating today, and is the real departure point Durham? Model B-T fits best at this distance.</t>
+          <t>OWNER DECISION 9-30: KEPT on the list with its status note — an undated YellowPages 'CLOSED' flag conflicts with a live company site and a 2025 price sheet; the first call settles it. 9-30 SOCIAL: YellowPages lists it CLOSED and the phone conflicts across listings — operating status is the first call question. 9-28 BOAR/STAG RULE: FSIS flags boar/stag slaughter here — the client will not mix boars with our hogs. ANAT capped at 2 (was 4); tier 3. GATE on the call: are boars / stags ever run with market hogs, or only on separate days? If never with ours, this can revert. 9-28 v2.1: Tier 3 → 2, with a GATE. Beebop's point stands — this is a Model B-T harvesting-service call, not a volume play; its A/B scores (3.6 / 3.5) sit at Tier-2 level and parking it contradicted them. Gate on the call: is it operating today, and how many hogs in the 140-220 lb range per week (expect tens, not hundreds — Virginia's whole federal total is 7,841/yr). 9-28 VOLUME: Tier 2 → 3. NASS 2025 shows Virginia's 16 federal plants killed 7,841 hogs all year; the cat-3 band here is poultry-driven. Welfare-branded pilot candidate, not a volume lane. 9-28 r2: exact-address routing puts it at 120.4 road miles — a boundary case; PROX held at 4 pending the real departure point. 9-28 NEW ON THE SHORTLIST: the Durham origin brings it to ~112 road miles (city-level estimate — it was 198 from Pikeville). Cat 3 with all four hog classes and Certified Humane branding; Tier 2 with one gate — is it operating today, and is the real departure point Durham? Model B-T fits best at this distance.</t>
         </is>
       </c>
       <c r="W24" s="200" t="n">

</xml_diff>